<commit_message>
Session-Ende 19.10.2026: Makler-Antworten Lieb/KSK, Excel aktualisiert
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/makler_antworten_archiv.xlsx
+++ b/data/makler_antworten_archiv.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legende" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Übersicht'!$A$1:$F$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Übersicht'!$A$1:$F$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Angebote'!$A$1:$S$100</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -537,7 +537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -711,17 +711,17 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Schneider &amp; Prell Immobilientreuhand</t>
+          <t>KSK München – BaufinanzierungsCenter</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Wolfratshausen · Fr. Pfeiffer</t>
+          <t>München · Hr. Basile (Baufinanzierung)</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>h.pfeiffer@schneider-prell.de</t>
+          <t>leonardo.basile@kskmse.de</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -736,61 +736,61 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>14.10. Kontaktformular ausgefüllt (Anschrift, Festnetz)</t>
+          <t>19.10. Antwort: nimmt uns in Datenbank auf; Anschrift + Mail gesendet (ohne Telefon)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>FT Immobilien 24</t>
+          <t>Lieb Immobilien</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Unterföhring · Hr. Tortorici</t>
+          <t>Weilheim · Hr. Lieb</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>kontakt@ftimmobilien24.com</t>
+          <t>info@lieb-immobilien.de</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Wartet auf Objekte</t>
+          <t>Wartet auf Antwort</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Exposé der Neubauwohnung abwarten und prüfen (Aufzug, Südterrasse, ~100 m²)</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>14.10. in Interessentenkartei aufgenommen</t>
+          <t>19.10. bietet passende Neubauwohnung an; Anschrift, Festnetz + Kriterien gesendet, Exposé erbeten</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Engel &amp; Völkers Starnberg</t>
+          <t>Schneider &amp; Prell Immobilientreuhand</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Starnberg</t>
+          <t>Wolfratshausen · Fr. Pfeiffer</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>contact@ (Ersatz-Adresse)</t>
+          <t>h.pfeiffer@schneider-prell.de</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Wartet auf Antwort</t>
+          <t>Wartet auf Objekte</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -800,83 +800,83 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>15.10. Voranfrage v4 an Ersatz-Adresse gesendet (alte Mail unzustellbar)</t>
+          <t>14.10. Kontaktformular ausgefüllt (Anschrift, Festnetz)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Engel &amp; Völkers München West</t>
+          <t>FT Immobilien 24</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Germering</t>
+          <t>Unterföhring · Hr. Tortorici</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>nur Kontaktformular</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Formular manuell</t>
+          <t>kontakt@ftimmobilien24.com</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Wartet auf Objekte</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Formular selbst absenden (Captcha) – Text: scratch/makler_formulare_20261014/formular_text.txt</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>14.10. Formular-Versuch: Captcha</t>
+          <t>14.10. in Interessentenkartei aufgenommen</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Engel &amp; Völkers Münchner Westen</t>
+          <t>Engel &amp; Völkers Starnberg</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Gräfelfing</t>
+          <t>Starnberg</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>nur Kontaktformular</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Formular manuell</t>
+          <t>contact@ (Ersatz-Adresse)</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Wartet auf Antwort</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Formular selbst absenden (Captcha)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>14.10. Formular-Versuch: Captcha</t>
+          <t>15.10. Voranfrage v4 an Ersatz-Adresse gesendet (alte Mail unzustellbar)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Engel &amp; Völkers Ostallgäu – Maria Platz</t>
+          <t>Engel &amp; Völkers München West</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Ostallgäu</t>
+          <t>Germering</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -891,7 +891,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Formular selbst absenden (Captcha)</t>
+          <t>Formular selbst absenden (Captcha) – Text: scratch/makler_formulare_20261014/formular_text.txt</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -903,12 +903,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>VON POLL IMMOBILIEN Füssen</t>
+          <t>Engel &amp; Völkers Münchner Westen</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Füssen</t>
+          <t>Gräfelfing</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -923,24 +923,24 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Formular selbst absenden (Bot-Schutz 403)</t>
+          <t>Formular selbst absenden (Captcha)</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>14.10. Formular-Versuch: blockt Automat</t>
+          <t>14.10. Formular-Versuch: Captcha</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>RE/MAX Immobilien Bad Tölz</t>
+          <t>Engel &amp; Völkers Ostallgäu – Maria Platz</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Bad Tölz</t>
+          <t>Ostallgäu</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -955,51 +955,115 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Formular selbst absenden (Security Verification)</t>
+          <t>Formular selbst absenden (Captcha)</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>14.10. Formular-Versuch: blockt Automat</t>
+          <t>14.10. Formular-Versuch: Captcha</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
+          <t>VON POLL IMMOBILIEN Füssen</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Füssen</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>nur Kontaktformular</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Formular manuell</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Formular selbst absenden (Bot-Schutz 403)</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>14.10. Formular-Versuch: blockt Automat</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>RE/MAX Immobilien Bad Tölz</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Bad Tölz</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>nur Kontaktformular</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Formular manuell</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Formular selbst absenden (Security Verification)</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>14.10. Formular-Versuch: blockt Automat</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
           <t>Aigner Immobilien</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>München Sendling · Fr. Becker</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>info@aigner-immobilien.de</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>Absage</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>14.10. Absage gesendet (Obermenzing = Etagenwohnung, No-Go)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F14"/>
+  <autoFilter ref="A1:F16"/>
   <dataValidations count="1">
-    <dataValidation sqref="D2:D34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Wartet auf Antwort,Wartet auf Objekte,Formular manuell,Absage,Neu prüfen"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Makler: Triage-Fix, Excel-Automatik mit Nebenkosten, Absagen Lieb/deltapro
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/makler_antworten_archiv.xlsx
+++ b/data/makler_antworten_archiv.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legende" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Übersicht'!$A$1:$F$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Angebote'!$A$1:$S$100</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Übersicht'!$A$1:$F$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Angebote'!$A$1:$V$100</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,10 +21,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="#,##0 &quot;€&quot;"/>
+    <numFmt numFmtId="165" formatCode="0.000&quot;%&quot;"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,6 +50,9 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -68,12 +73,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00EDEDED"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EDEDED"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -103,7 +108,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -135,6 +140,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -537,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -758,39 +767,39 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Wartet auf Antwort</t>
+          <t>Wartet auf Objekte</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Exposé der Neubauwohnung abwarten und prüfen (Aufzug, Südterrasse, ~100 m²)</t>
+          <t>Nur noch bei Penthouse/DG mit großer Südterrasse + Aufzug melden</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>19.10. bietet passende Neubauwohnung an; Anschrift, Festnetz + Kriterien gesendet, Exposé erbeten</t>
+          <t>19.10. Anschrift, Festnetz + Kriterien gesendet; 21.10. Exposé Peißenberg (nur überdachter Balkon) → Absage gesendet, Kontakt bleibt offen</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Schneider &amp; Prell Immobilientreuhand</t>
+          <t>deltapro Immobilien</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Wolfratshausen · Fr. Pfeiffer</t>
+          <t>Gilching · Fr. Götz</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>h.pfeiffer@schneider-prell.de</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>Wartet auf Objekte</t>
+          <t>info@deltapro.immobilien</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Absage</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -800,24 +809,24 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>14.10. Kontaktformular ausgefüllt (Anschrift, Festnetz)</t>
+          <t>21.10. Antwort mit Westpark-Sendling (kein PH/keine Terrasse) + Obermenzing DG 145 m² (Preis viel zu hoch) → Absage gesendet</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>FT Immobilien 24</t>
+          <t>Schneider &amp; Prell Immobilientreuhand</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Unterföhring · Hr. Tortorici</t>
+          <t>Wolfratshausen · Fr. Pfeiffer</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>kontakt@ftimmobilien24.com</t>
+          <t>h.pfeiffer@schneider-prell.de</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -832,29 +841,29 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>14.10. in Interessentenkartei aufgenommen</t>
+          <t>14.10. Kontaktformular ausgefüllt (Anschrift, Festnetz)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Engel &amp; Völkers Starnberg</t>
+          <t>FT Immobilien 24</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Starnberg</t>
+          <t>Unterföhring · Hr. Tortorici</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>contact@ (Ersatz-Adresse)</t>
+          <t>kontakt@ftimmobilien24.com</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Wartet auf Antwort</t>
+          <t>Wartet auf Objekte</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -864,51 +873,51 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>15.10. Voranfrage v4 an Ersatz-Adresse gesendet (alte Mail unzustellbar)</t>
+          <t>14.10. in Interessentenkartei aufgenommen</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Engel &amp; Völkers München West</t>
+          <t>Engel &amp; Völkers Starnberg</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Germering</t>
+          <t>Starnberg</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>nur Kontaktformular</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Formular manuell</t>
+          <t>contact@ (Ersatz-Adresse)</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Wartet auf Antwort</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Formular selbst absenden (Captcha) – Text: scratch/makler_formulare_20261014/formular_text.txt</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>14.10. Formular-Versuch: Captcha</t>
+          <t>15.10. Voranfrage v4 an Ersatz-Adresse gesendet (alte Mail unzustellbar)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Engel &amp; Völkers Münchner Westen</t>
+          <t>Engel &amp; Völkers München West</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Gräfelfing</t>
+          <t>Germering</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -916,14 +925,14 @@
           <t>nur Kontaktformular</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>Formular manuell</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Formular selbst absenden (Captcha)</t>
+          <t>Formular selbst absenden (Captcha) – Text: scratch/makler_formulare_20261014/formular_text.txt</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -935,12 +944,12 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Engel &amp; Völkers Ostallgäu – Maria Platz</t>
+          <t>Engel &amp; Völkers Münchner Westen</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Ostallgäu</t>
+          <t>Gräfelfing</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -948,7 +957,7 @@
           <t>nur Kontaktformular</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>Formular manuell</t>
         </is>
@@ -967,12 +976,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>VON POLL IMMOBILIEN Füssen</t>
+          <t>Engel &amp; Völkers Ostallgäu – Maria Platz</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Füssen</t>
+          <t>Ostallgäu</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -980,31 +989,31 @@
           <t>nur Kontaktformular</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>Formular manuell</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Formular selbst absenden (Bot-Schutz 403)</t>
+          <t>Formular selbst absenden (Captcha)</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>14.10. Formular-Versuch: blockt Automat</t>
+          <t>14.10. Formular-Versuch: Captcha</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>RE/MAX Immobilien Bad Tölz</t>
+          <t>VON POLL IMMOBILIEN Füssen</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Bad Tölz</t>
+          <t>Füssen</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -1012,14 +1021,14 @@
           <t>nur Kontaktformular</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>Formular manuell</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Formular selbst absenden (Security Verification)</t>
+          <t>Formular selbst absenden (Bot-Schutz 403)</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
@@ -1031,39 +1040,71 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
+          <t>RE/MAX Immobilien Bad Tölz</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Bad Tölz</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>nur Kontaktformular</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>Formular manuell</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Formular selbst absenden (Security Verification)</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>14.10. Formular-Versuch: blockt Automat</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
           <t>Aigner Immobilien</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>München Sendling · Fr. Becker</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>info@aigner-immobilien.de</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>Absage</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>14.10. Absage gesendet (Obermenzing = Etagenwohnung, No-Go)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F16"/>
+  <autoFilter ref="A1:F17"/>
   <dataValidations count="1">
-    <dataValidation sqref="D2:D36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Wartet auf Antwort,Wartet auf Objekte,Formular manuell,Absage,Neu prüfen"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1077,7 +1118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S100"/>
+  <dimension ref="A1:V100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1088,7 +1129,7 @@
     <col width="9" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="44" customWidth="1" min="8" max="8"/>
-    <col outlineLevel="1" width="12" customWidth="1" min="9" max="19"/>
+    <col outlineLevel="1" width="12" customWidth="1" min="9" max="22"/>
   </cols>
   <sheetData>
     <row r="1" ht="44" customHeight="1">
@@ -1187,6 +1228,21 @@
           <t>Größe ca. 100</t>
         </is>
       </c>
+      <c r="T1" s="7" t="inlineStr">
+        <is>
+          <t>Provision % (Käufer, inkl. MwSt.)</t>
+        </is>
+      </c>
+      <c r="U1" s="7" t="inlineStr">
+        <is>
+          <t>Nebenkosten €</t>
+        </is>
+      </c>
+      <c r="V1" s="7" t="inlineStr">
+        <is>
+          <t>Gesamtkosten €</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
@@ -1209,7 +1265,7 @@
         <v>91.42</v>
       </c>
       <c r="F2" s="10">
-        <f>IF(A2="","",IF(OR(C2="Etagenwohnung",I2="N"),0,ROUND(100*(3*IF(J2="J",1,IF(J2="N",0,0.5))+3*IF(K2="J",1,IF(K2="N",0,0.5))+2*IF(L2="J",1,IF(L2="N",0,0.5))+2*IF(M2="J",1,IF(M2="N",0,0.5))+1*IF(N2="J",1,IF(N2="N",0,0.5))+1*IF(O2="J",1,IF(O2="N",0,0.5))+1*IF(P2="J",1,IF(P2="N",0,0.5))+1*IF(Q2="J",1,IF(Q2="N",0,0.5))+2*IF(R2="J",1,IF(R2="N",0,0.5))+3*IF(S2="J",1,IF(S2="N",0,0.5)))/19,0)))</f>
+        <f>IF(A2="","",IF(OR(C2="Etagenwohnung",I2="N",J2="N"),0,ROUND(100*(3*IF(J2="J",1,IF(J2="N",0,0.5))+3*IF(K2="J",1,IF(K2="N",0,0.5))+2*IF(L2="J",1,IF(L2="N",0,0.5))+2*IF(M2="J",1,IF(M2="N",0,0.5))+1*IF(N2="J",1,IF(N2="N",0,0.5))+1*IF(O2="J",1,IF(O2="N",0,0.5))+1*IF(P2="J",1,IF(P2="N",0,0.5))+1*IF(Q2="J",1,IF(Q2="N",0,0.5))+2*IF(R2="J",1,IF(R2="N",0,0.5))+3*IF(S2="J",1,IF(S2="N",0,0.5))+IF(T2="",0,1*IF(T2="?",0.5,MAX(0,1-T2/3.57))))/(19+IF(T2="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G2" s="10" t="inlineStr">
@@ -1275,6 +1331,15 @@
         <f>IF(A2="","",IF(E2="","?",IF(AND(E2&gt;=90,E2&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T2" s="11" t="n"/>
+      <c r="U2" s="9">
+        <f>IF(OR(D2="",T2="",T2="?"),"",ROUND(D2*(Legende!$B$9+Legende!$B$10+T2/100),0))</f>
+        <v/>
+      </c>
+      <c r="V2" s="9">
+        <f>IF(U2="","",D2+U2)</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
@@ -1297,7 +1362,7 @@
       </c>
       <c r="E3" s="10" t="n"/>
       <c r="F3" s="10">
-        <f>IF(A3="","",IF(OR(C3="Etagenwohnung",I3="N"),0,ROUND(100*(3*IF(J3="J",1,IF(J3="N",0,0.5))+3*IF(K3="J",1,IF(K3="N",0,0.5))+2*IF(L3="J",1,IF(L3="N",0,0.5))+2*IF(M3="J",1,IF(M3="N",0,0.5))+1*IF(N3="J",1,IF(N3="N",0,0.5))+1*IF(O3="J",1,IF(O3="N",0,0.5))+1*IF(P3="J",1,IF(P3="N",0,0.5))+1*IF(Q3="J",1,IF(Q3="N",0,0.5))+2*IF(R3="J",1,IF(R3="N",0,0.5))+3*IF(S3="J",1,IF(S3="N",0,0.5)))/19,0)))</f>
+        <f>IF(A3="","",IF(OR(C3="Etagenwohnung",I3="N",J3="N"),0,ROUND(100*(3*IF(J3="J",1,IF(J3="N",0,0.5))+3*IF(K3="J",1,IF(K3="N",0,0.5))+2*IF(L3="J",1,IF(L3="N",0,0.5))+2*IF(M3="J",1,IF(M3="N",0,0.5))+1*IF(N3="J",1,IF(N3="N",0,0.5))+1*IF(O3="J",1,IF(O3="N",0,0.5))+1*IF(P3="J",1,IF(P3="N",0,0.5))+1*IF(Q3="J",1,IF(Q3="N",0,0.5))+2*IF(R3="J",1,IF(R3="N",0,0.5))+3*IF(S3="J",1,IF(S3="N",0,0.5))+IF(T3="",0,1*IF(T3="?",0.5,MAX(0,1-T3/3.57))))/(19+IF(T3="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G3" s="10" t="inlineStr">
@@ -1363,28 +1428,97 @@
         <f>IF(A3="","",IF(E3="","?",IF(AND(E3&gt;=90,E3&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T3" s="11" t="n"/>
+      <c r="U3" s="9">
+        <f>IF(OR(D3="",T3="",T3="?"),"",ROUND(D3*(Legende!$B$9+Legende!$B$10+T3/100),0))</f>
+        <v/>
+      </c>
+      <c r="V3" s="9">
+        <f>IF(U3="","",D3+U3)</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="n"/>
-      <c r="B4" s="8" t="n"/>
-      <c r="C4" s="8" t="n"/>
-      <c r="D4" s="9" t="n"/>
-      <c r="E4" s="10" t="n"/>
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Lieb Immobilien</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Neubau-DG, Wörther Str. 45, Peißenberg (5-Familienhaus, fertig Anfang 2027)</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Dachgeschoss</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="n">
+        <v>599000</v>
+      </c>
+      <c r="E4" s="10" t="n">
+        <v>122</v>
+      </c>
       <c r="F4" s="10">
-        <f>IF(A4="","",IF(OR(C4="Etagenwohnung",I4="N"),0,ROUND(100*(3*IF(J4="J",1,IF(J4="N",0,0.5))+3*IF(K4="J",1,IF(K4="N",0,0.5))+2*IF(L4="J",1,IF(L4="N",0,0.5))+2*IF(M4="J",1,IF(M4="N",0,0.5))+1*IF(N4="J",1,IF(N4="N",0,0.5))+1*IF(O4="J",1,IF(O4="N",0,0.5))+1*IF(P4="J",1,IF(P4="N",0,0.5))+1*IF(Q4="J",1,IF(Q4="N",0,0.5))+2*IF(R4="J",1,IF(R4="N",0,0.5))+3*IF(S4="J",1,IF(S4="N",0,0.5)))/19,0)))</f>
-        <v/>
-      </c>
-      <c r="G4" s="10" t="n"/>
-      <c r="H4" s="8" t="n"/>
-      <c r="I4" s="10" t="n"/>
-      <c r="J4" s="10" t="n"/>
-      <c r="K4" s="10" t="n"/>
-      <c r="L4" s="10" t="n"/>
-      <c r="M4" s="10" t="n"/>
-      <c r="N4" s="10" t="n"/>
-      <c r="O4" s="10" t="n"/>
-      <c r="P4" s="10" t="n"/>
-      <c r="Q4" s="10" t="n"/>
+        <f>IF(A4="","",IF(OR(C4="Etagenwohnung",I4="N",J4="N"),0,ROUND(100*(3*IF(J4="J",1,IF(J4="N",0,0.5))+3*IF(K4="J",1,IF(K4="N",0,0.5))+2*IF(L4="J",1,IF(L4="N",0,0.5))+2*IF(M4="J",1,IF(M4="N",0,0.5))+1*IF(N4="J",1,IF(N4="N",0,0.5))+1*IF(O4="J",1,IF(O4="N",0,0.5))+1*IF(P4="J",1,IF(P4="N",0,0.5))+1*IF(Q4="J",1,IF(Q4="N",0,0.5))+2*IF(R4="J",1,IF(R4="N",0,0.5))+3*IF(S4="J",1,IF(S4="N",0,0.5))+IF(T4="",0,1*IF(T4="?",0.5,MAX(0,1-T4/3.57))))/(19+IF(T4="",0,1)),0)))</f>
+        <v/>
+      </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>Absage</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>21.10. Absage: nur überdachter Balkon (große Terrasse = K.O.), Aufzug unklar; sonst FBH, WP, Keller, Garage</t>
+        </is>
+      </c>
+      <c r="I4" s="10" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="J4" s="10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="K4" s="10" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="L4" s="10" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="M4" s="10" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="N4" s="10" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="O4" s="10" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="P4" s="10" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="Q4" s="10" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
       <c r="R4" s="10">
         <f>IF(A4="","",IF(D4="","?",IF(D4&lt;=1250000,"J","N")))</f>
         <v/>
@@ -1393,34 +1527,110 @@
         <f>IF(A4="","",IF(E4="","?",IF(AND(E4&gt;=90,E4&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T4" s="11" t="n"/>
+      <c r="U4" s="9">
+        <f>IF(OR(D4="",T4="",T4="?"),"",ROUND(D4*(Legende!$B$9+Legende!$B$10+T4/100),0))</f>
+        <v/>
+      </c>
+      <c r="V4" s="9">
+        <f>IF(U4="","",D4+U4)</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="n"/>
-      <c r="B5" s="8" t="n"/>
-      <c r="C5" s="8" t="n"/>
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>deltapro Immobilien</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Obermenzing DG ca. 145 m², Bj. 2008/09 (+ Neubau Westpark Sendling)</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Dachgeschoss</t>
+        </is>
+      </c>
       <c r="D5" s="9" t="n"/>
-      <c r="E5" s="10" t="n"/>
+      <c r="E5" s="10" t="n">
+        <v>145</v>
+      </c>
       <c r="F5" s="10">
-        <f>IF(A5="","",IF(OR(C5="Etagenwohnung",I5="N"),0,ROUND(100*(3*IF(J5="J",1,IF(J5="N",0,0.5))+3*IF(K5="J",1,IF(K5="N",0,0.5))+2*IF(L5="J",1,IF(L5="N",0,0.5))+2*IF(M5="J",1,IF(M5="N",0,0.5))+1*IF(N5="J",1,IF(N5="N",0,0.5))+1*IF(O5="J",1,IF(O5="N",0,0.5))+1*IF(P5="J",1,IF(P5="N",0,0.5))+1*IF(Q5="J",1,IF(Q5="N",0,0.5))+2*IF(R5="J",1,IF(R5="N",0,0.5))+3*IF(S5="J",1,IF(S5="N",0,0.5)))/19,0)))</f>
-        <v/>
-      </c>
-      <c r="G5" s="10" t="n"/>
-      <c r="H5" s="8" t="n"/>
-      <c r="I5" s="10" t="n"/>
-      <c r="J5" s="10" t="n"/>
-      <c r="K5" s="10" t="n"/>
-      <c r="L5" s="10" t="n"/>
-      <c r="M5" s="10" t="n"/>
-      <c r="N5" s="10" t="n"/>
-      <c r="O5" s="10" t="n"/>
-      <c r="P5" s="10" t="n"/>
-      <c r="Q5" s="10" t="n"/>
+        <f>IF(A5="","",IF(OR(C5="Etagenwohnung",I5="N",J5="N"),0,ROUND(100*(3*IF(J5="J",1,IF(J5="N",0,0.5))+3*IF(K5="J",1,IF(K5="N",0,0.5))+2*IF(L5="J",1,IF(L5="N",0,0.5))+2*IF(M5="J",1,IF(M5="N",0,0.5))+1*IF(N5="J",1,IF(N5="N",0,0.5))+1*IF(O5="J",1,IF(O5="N",0,0.5))+1*IF(P5="J",1,IF(P5="N",0,0.5))+1*IF(Q5="J",1,IF(Q5="N",0,0.5))+2*IF(R5="J",1,IF(R5="N",0,0.5))+3*IF(S5="J",1,IF(S5="N",0,0.5))+IF(T5="",0,1*IF(T5="?",0.5,MAX(0,1-T5/3.57))))/(19+IF(T5="",0,1)),0)))</f>
+        <v/>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>Absage</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>21.10. Absage: Westpark ohne PH/Terrasse, Obermenzing Preis weit über Rahmen</t>
+        </is>
+      </c>
+      <c r="I5" s="10" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="J5" s="10" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="K5" s="10" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="L5" s="10" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="M5" s="10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N5" s="10" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="O5" s="10" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="P5" s="10" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="Q5" s="10" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
       <c r="R5" s="10">
         <f>IF(A5="","",IF(D5="","?",IF(D5&lt;=1250000,"J","N")))</f>
         <v/>
       </c>
       <c r="S5" s="10">
         <f>IF(A5="","",IF(E5="","?",IF(AND(E5&gt;=90,E5&lt;=115),"J","N")))</f>
+        <v/>
+      </c>
+      <c r="T5" s="11" t="n"/>
+      <c r="U5" s="9">
+        <f>IF(OR(D5="",T5="",T5="?"),"",ROUND(D5*(Legende!$B$9+Legende!$B$10+T5/100),0))</f>
+        <v/>
+      </c>
+      <c r="V5" s="9">
+        <f>IF(U5="","",D5+U5)</f>
         <v/>
       </c>
     </row>
@@ -1431,7 +1641,7 @@
       <c r="D6" s="9" t="n"/>
       <c r="E6" s="10" t="n"/>
       <c r="F6" s="10">
-        <f>IF(A6="","",IF(OR(C6="Etagenwohnung",I6="N"),0,ROUND(100*(3*IF(J6="J",1,IF(J6="N",0,0.5))+3*IF(K6="J",1,IF(K6="N",0,0.5))+2*IF(L6="J",1,IF(L6="N",0,0.5))+2*IF(M6="J",1,IF(M6="N",0,0.5))+1*IF(N6="J",1,IF(N6="N",0,0.5))+1*IF(O6="J",1,IF(O6="N",0,0.5))+1*IF(P6="J",1,IF(P6="N",0,0.5))+1*IF(Q6="J",1,IF(Q6="N",0,0.5))+2*IF(R6="J",1,IF(R6="N",0,0.5))+3*IF(S6="J",1,IF(S6="N",0,0.5)))/19,0)))</f>
+        <f>IF(A6="","",IF(OR(C6="Etagenwohnung",I6="N",J6="N"),0,ROUND(100*(3*IF(J6="J",1,IF(J6="N",0,0.5))+3*IF(K6="J",1,IF(K6="N",0,0.5))+2*IF(L6="J",1,IF(L6="N",0,0.5))+2*IF(M6="J",1,IF(M6="N",0,0.5))+1*IF(N6="J",1,IF(N6="N",0,0.5))+1*IF(O6="J",1,IF(O6="N",0,0.5))+1*IF(P6="J",1,IF(P6="N",0,0.5))+1*IF(Q6="J",1,IF(Q6="N",0,0.5))+2*IF(R6="J",1,IF(R6="N",0,0.5))+3*IF(S6="J",1,IF(S6="N",0,0.5))+IF(T6="",0,1*IF(T6="?",0.5,MAX(0,1-T6/3.57))))/(19+IF(T6="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G6" s="10" t="n"/>
@@ -1453,6 +1663,15 @@
         <f>IF(A6="","",IF(E6="","?",IF(AND(E6&gt;=90,E6&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T6" s="11" t="n"/>
+      <c r="U6" s="9">
+        <f>IF(OR(D6="",T6="",T6="?"),"",ROUND(D6*(Legende!$B$9+Legende!$B$10+T6/100),0))</f>
+        <v/>
+      </c>
+      <c r="V6" s="9">
+        <f>IF(U6="","",D6+U6)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="n"/>
@@ -1461,7 +1680,7 @@
       <c r="D7" s="9" t="n"/>
       <c r="E7" s="10" t="n"/>
       <c r="F7" s="10">
-        <f>IF(A7="","",IF(OR(C7="Etagenwohnung",I7="N"),0,ROUND(100*(3*IF(J7="J",1,IF(J7="N",0,0.5))+3*IF(K7="J",1,IF(K7="N",0,0.5))+2*IF(L7="J",1,IF(L7="N",0,0.5))+2*IF(M7="J",1,IF(M7="N",0,0.5))+1*IF(N7="J",1,IF(N7="N",0,0.5))+1*IF(O7="J",1,IF(O7="N",0,0.5))+1*IF(P7="J",1,IF(P7="N",0,0.5))+1*IF(Q7="J",1,IF(Q7="N",0,0.5))+2*IF(R7="J",1,IF(R7="N",0,0.5))+3*IF(S7="J",1,IF(S7="N",0,0.5)))/19,0)))</f>
+        <f>IF(A7="","",IF(OR(C7="Etagenwohnung",I7="N",J7="N"),0,ROUND(100*(3*IF(J7="J",1,IF(J7="N",0,0.5))+3*IF(K7="J",1,IF(K7="N",0,0.5))+2*IF(L7="J",1,IF(L7="N",0,0.5))+2*IF(M7="J",1,IF(M7="N",0,0.5))+1*IF(N7="J",1,IF(N7="N",0,0.5))+1*IF(O7="J",1,IF(O7="N",0,0.5))+1*IF(P7="J",1,IF(P7="N",0,0.5))+1*IF(Q7="J",1,IF(Q7="N",0,0.5))+2*IF(R7="J",1,IF(R7="N",0,0.5))+3*IF(S7="J",1,IF(S7="N",0,0.5))+IF(T7="",0,1*IF(T7="?",0.5,MAX(0,1-T7/3.57))))/(19+IF(T7="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G7" s="10" t="n"/>
@@ -1483,6 +1702,15 @@
         <f>IF(A7="","",IF(E7="","?",IF(AND(E7&gt;=90,E7&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T7" s="11" t="n"/>
+      <c r="U7" s="9">
+        <f>IF(OR(D7="",T7="",T7="?"),"",ROUND(D7*(Legende!$B$9+Legende!$B$10+T7/100),0))</f>
+        <v/>
+      </c>
+      <c r="V7" s="9">
+        <f>IF(U7="","",D7+U7)</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="n"/>
@@ -1491,7 +1719,7 @@
       <c r="D8" s="9" t="n"/>
       <c r="E8" s="10" t="n"/>
       <c r="F8" s="10">
-        <f>IF(A8="","",IF(OR(C8="Etagenwohnung",I8="N"),0,ROUND(100*(3*IF(J8="J",1,IF(J8="N",0,0.5))+3*IF(K8="J",1,IF(K8="N",0,0.5))+2*IF(L8="J",1,IF(L8="N",0,0.5))+2*IF(M8="J",1,IF(M8="N",0,0.5))+1*IF(N8="J",1,IF(N8="N",0,0.5))+1*IF(O8="J",1,IF(O8="N",0,0.5))+1*IF(P8="J",1,IF(P8="N",0,0.5))+1*IF(Q8="J",1,IF(Q8="N",0,0.5))+2*IF(R8="J",1,IF(R8="N",0,0.5))+3*IF(S8="J",1,IF(S8="N",0,0.5)))/19,0)))</f>
+        <f>IF(A8="","",IF(OR(C8="Etagenwohnung",I8="N",J8="N"),0,ROUND(100*(3*IF(J8="J",1,IF(J8="N",0,0.5))+3*IF(K8="J",1,IF(K8="N",0,0.5))+2*IF(L8="J",1,IF(L8="N",0,0.5))+2*IF(M8="J",1,IF(M8="N",0,0.5))+1*IF(N8="J",1,IF(N8="N",0,0.5))+1*IF(O8="J",1,IF(O8="N",0,0.5))+1*IF(P8="J",1,IF(P8="N",0,0.5))+1*IF(Q8="J",1,IF(Q8="N",0,0.5))+2*IF(R8="J",1,IF(R8="N",0,0.5))+3*IF(S8="J",1,IF(S8="N",0,0.5))+IF(T8="",0,1*IF(T8="?",0.5,MAX(0,1-T8/3.57))))/(19+IF(T8="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G8" s="10" t="n"/>
@@ -1513,6 +1741,15 @@
         <f>IF(A8="","",IF(E8="","?",IF(AND(E8&gt;=90,E8&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T8" s="11" t="n"/>
+      <c r="U8" s="9">
+        <f>IF(OR(D8="",T8="",T8="?"),"",ROUND(D8*(Legende!$B$9+Legende!$B$10+T8/100),0))</f>
+        <v/>
+      </c>
+      <c r="V8" s="9">
+        <f>IF(U8="","",D8+U8)</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="n"/>
@@ -1521,7 +1758,7 @@
       <c r="D9" s="9" t="n"/>
       <c r="E9" s="10" t="n"/>
       <c r="F9" s="10">
-        <f>IF(A9="","",IF(OR(C9="Etagenwohnung",I9="N"),0,ROUND(100*(3*IF(J9="J",1,IF(J9="N",0,0.5))+3*IF(K9="J",1,IF(K9="N",0,0.5))+2*IF(L9="J",1,IF(L9="N",0,0.5))+2*IF(M9="J",1,IF(M9="N",0,0.5))+1*IF(N9="J",1,IF(N9="N",0,0.5))+1*IF(O9="J",1,IF(O9="N",0,0.5))+1*IF(P9="J",1,IF(P9="N",0,0.5))+1*IF(Q9="J",1,IF(Q9="N",0,0.5))+2*IF(R9="J",1,IF(R9="N",0,0.5))+3*IF(S9="J",1,IF(S9="N",0,0.5)))/19,0)))</f>
+        <f>IF(A9="","",IF(OR(C9="Etagenwohnung",I9="N",J9="N"),0,ROUND(100*(3*IF(J9="J",1,IF(J9="N",0,0.5))+3*IF(K9="J",1,IF(K9="N",0,0.5))+2*IF(L9="J",1,IF(L9="N",0,0.5))+2*IF(M9="J",1,IF(M9="N",0,0.5))+1*IF(N9="J",1,IF(N9="N",0,0.5))+1*IF(O9="J",1,IF(O9="N",0,0.5))+1*IF(P9="J",1,IF(P9="N",0,0.5))+1*IF(Q9="J",1,IF(Q9="N",0,0.5))+2*IF(R9="J",1,IF(R9="N",0,0.5))+3*IF(S9="J",1,IF(S9="N",0,0.5))+IF(T9="",0,1*IF(T9="?",0.5,MAX(0,1-T9/3.57))))/(19+IF(T9="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G9" s="10" t="n"/>
@@ -1543,6 +1780,15 @@
         <f>IF(A9="","",IF(E9="","?",IF(AND(E9&gt;=90,E9&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T9" s="11" t="n"/>
+      <c r="U9" s="9">
+        <f>IF(OR(D9="",T9="",T9="?"),"",ROUND(D9*(Legende!$B$9+Legende!$B$10+T9/100),0))</f>
+        <v/>
+      </c>
+      <c r="V9" s="9">
+        <f>IF(U9="","",D9+U9)</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="n"/>
@@ -1551,7 +1797,7 @@
       <c r="D10" s="9" t="n"/>
       <c r="E10" s="10" t="n"/>
       <c r="F10" s="10">
-        <f>IF(A10="","",IF(OR(C10="Etagenwohnung",I10="N"),0,ROUND(100*(3*IF(J10="J",1,IF(J10="N",0,0.5))+3*IF(K10="J",1,IF(K10="N",0,0.5))+2*IF(L10="J",1,IF(L10="N",0,0.5))+2*IF(M10="J",1,IF(M10="N",0,0.5))+1*IF(N10="J",1,IF(N10="N",0,0.5))+1*IF(O10="J",1,IF(O10="N",0,0.5))+1*IF(P10="J",1,IF(P10="N",0,0.5))+1*IF(Q10="J",1,IF(Q10="N",0,0.5))+2*IF(R10="J",1,IF(R10="N",0,0.5))+3*IF(S10="J",1,IF(S10="N",0,0.5)))/19,0)))</f>
+        <f>IF(A10="","",IF(OR(C10="Etagenwohnung",I10="N",J10="N"),0,ROUND(100*(3*IF(J10="J",1,IF(J10="N",0,0.5))+3*IF(K10="J",1,IF(K10="N",0,0.5))+2*IF(L10="J",1,IF(L10="N",0,0.5))+2*IF(M10="J",1,IF(M10="N",0,0.5))+1*IF(N10="J",1,IF(N10="N",0,0.5))+1*IF(O10="J",1,IF(O10="N",0,0.5))+1*IF(P10="J",1,IF(P10="N",0,0.5))+1*IF(Q10="J",1,IF(Q10="N",0,0.5))+2*IF(R10="J",1,IF(R10="N",0,0.5))+3*IF(S10="J",1,IF(S10="N",0,0.5))+IF(T10="",0,1*IF(T10="?",0.5,MAX(0,1-T10/3.57))))/(19+IF(T10="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G10" s="10" t="n"/>
@@ -1573,6 +1819,15 @@
         <f>IF(A10="","",IF(E10="","?",IF(AND(E10&gt;=90,E10&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T10" s="11" t="n"/>
+      <c r="U10" s="9">
+        <f>IF(OR(D10="",T10="",T10="?"),"",ROUND(D10*(Legende!$B$9+Legende!$B$10+T10/100),0))</f>
+        <v/>
+      </c>
+      <c r="V10" s="9">
+        <f>IF(U10="","",D10+U10)</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="n"/>
@@ -1581,7 +1836,7 @@
       <c r="D11" s="9" t="n"/>
       <c r="E11" s="10" t="n"/>
       <c r="F11" s="10">
-        <f>IF(A11="","",IF(OR(C11="Etagenwohnung",I11="N"),0,ROUND(100*(3*IF(J11="J",1,IF(J11="N",0,0.5))+3*IF(K11="J",1,IF(K11="N",0,0.5))+2*IF(L11="J",1,IF(L11="N",0,0.5))+2*IF(M11="J",1,IF(M11="N",0,0.5))+1*IF(N11="J",1,IF(N11="N",0,0.5))+1*IF(O11="J",1,IF(O11="N",0,0.5))+1*IF(P11="J",1,IF(P11="N",0,0.5))+1*IF(Q11="J",1,IF(Q11="N",0,0.5))+2*IF(R11="J",1,IF(R11="N",0,0.5))+3*IF(S11="J",1,IF(S11="N",0,0.5)))/19,0)))</f>
+        <f>IF(A11="","",IF(OR(C11="Etagenwohnung",I11="N",J11="N"),0,ROUND(100*(3*IF(J11="J",1,IF(J11="N",0,0.5))+3*IF(K11="J",1,IF(K11="N",0,0.5))+2*IF(L11="J",1,IF(L11="N",0,0.5))+2*IF(M11="J",1,IF(M11="N",0,0.5))+1*IF(N11="J",1,IF(N11="N",0,0.5))+1*IF(O11="J",1,IF(O11="N",0,0.5))+1*IF(P11="J",1,IF(P11="N",0,0.5))+1*IF(Q11="J",1,IF(Q11="N",0,0.5))+2*IF(R11="J",1,IF(R11="N",0,0.5))+3*IF(S11="J",1,IF(S11="N",0,0.5))+IF(T11="",0,1*IF(T11="?",0.5,MAX(0,1-T11/3.57))))/(19+IF(T11="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G11" s="10" t="n"/>
@@ -1603,6 +1858,15 @@
         <f>IF(A11="","",IF(E11="","?",IF(AND(E11&gt;=90,E11&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T11" s="11" t="n"/>
+      <c r="U11" s="9">
+        <f>IF(OR(D11="",T11="",T11="?"),"",ROUND(D11*(Legende!$B$9+Legende!$B$10+T11/100),0))</f>
+        <v/>
+      </c>
+      <c r="V11" s="9">
+        <f>IF(U11="","",D11+U11)</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="n"/>
@@ -1611,7 +1875,7 @@
       <c r="D12" s="9" t="n"/>
       <c r="E12" s="10" t="n"/>
       <c r="F12" s="10">
-        <f>IF(A12="","",IF(OR(C12="Etagenwohnung",I12="N"),0,ROUND(100*(3*IF(J12="J",1,IF(J12="N",0,0.5))+3*IF(K12="J",1,IF(K12="N",0,0.5))+2*IF(L12="J",1,IF(L12="N",0,0.5))+2*IF(M12="J",1,IF(M12="N",0,0.5))+1*IF(N12="J",1,IF(N12="N",0,0.5))+1*IF(O12="J",1,IF(O12="N",0,0.5))+1*IF(P12="J",1,IF(P12="N",0,0.5))+1*IF(Q12="J",1,IF(Q12="N",0,0.5))+2*IF(R12="J",1,IF(R12="N",0,0.5))+3*IF(S12="J",1,IF(S12="N",0,0.5)))/19,0)))</f>
+        <f>IF(A12="","",IF(OR(C12="Etagenwohnung",I12="N",J12="N"),0,ROUND(100*(3*IF(J12="J",1,IF(J12="N",0,0.5))+3*IF(K12="J",1,IF(K12="N",0,0.5))+2*IF(L12="J",1,IF(L12="N",0,0.5))+2*IF(M12="J",1,IF(M12="N",0,0.5))+1*IF(N12="J",1,IF(N12="N",0,0.5))+1*IF(O12="J",1,IF(O12="N",0,0.5))+1*IF(P12="J",1,IF(P12="N",0,0.5))+1*IF(Q12="J",1,IF(Q12="N",0,0.5))+2*IF(R12="J",1,IF(R12="N",0,0.5))+3*IF(S12="J",1,IF(S12="N",0,0.5))+IF(T12="",0,1*IF(T12="?",0.5,MAX(0,1-T12/3.57))))/(19+IF(T12="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G12" s="10" t="n"/>
@@ -1633,6 +1897,15 @@
         <f>IF(A12="","",IF(E12="","?",IF(AND(E12&gt;=90,E12&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T12" s="11" t="n"/>
+      <c r="U12" s="9">
+        <f>IF(OR(D12="",T12="",T12="?"),"",ROUND(D12*(Legende!$B$9+Legende!$B$10+T12/100),0))</f>
+        <v/>
+      </c>
+      <c r="V12" s="9">
+        <f>IF(U12="","",D12+U12)</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="n"/>
@@ -1641,7 +1914,7 @@
       <c r="D13" s="9" t="n"/>
       <c r="E13" s="10" t="n"/>
       <c r="F13" s="10">
-        <f>IF(A13="","",IF(OR(C13="Etagenwohnung",I13="N"),0,ROUND(100*(3*IF(J13="J",1,IF(J13="N",0,0.5))+3*IF(K13="J",1,IF(K13="N",0,0.5))+2*IF(L13="J",1,IF(L13="N",0,0.5))+2*IF(M13="J",1,IF(M13="N",0,0.5))+1*IF(N13="J",1,IF(N13="N",0,0.5))+1*IF(O13="J",1,IF(O13="N",0,0.5))+1*IF(P13="J",1,IF(P13="N",0,0.5))+1*IF(Q13="J",1,IF(Q13="N",0,0.5))+2*IF(R13="J",1,IF(R13="N",0,0.5))+3*IF(S13="J",1,IF(S13="N",0,0.5)))/19,0)))</f>
+        <f>IF(A13="","",IF(OR(C13="Etagenwohnung",I13="N",J13="N"),0,ROUND(100*(3*IF(J13="J",1,IF(J13="N",0,0.5))+3*IF(K13="J",1,IF(K13="N",0,0.5))+2*IF(L13="J",1,IF(L13="N",0,0.5))+2*IF(M13="J",1,IF(M13="N",0,0.5))+1*IF(N13="J",1,IF(N13="N",0,0.5))+1*IF(O13="J",1,IF(O13="N",0,0.5))+1*IF(P13="J",1,IF(P13="N",0,0.5))+1*IF(Q13="J",1,IF(Q13="N",0,0.5))+2*IF(R13="J",1,IF(R13="N",0,0.5))+3*IF(S13="J",1,IF(S13="N",0,0.5))+IF(T13="",0,1*IF(T13="?",0.5,MAX(0,1-T13/3.57))))/(19+IF(T13="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G13" s="10" t="n"/>
@@ -1663,6 +1936,15 @@
         <f>IF(A13="","",IF(E13="","?",IF(AND(E13&gt;=90,E13&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T13" s="11" t="n"/>
+      <c r="U13" s="9">
+        <f>IF(OR(D13="",T13="",T13="?"),"",ROUND(D13*(Legende!$B$9+Legende!$B$10+T13/100),0))</f>
+        <v/>
+      </c>
+      <c r="V13" s="9">
+        <f>IF(U13="","",D13+U13)</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="n"/>
@@ -1671,7 +1953,7 @@
       <c r="D14" s="9" t="n"/>
       <c r="E14" s="10" t="n"/>
       <c r="F14" s="10">
-        <f>IF(A14="","",IF(OR(C14="Etagenwohnung",I14="N"),0,ROUND(100*(3*IF(J14="J",1,IF(J14="N",0,0.5))+3*IF(K14="J",1,IF(K14="N",0,0.5))+2*IF(L14="J",1,IF(L14="N",0,0.5))+2*IF(M14="J",1,IF(M14="N",0,0.5))+1*IF(N14="J",1,IF(N14="N",0,0.5))+1*IF(O14="J",1,IF(O14="N",0,0.5))+1*IF(P14="J",1,IF(P14="N",0,0.5))+1*IF(Q14="J",1,IF(Q14="N",0,0.5))+2*IF(R14="J",1,IF(R14="N",0,0.5))+3*IF(S14="J",1,IF(S14="N",0,0.5)))/19,0)))</f>
+        <f>IF(A14="","",IF(OR(C14="Etagenwohnung",I14="N",J14="N"),0,ROUND(100*(3*IF(J14="J",1,IF(J14="N",0,0.5))+3*IF(K14="J",1,IF(K14="N",0,0.5))+2*IF(L14="J",1,IF(L14="N",0,0.5))+2*IF(M14="J",1,IF(M14="N",0,0.5))+1*IF(N14="J",1,IF(N14="N",0,0.5))+1*IF(O14="J",1,IF(O14="N",0,0.5))+1*IF(P14="J",1,IF(P14="N",0,0.5))+1*IF(Q14="J",1,IF(Q14="N",0,0.5))+2*IF(R14="J",1,IF(R14="N",0,0.5))+3*IF(S14="J",1,IF(S14="N",0,0.5))+IF(T14="",0,1*IF(T14="?",0.5,MAX(0,1-T14/3.57))))/(19+IF(T14="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G14" s="10" t="n"/>
@@ -1693,6 +1975,15 @@
         <f>IF(A14="","",IF(E14="","?",IF(AND(E14&gt;=90,E14&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T14" s="11" t="n"/>
+      <c r="U14" s="9">
+        <f>IF(OR(D14="",T14="",T14="?"),"",ROUND(D14*(Legende!$B$9+Legende!$B$10+T14/100),0))</f>
+        <v/>
+      </c>
+      <c r="V14" s="9">
+        <f>IF(U14="","",D14+U14)</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="n"/>
@@ -1701,7 +1992,7 @@
       <c r="D15" s="9" t="n"/>
       <c r="E15" s="10" t="n"/>
       <c r="F15" s="10">
-        <f>IF(A15="","",IF(OR(C15="Etagenwohnung",I15="N"),0,ROUND(100*(3*IF(J15="J",1,IF(J15="N",0,0.5))+3*IF(K15="J",1,IF(K15="N",0,0.5))+2*IF(L15="J",1,IF(L15="N",0,0.5))+2*IF(M15="J",1,IF(M15="N",0,0.5))+1*IF(N15="J",1,IF(N15="N",0,0.5))+1*IF(O15="J",1,IF(O15="N",0,0.5))+1*IF(P15="J",1,IF(P15="N",0,0.5))+1*IF(Q15="J",1,IF(Q15="N",0,0.5))+2*IF(R15="J",1,IF(R15="N",0,0.5))+3*IF(S15="J",1,IF(S15="N",0,0.5)))/19,0)))</f>
+        <f>IF(A15="","",IF(OR(C15="Etagenwohnung",I15="N",J15="N"),0,ROUND(100*(3*IF(J15="J",1,IF(J15="N",0,0.5))+3*IF(K15="J",1,IF(K15="N",0,0.5))+2*IF(L15="J",1,IF(L15="N",0,0.5))+2*IF(M15="J",1,IF(M15="N",0,0.5))+1*IF(N15="J",1,IF(N15="N",0,0.5))+1*IF(O15="J",1,IF(O15="N",0,0.5))+1*IF(P15="J",1,IF(P15="N",0,0.5))+1*IF(Q15="J",1,IF(Q15="N",0,0.5))+2*IF(R15="J",1,IF(R15="N",0,0.5))+3*IF(S15="J",1,IF(S15="N",0,0.5))+IF(T15="",0,1*IF(T15="?",0.5,MAX(0,1-T15/3.57))))/(19+IF(T15="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G15" s="10" t="n"/>
@@ -1723,6 +2014,15 @@
         <f>IF(A15="","",IF(E15="","?",IF(AND(E15&gt;=90,E15&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T15" s="11" t="n"/>
+      <c r="U15" s="9">
+        <f>IF(OR(D15="",T15="",T15="?"),"",ROUND(D15*(Legende!$B$9+Legende!$B$10+T15/100),0))</f>
+        <v/>
+      </c>
+      <c r="V15" s="9">
+        <f>IF(U15="","",D15+U15)</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="n"/>
@@ -1731,7 +2031,7 @@
       <c r="D16" s="9" t="n"/>
       <c r="E16" s="10" t="n"/>
       <c r="F16" s="10">
-        <f>IF(A16="","",IF(OR(C16="Etagenwohnung",I16="N"),0,ROUND(100*(3*IF(J16="J",1,IF(J16="N",0,0.5))+3*IF(K16="J",1,IF(K16="N",0,0.5))+2*IF(L16="J",1,IF(L16="N",0,0.5))+2*IF(M16="J",1,IF(M16="N",0,0.5))+1*IF(N16="J",1,IF(N16="N",0,0.5))+1*IF(O16="J",1,IF(O16="N",0,0.5))+1*IF(P16="J",1,IF(P16="N",0,0.5))+1*IF(Q16="J",1,IF(Q16="N",0,0.5))+2*IF(R16="J",1,IF(R16="N",0,0.5))+3*IF(S16="J",1,IF(S16="N",0,0.5)))/19,0)))</f>
+        <f>IF(A16="","",IF(OR(C16="Etagenwohnung",I16="N",J16="N"),0,ROUND(100*(3*IF(J16="J",1,IF(J16="N",0,0.5))+3*IF(K16="J",1,IF(K16="N",0,0.5))+2*IF(L16="J",1,IF(L16="N",0,0.5))+2*IF(M16="J",1,IF(M16="N",0,0.5))+1*IF(N16="J",1,IF(N16="N",0,0.5))+1*IF(O16="J",1,IF(O16="N",0,0.5))+1*IF(P16="J",1,IF(P16="N",0,0.5))+1*IF(Q16="J",1,IF(Q16="N",0,0.5))+2*IF(R16="J",1,IF(R16="N",0,0.5))+3*IF(S16="J",1,IF(S16="N",0,0.5))+IF(T16="",0,1*IF(T16="?",0.5,MAX(0,1-T16/3.57))))/(19+IF(T16="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G16" s="10" t="n"/>
@@ -1753,6 +2053,15 @@
         <f>IF(A16="","",IF(E16="","?",IF(AND(E16&gt;=90,E16&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T16" s="11" t="n"/>
+      <c r="U16" s="9">
+        <f>IF(OR(D16="",T16="",T16="?"),"",ROUND(D16*(Legende!$B$9+Legende!$B$10+T16/100),0))</f>
+        <v/>
+      </c>
+      <c r="V16" s="9">
+        <f>IF(U16="","",D16+U16)</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="n"/>
@@ -1761,7 +2070,7 @@
       <c r="D17" s="9" t="n"/>
       <c r="E17" s="10" t="n"/>
       <c r="F17" s="10">
-        <f>IF(A17="","",IF(OR(C17="Etagenwohnung",I17="N"),0,ROUND(100*(3*IF(J17="J",1,IF(J17="N",0,0.5))+3*IF(K17="J",1,IF(K17="N",0,0.5))+2*IF(L17="J",1,IF(L17="N",0,0.5))+2*IF(M17="J",1,IF(M17="N",0,0.5))+1*IF(N17="J",1,IF(N17="N",0,0.5))+1*IF(O17="J",1,IF(O17="N",0,0.5))+1*IF(P17="J",1,IF(P17="N",0,0.5))+1*IF(Q17="J",1,IF(Q17="N",0,0.5))+2*IF(R17="J",1,IF(R17="N",0,0.5))+3*IF(S17="J",1,IF(S17="N",0,0.5)))/19,0)))</f>
+        <f>IF(A17="","",IF(OR(C17="Etagenwohnung",I17="N",J17="N"),0,ROUND(100*(3*IF(J17="J",1,IF(J17="N",0,0.5))+3*IF(K17="J",1,IF(K17="N",0,0.5))+2*IF(L17="J",1,IF(L17="N",0,0.5))+2*IF(M17="J",1,IF(M17="N",0,0.5))+1*IF(N17="J",1,IF(N17="N",0,0.5))+1*IF(O17="J",1,IF(O17="N",0,0.5))+1*IF(P17="J",1,IF(P17="N",0,0.5))+1*IF(Q17="J",1,IF(Q17="N",0,0.5))+2*IF(R17="J",1,IF(R17="N",0,0.5))+3*IF(S17="J",1,IF(S17="N",0,0.5))+IF(T17="",0,1*IF(T17="?",0.5,MAX(0,1-T17/3.57))))/(19+IF(T17="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G17" s="10" t="n"/>
@@ -1783,6 +2092,15 @@
         <f>IF(A17="","",IF(E17="","?",IF(AND(E17&gt;=90,E17&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T17" s="11" t="n"/>
+      <c r="U17" s="9">
+        <f>IF(OR(D17="",T17="",T17="?"),"",ROUND(D17*(Legende!$B$9+Legende!$B$10+T17/100),0))</f>
+        <v/>
+      </c>
+      <c r="V17" s="9">
+        <f>IF(U17="","",D17+U17)</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="n"/>
@@ -1791,7 +2109,7 @@
       <c r="D18" s="9" t="n"/>
       <c r="E18" s="10" t="n"/>
       <c r="F18" s="10">
-        <f>IF(A18="","",IF(OR(C18="Etagenwohnung",I18="N"),0,ROUND(100*(3*IF(J18="J",1,IF(J18="N",0,0.5))+3*IF(K18="J",1,IF(K18="N",0,0.5))+2*IF(L18="J",1,IF(L18="N",0,0.5))+2*IF(M18="J",1,IF(M18="N",0,0.5))+1*IF(N18="J",1,IF(N18="N",0,0.5))+1*IF(O18="J",1,IF(O18="N",0,0.5))+1*IF(P18="J",1,IF(P18="N",0,0.5))+1*IF(Q18="J",1,IF(Q18="N",0,0.5))+2*IF(R18="J",1,IF(R18="N",0,0.5))+3*IF(S18="J",1,IF(S18="N",0,0.5)))/19,0)))</f>
+        <f>IF(A18="","",IF(OR(C18="Etagenwohnung",I18="N",J18="N"),0,ROUND(100*(3*IF(J18="J",1,IF(J18="N",0,0.5))+3*IF(K18="J",1,IF(K18="N",0,0.5))+2*IF(L18="J",1,IF(L18="N",0,0.5))+2*IF(M18="J",1,IF(M18="N",0,0.5))+1*IF(N18="J",1,IF(N18="N",0,0.5))+1*IF(O18="J",1,IF(O18="N",0,0.5))+1*IF(P18="J",1,IF(P18="N",0,0.5))+1*IF(Q18="J",1,IF(Q18="N",0,0.5))+2*IF(R18="J",1,IF(R18="N",0,0.5))+3*IF(S18="J",1,IF(S18="N",0,0.5))+IF(T18="",0,1*IF(T18="?",0.5,MAX(0,1-T18/3.57))))/(19+IF(T18="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G18" s="10" t="n"/>
@@ -1813,6 +2131,15 @@
         <f>IF(A18="","",IF(E18="","?",IF(AND(E18&gt;=90,E18&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T18" s="11" t="n"/>
+      <c r="U18" s="9">
+        <f>IF(OR(D18="",T18="",T18="?"),"",ROUND(D18*(Legende!$B$9+Legende!$B$10+T18/100),0))</f>
+        <v/>
+      </c>
+      <c r="V18" s="9">
+        <f>IF(U18="","",D18+U18)</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="n"/>
@@ -1821,7 +2148,7 @@
       <c r="D19" s="9" t="n"/>
       <c r="E19" s="10" t="n"/>
       <c r="F19" s="10">
-        <f>IF(A19="","",IF(OR(C19="Etagenwohnung",I19="N"),0,ROUND(100*(3*IF(J19="J",1,IF(J19="N",0,0.5))+3*IF(K19="J",1,IF(K19="N",0,0.5))+2*IF(L19="J",1,IF(L19="N",0,0.5))+2*IF(M19="J",1,IF(M19="N",0,0.5))+1*IF(N19="J",1,IF(N19="N",0,0.5))+1*IF(O19="J",1,IF(O19="N",0,0.5))+1*IF(P19="J",1,IF(P19="N",0,0.5))+1*IF(Q19="J",1,IF(Q19="N",0,0.5))+2*IF(R19="J",1,IF(R19="N",0,0.5))+3*IF(S19="J",1,IF(S19="N",0,0.5)))/19,0)))</f>
+        <f>IF(A19="","",IF(OR(C19="Etagenwohnung",I19="N",J19="N"),0,ROUND(100*(3*IF(J19="J",1,IF(J19="N",0,0.5))+3*IF(K19="J",1,IF(K19="N",0,0.5))+2*IF(L19="J",1,IF(L19="N",0,0.5))+2*IF(M19="J",1,IF(M19="N",0,0.5))+1*IF(N19="J",1,IF(N19="N",0,0.5))+1*IF(O19="J",1,IF(O19="N",0,0.5))+1*IF(P19="J",1,IF(P19="N",0,0.5))+1*IF(Q19="J",1,IF(Q19="N",0,0.5))+2*IF(R19="J",1,IF(R19="N",0,0.5))+3*IF(S19="J",1,IF(S19="N",0,0.5))+IF(T19="",0,1*IF(T19="?",0.5,MAX(0,1-T19/3.57))))/(19+IF(T19="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G19" s="10" t="n"/>
@@ -1843,6 +2170,15 @@
         <f>IF(A19="","",IF(E19="","?",IF(AND(E19&gt;=90,E19&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T19" s="11" t="n"/>
+      <c r="U19" s="9">
+        <f>IF(OR(D19="",T19="",T19="?"),"",ROUND(D19*(Legende!$B$9+Legende!$B$10+T19/100),0))</f>
+        <v/>
+      </c>
+      <c r="V19" s="9">
+        <f>IF(U19="","",D19+U19)</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="n"/>
@@ -1851,7 +2187,7 @@
       <c r="D20" s="9" t="n"/>
       <c r="E20" s="10" t="n"/>
       <c r="F20" s="10">
-        <f>IF(A20="","",IF(OR(C20="Etagenwohnung",I20="N"),0,ROUND(100*(3*IF(J20="J",1,IF(J20="N",0,0.5))+3*IF(K20="J",1,IF(K20="N",0,0.5))+2*IF(L20="J",1,IF(L20="N",0,0.5))+2*IF(M20="J",1,IF(M20="N",0,0.5))+1*IF(N20="J",1,IF(N20="N",0,0.5))+1*IF(O20="J",1,IF(O20="N",0,0.5))+1*IF(P20="J",1,IF(P20="N",0,0.5))+1*IF(Q20="J",1,IF(Q20="N",0,0.5))+2*IF(R20="J",1,IF(R20="N",0,0.5))+3*IF(S20="J",1,IF(S20="N",0,0.5)))/19,0)))</f>
+        <f>IF(A20="","",IF(OR(C20="Etagenwohnung",I20="N",J20="N"),0,ROUND(100*(3*IF(J20="J",1,IF(J20="N",0,0.5))+3*IF(K20="J",1,IF(K20="N",0,0.5))+2*IF(L20="J",1,IF(L20="N",0,0.5))+2*IF(M20="J",1,IF(M20="N",0,0.5))+1*IF(N20="J",1,IF(N20="N",0,0.5))+1*IF(O20="J",1,IF(O20="N",0,0.5))+1*IF(P20="J",1,IF(P20="N",0,0.5))+1*IF(Q20="J",1,IF(Q20="N",0,0.5))+2*IF(R20="J",1,IF(R20="N",0,0.5))+3*IF(S20="J",1,IF(S20="N",0,0.5))+IF(T20="",0,1*IF(T20="?",0.5,MAX(0,1-T20/3.57))))/(19+IF(T20="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G20" s="10" t="n"/>
@@ -1873,6 +2209,15 @@
         <f>IF(A20="","",IF(E20="","?",IF(AND(E20&gt;=90,E20&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T20" s="11" t="n"/>
+      <c r="U20" s="9">
+        <f>IF(OR(D20="",T20="",T20="?"),"",ROUND(D20*(Legende!$B$9+Legende!$B$10+T20/100),0))</f>
+        <v/>
+      </c>
+      <c r="V20" s="9">
+        <f>IF(U20="","",D20+U20)</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="n"/>
@@ -1881,7 +2226,7 @@
       <c r="D21" s="9" t="n"/>
       <c r="E21" s="10" t="n"/>
       <c r="F21" s="10">
-        <f>IF(A21="","",IF(OR(C21="Etagenwohnung",I21="N"),0,ROUND(100*(3*IF(J21="J",1,IF(J21="N",0,0.5))+3*IF(K21="J",1,IF(K21="N",0,0.5))+2*IF(L21="J",1,IF(L21="N",0,0.5))+2*IF(M21="J",1,IF(M21="N",0,0.5))+1*IF(N21="J",1,IF(N21="N",0,0.5))+1*IF(O21="J",1,IF(O21="N",0,0.5))+1*IF(P21="J",1,IF(P21="N",0,0.5))+1*IF(Q21="J",1,IF(Q21="N",0,0.5))+2*IF(R21="J",1,IF(R21="N",0,0.5))+3*IF(S21="J",1,IF(S21="N",0,0.5)))/19,0)))</f>
+        <f>IF(A21="","",IF(OR(C21="Etagenwohnung",I21="N",J21="N"),0,ROUND(100*(3*IF(J21="J",1,IF(J21="N",0,0.5))+3*IF(K21="J",1,IF(K21="N",0,0.5))+2*IF(L21="J",1,IF(L21="N",0,0.5))+2*IF(M21="J",1,IF(M21="N",0,0.5))+1*IF(N21="J",1,IF(N21="N",0,0.5))+1*IF(O21="J",1,IF(O21="N",0,0.5))+1*IF(P21="J",1,IF(P21="N",0,0.5))+1*IF(Q21="J",1,IF(Q21="N",0,0.5))+2*IF(R21="J",1,IF(R21="N",0,0.5))+3*IF(S21="J",1,IF(S21="N",0,0.5))+IF(T21="",0,1*IF(T21="?",0.5,MAX(0,1-T21/3.57))))/(19+IF(T21="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G21" s="10" t="n"/>
@@ -1903,6 +2248,15 @@
         <f>IF(A21="","",IF(E21="","?",IF(AND(E21&gt;=90,E21&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T21" s="11" t="n"/>
+      <c r="U21" s="9">
+        <f>IF(OR(D21="",T21="",T21="?"),"",ROUND(D21*(Legende!$B$9+Legende!$B$10+T21/100),0))</f>
+        <v/>
+      </c>
+      <c r="V21" s="9">
+        <f>IF(U21="","",D21+U21)</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="n"/>
@@ -1911,7 +2265,7 @@
       <c r="D22" s="9" t="n"/>
       <c r="E22" s="10" t="n"/>
       <c r="F22" s="10">
-        <f>IF(A22="","",IF(OR(C22="Etagenwohnung",I22="N"),0,ROUND(100*(3*IF(J22="J",1,IF(J22="N",0,0.5))+3*IF(K22="J",1,IF(K22="N",0,0.5))+2*IF(L22="J",1,IF(L22="N",0,0.5))+2*IF(M22="J",1,IF(M22="N",0,0.5))+1*IF(N22="J",1,IF(N22="N",0,0.5))+1*IF(O22="J",1,IF(O22="N",0,0.5))+1*IF(P22="J",1,IF(P22="N",0,0.5))+1*IF(Q22="J",1,IF(Q22="N",0,0.5))+2*IF(R22="J",1,IF(R22="N",0,0.5))+3*IF(S22="J",1,IF(S22="N",0,0.5)))/19,0)))</f>
+        <f>IF(A22="","",IF(OR(C22="Etagenwohnung",I22="N",J22="N"),0,ROUND(100*(3*IF(J22="J",1,IF(J22="N",0,0.5))+3*IF(K22="J",1,IF(K22="N",0,0.5))+2*IF(L22="J",1,IF(L22="N",0,0.5))+2*IF(M22="J",1,IF(M22="N",0,0.5))+1*IF(N22="J",1,IF(N22="N",0,0.5))+1*IF(O22="J",1,IF(O22="N",0,0.5))+1*IF(P22="J",1,IF(P22="N",0,0.5))+1*IF(Q22="J",1,IF(Q22="N",0,0.5))+2*IF(R22="J",1,IF(R22="N",0,0.5))+3*IF(S22="J",1,IF(S22="N",0,0.5))+IF(T22="",0,1*IF(T22="?",0.5,MAX(0,1-T22/3.57))))/(19+IF(T22="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G22" s="10" t="n"/>
@@ -1933,6 +2287,15 @@
         <f>IF(A22="","",IF(E22="","?",IF(AND(E22&gt;=90,E22&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T22" s="11" t="n"/>
+      <c r="U22" s="9">
+        <f>IF(OR(D22="",T22="",T22="?"),"",ROUND(D22*(Legende!$B$9+Legende!$B$10+T22/100),0))</f>
+        <v/>
+      </c>
+      <c r="V22" s="9">
+        <f>IF(U22="","",D22+U22)</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="n"/>
@@ -1941,7 +2304,7 @@
       <c r="D23" s="9" t="n"/>
       <c r="E23" s="10" t="n"/>
       <c r="F23" s="10">
-        <f>IF(A23="","",IF(OR(C23="Etagenwohnung",I23="N"),0,ROUND(100*(3*IF(J23="J",1,IF(J23="N",0,0.5))+3*IF(K23="J",1,IF(K23="N",0,0.5))+2*IF(L23="J",1,IF(L23="N",0,0.5))+2*IF(M23="J",1,IF(M23="N",0,0.5))+1*IF(N23="J",1,IF(N23="N",0,0.5))+1*IF(O23="J",1,IF(O23="N",0,0.5))+1*IF(P23="J",1,IF(P23="N",0,0.5))+1*IF(Q23="J",1,IF(Q23="N",0,0.5))+2*IF(R23="J",1,IF(R23="N",0,0.5))+3*IF(S23="J",1,IF(S23="N",0,0.5)))/19,0)))</f>
+        <f>IF(A23="","",IF(OR(C23="Etagenwohnung",I23="N",J23="N"),0,ROUND(100*(3*IF(J23="J",1,IF(J23="N",0,0.5))+3*IF(K23="J",1,IF(K23="N",0,0.5))+2*IF(L23="J",1,IF(L23="N",0,0.5))+2*IF(M23="J",1,IF(M23="N",0,0.5))+1*IF(N23="J",1,IF(N23="N",0,0.5))+1*IF(O23="J",1,IF(O23="N",0,0.5))+1*IF(P23="J",1,IF(P23="N",0,0.5))+1*IF(Q23="J",1,IF(Q23="N",0,0.5))+2*IF(R23="J",1,IF(R23="N",0,0.5))+3*IF(S23="J",1,IF(S23="N",0,0.5))+IF(T23="",0,1*IF(T23="?",0.5,MAX(0,1-T23/3.57))))/(19+IF(T23="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G23" s="10" t="n"/>
@@ -1963,6 +2326,15 @@
         <f>IF(A23="","",IF(E23="","?",IF(AND(E23&gt;=90,E23&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T23" s="11" t="n"/>
+      <c r="U23" s="9">
+        <f>IF(OR(D23="",T23="",T23="?"),"",ROUND(D23*(Legende!$B$9+Legende!$B$10+T23/100),0))</f>
+        <v/>
+      </c>
+      <c r="V23" s="9">
+        <f>IF(U23="","",D23+U23)</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="n"/>
@@ -1971,7 +2343,7 @@
       <c r="D24" s="9" t="n"/>
       <c r="E24" s="10" t="n"/>
       <c r="F24" s="10">
-        <f>IF(A24="","",IF(OR(C24="Etagenwohnung",I24="N"),0,ROUND(100*(3*IF(J24="J",1,IF(J24="N",0,0.5))+3*IF(K24="J",1,IF(K24="N",0,0.5))+2*IF(L24="J",1,IF(L24="N",0,0.5))+2*IF(M24="J",1,IF(M24="N",0,0.5))+1*IF(N24="J",1,IF(N24="N",0,0.5))+1*IF(O24="J",1,IF(O24="N",0,0.5))+1*IF(P24="J",1,IF(P24="N",0,0.5))+1*IF(Q24="J",1,IF(Q24="N",0,0.5))+2*IF(R24="J",1,IF(R24="N",0,0.5))+3*IF(S24="J",1,IF(S24="N",0,0.5)))/19,0)))</f>
+        <f>IF(A24="","",IF(OR(C24="Etagenwohnung",I24="N",J24="N"),0,ROUND(100*(3*IF(J24="J",1,IF(J24="N",0,0.5))+3*IF(K24="J",1,IF(K24="N",0,0.5))+2*IF(L24="J",1,IF(L24="N",0,0.5))+2*IF(M24="J",1,IF(M24="N",0,0.5))+1*IF(N24="J",1,IF(N24="N",0,0.5))+1*IF(O24="J",1,IF(O24="N",0,0.5))+1*IF(P24="J",1,IF(P24="N",0,0.5))+1*IF(Q24="J",1,IF(Q24="N",0,0.5))+2*IF(R24="J",1,IF(R24="N",0,0.5))+3*IF(S24="J",1,IF(S24="N",0,0.5))+IF(T24="",0,1*IF(T24="?",0.5,MAX(0,1-T24/3.57))))/(19+IF(T24="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G24" s="10" t="n"/>
@@ -1993,6 +2365,15 @@
         <f>IF(A24="","",IF(E24="","?",IF(AND(E24&gt;=90,E24&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T24" s="11" t="n"/>
+      <c r="U24" s="9">
+        <f>IF(OR(D24="",T24="",T24="?"),"",ROUND(D24*(Legende!$B$9+Legende!$B$10+T24/100),0))</f>
+        <v/>
+      </c>
+      <c r="V24" s="9">
+        <f>IF(U24="","",D24+U24)</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="n"/>
@@ -2001,7 +2382,7 @@
       <c r="D25" s="9" t="n"/>
       <c r="E25" s="10" t="n"/>
       <c r="F25" s="10">
-        <f>IF(A25="","",IF(OR(C25="Etagenwohnung",I25="N"),0,ROUND(100*(3*IF(J25="J",1,IF(J25="N",0,0.5))+3*IF(K25="J",1,IF(K25="N",0,0.5))+2*IF(L25="J",1,IF(L25="N",0,0.5))+2*IF(M25="J",1,IF(M25="N",0,0.5))+1*IF(N25="J",1,IF(N25="N",0,0.5))+1*IF(O25="J",1,IF(O25="N",0,0.5))+1*IF(P25="J",1,IF(P25="N",0,0.5))+1*IF(Q25="J",1,IF(Q25="N",0,0.5))+2*IF(R25="J",1,IF(R25="N",0,0.5))+3*IF(S25="J",1,IF(S25="N",0,0.5)))/19,0)))</f>
+        <f>IF(A25="","",IF(OR(C25="Etagenwohnung",I25="N",J25="N"),0,ROUND(100*(3*IF(J25="J",1,IF(J25="N",0,0.5))+3*IF(K25="J",1,IF(K25="N",0,0.5))+2*IF(L25="J",1,IF(L25="N",0,0.5))+2*IF(M25="J",1,IF(M25="N",0,0.5))+1*IF(N25="J",1,IF(N25="N",0,0.5))+1*IF(O25="J",1,IF(O25="N",0,0.5))+1*IF(P25="J",1,IF(P25="N",0,0.5))+1*IF(Q25="J",1,IF(Q25="N",0,0.5))+2*IF(R25="J",1,IF(R25="N",0,0.5))+3*IF(S25="J",1,IF(S25="N",0,0.5))+IF(T25="",0,1*IF(T25="?",0.5,MAX(0,1-T25/3.57))))/(19+IF(T25="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G25" s="10" t="n"/>
@@ -2023,6 +2404,15 @@
         <f>IF(A25="","",IF(E25="","?",IF(AND(E25&gt;=90,E25&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T25" s="11" t="n"/>
+      <c r="U25" s="9">
+        <f>IF(OR(D25="",T25="",T25="?"),"",ROUND(D25*(Legende!$B$9+Legende!$B$10+T25/100),0))</f>
+        <v/>
+      </c>
+      <c r="V25" s="9">
+        <f>IF(U25="","",D25+U25)</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="n"/>
@@ -2031,7 +2421,7 @@
       <c r="D26" s="9" t="n"/>
       <c r="E26" s="10" t="n"/>
       <c r="F26" s="10">
-        <f>IF(A26="","",IF(OR(C26="Etagenwohnung",I26="N"),0,ROUND(100*(3*IF(J26="J",1,IF(J26="N",0,0.5))+3*IF(K26="J",1,IF(K26="N",0,0.5))+2*IF(L26="J",1,IF(L26="N",0,0.5))+2*IF(M26="J",1,IF(M26="N",0,0.5))+1*IF(N26="J",1,IF(N26="N",0,0.5))+1*IF(O26="J",1,IF(O26="N",0,0.5))+1*IF(P26="J",1,IF(P26="N",0,0.5))+1*IF(Q26="J",1,IF(Q26="N",0,0.5))+2*IF(R26="J",1,IF(R26="N",0,0.5))+3*IF(S26="J",1,IF(S26="N",0,0.5)))/19,0)))</f>
+        <f>IF(A26="","",IF(OR(C26="Etagenwohnung",I26="N",J26="N"),0,ROUND(100*(3*IF(J26="J",1,IF(J26="N",0,0.5))+3*IF(K26="J",1,IF(K26="N",0,0.5))+2*IF(L26="J",1,IF(L26="N",0,0.5))+2*IF(M26="J",1,IF(M26="N",0,0.5))+1*IF(N26="J",1,IF(N26="N",0,0.5))+1*IF(O26="J",1,IF(O26="N",0,0.5))+1*IF(P26="J",1,IF(P26="N",0,0.5))+1*IF(Q26="J",1,IF(Q26="N",0,0.5))+2*IF(R26="J",1,IF(R26="N",0,0.5))+3*IF(S26="J",1,IF(S26="N",0,0.5))+IF(T26="",0,1*IF(T26="?",0.5,MAX(0,1-T26/3.57))))/(19+IF(T26="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G26" s="10" t="n"/>
@@ -2053,6 +2443,15 @@
         <f>IF(A26="","",IF(E26="","?",IF(AND(E26&gt;=90,E26&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T26" s="11" t="n"/>
+      <c r="U26" s="9">
+        <f>IF(OR(D26="",T26="",T26="?"),"",ROUND(D26*(Legende!$B$9+Legende!$B$10+T26/100),0))</f>
+        <v/>
+      </c>
+      <c r="V26" s="9">
+        <f>IF(U26="","",D26+U26)</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="n"/>
@@ -2061,7 +2460,7 @@
       <c r="D27" s="9" t="n"/>
       <c r="E27" s="10" t="n"/>
       <c r="F27" s="10">
-        <f>IF(A27="","",IF(OR(C27="Etagenwohnung",I27="N"),0,ROUND(100*(3*IF(J27="J",1,IF(J27="N",0,0.5))+3*IF(K27="J",1,IF(K27="N",0,0.5))+2*IF(L27="J",1,IF(L27="N",0,0.5))+2*IF(M27="J",1,IF(M27="N",0,0.5))+1*IF(N27="J",1,IF(N27="N",0,0.5))+1*IF(O27="J",1,IF(O27="N",0,0.5))+1*IF(P27="J",1,IF(P27="N",0,0.5))+1*IF(Q27="J",1,IF(Q27="N",0,0.5))+2*IF(R27="J",1,IF(R27="N",0,0.5))+3*IF(S27="J",1,IF(S27="N",0,0.5)))/19,0)))</f>
+        <f>IF(A27="","",IF(OR(C27="Etagenwohnung",I27="N",J27="N"),0,ROUND(100*(3*IF(J27="J",1,IF(J27="N",0,0.5))+3*IF(K27="J",1,IF(K27="N",0,0.5))+2*IF(L27="J",1,IF(L27="N",0,0.5))+2*IF(M27="J",1,IF(M27="N",0,0.5))+1*IF(N27="J",1,IF(N27="N",0,0.5))+1*IF(O27="J",1,IF(O27="N",0,0.5))+1*IF(P27="J",1,IF(P27="N",0,0.5))+1*IF(Q27="J",1,IF(Q27="N",0,0.5))+2*IF(R27="J",1,IF(R27="N",0,0.5))+3*IF(S27="J",1,IF(S27="N",0,0.5))+IF(T27="",0,1*IF(T27="?",0.5,MAX(0,1-T27/3.57))))/(19+IF(T27="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G27" s="10" t="n"/>
@@ -2083,6 +2482,15 @@
         <f>IF(A27="","",IF(E27="","?",IF(AND(E27&gt;=90,E27&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T27" s="11" t="n"/>
+      <c r="U27" s="9">
+        <f>IF(OR(D27="",T27="",T27="?"),"",ROUND(D27*(Legende!$B$9+Legende!$B$10+T27/100),0))</f>
+        <v/>
+      </c>
+      <c r="V27" s="9">
+        <f>IF(U27="","",D27+U27)</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="8" t="n"/>
@@ -2091,7 +2499,7 @@
       <c r="D28" s="9" t="n"/>
       <c r="E28" s="10" t="n"/>
       <c r="F28" s="10">
-        <f>IF(A28="","",IF(OR(C28="Etagenwohnung",I28="N"),0,ROUND(100*(3*IF(J28="J",1,IF(J28="N",0,0.5))+3*IF(K28="J",1,IF(K28="N",0,0.5))+2*IF(L28="J",1,IF(L28="N",0,0.5))+2*IF(M28="J",1,IF(M28="N",0,0.5))+1*IF(N28="J",1,IF(N28="N",0,0.5))+1*IF(O28="J",1,IF(O28="N",0,0.5))+1*IF(P28="J",1,IF(P28="N",0,0.5))+1*IF(Q28="J",1,IF(Q28="N",0,0.5))+2*IF(R28="J",1,IF(R28="N",0,0.5))+3*IF(S28="J",1,IF(S28="N",0,0.5)))/19,0)))</f>
+        <f>IF(A28="","",IF(OR(C28="Etagenwohnung",I28="N",J28="N"),0,ROUND(100*(3*IF(J28="J",1,IF(J28="N",0,0.5))+3*IF(K28="J",1,IF(K28="N",0,0.5))+2*IF(L28="J",1,IF(L28="N",0,0.5))+2*IF(M28="J",1,IF(M28="N",0,0.5))+1*IF(N28="J",1,IF(N28="N",0,0.5))+1*IF(O28="J",1,IF(O28="N",0,0.5))+1*IF(P28="J",1,IF(P28="N",0,0.5))+1*IF(Q28="J",1,IF(Q28="N",0,0.5))+2*IF(R28="J",1,IF(R28="N",0,0.5))+3*IF(S28="J",1,IF(S28="N",0,0.5))+IF(T28="",0,1*IF(T28="?",0.5,MAX(0,1-T28/3.57))))/(19+IF(T28="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G28" s="10" t="n"/>
@@ -2113,6 +2521,15 @@
         <f>IF(A28="","",IF(E28="","?",IF(AND(E28&gt;=90,E28&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T28" s="11" t="n"/>
+      <c r="U28" s="9">
+        <f>IF(OR(D28="",T28="",T28="?"),"",ROUND(D28*(Legende!$B$9+Legende!$B$10+T28/100),0))</f>
+        <v/>
+      </c>
+      <c r="V28" s="9">
+        <f>IF(U28="","",D28+U28)</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="n"/>
@@ -2121,7 +2538,7 @@
       <c r="D29" s="9" t="n"/>
       <c r="E29" s="10" t="n"/>
       <c r="F29" s="10">
-        <f>IF(A29="","",IF(OR(C29="Etagenwohnung",I29="N"),0,ROUND(100*(3*IF(J29="J",1,IF(J29="N",0,0.5))+3*IF(K29="J",1,IF(K29="N",0,0.5))+2*IF(L29="J",1,IF(L29="N",0,0.5))+2*IF(M29="J",1,IF(M29="N",0,0.5))+1*IF(N29="J",1,IF(N29="N",0,0.5))+1*IF(O29="J",1,IF(O29="N",0,0.5))+1*IF(P29="J",1,IF(P29="N",0,0.5))+1*IF(Q29="J",1,IF(Q29="N",0,0.5))+2*IF(R29="J",1,IF(R29="N",0,0.5))+3*IF(S29="J",1,IF(S29="N",0,0.5)))/19,0)))</f>
+        <f>IF(A29="","",IF(OR(C29="Etagenwohnung",I29="N",J29="N"),0,ROUND(100*(3*IF(J29="J",1,IF(J29="N",0,0.5))+3*IF(K29="J",1,IF(K29="N",0,0.5))+2*IF(L29="J",1,IF(L29="N",0,0.5))+2*IF(M29="J",1,IF(M29="N",0,0.5))+1*IF(N29="J",1,IF(N29="N",0,0.5))+1*IF(O29="J",1,IF(O29="N",0,0.5))+1*IF(P29="J",1,IF(P29="N",0,0.5))+1*IF(Q29="J",1,IF(Q29="N",0,0.5))+2*IF(R29="J",1,IF(R29="N",0,0.5))+3*IF(S29="J",1,IF(S29="N",0,0.5))+IF(T29="",0,1*IF(T29="?",0.5,MAX(0,1-T29/3.57))))/(19+IF(T29="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G29" s="10" t="n"/>
@@ -2143,6 +2560,15 @@
         <f>IF(A29="","",IF(E29="","?",IF(AND(E29&gt;=90,E29&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T29" s="11" t="n"/>
+      <c r="U29" s="9">
+        <f>IF(OR(D29="",T29="",T29="?"),"",ROUND(D29*(Legende!$B$9+Legende!$B$10+T29/100),0))</f>
+        <v/>
+      </c>
+      <c r="V29" s="9">
+        <f>IF(U29="","",D29+U29)</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="8" t="n"/>
@@ -2151,7 +2577,7 @@
       <c r="D30" s="9" t="n"/>
       <c r="E30" s="10" t="n"/>
       <c r="F30" s="10">
-        <f>IF(A30="","",IF(OR(C30="Etagenwohnung",I30="N"),0,ROUND(100*(3*IF(J30="J",1,IF(J30="N",0,0.5))+3*IF(K30="J",1,IF(K30="N",0,0.5))+2*IF(L30="J",1,IF(L30="N",0,0.5))+2*IF(M30="J",1,IF(M30="N",0,0.5))+1*IF(N30="J",1,IF(N30="N",0,0.5))+1*IF(O30="J",1,IF(O30="N",0,0.5))+1*IF(P30="J",1,IF(P30="N",0,0.5))+1*IF(Q30="J",1,IF(Q30="N",0,0.5))+2*IF(R30="J",1,IF(R30="N",0,0.5))+3*IF(S30="J",1,IF(S30="N",0,0.5)))/19,0)))</f>
+        <f>IF(A30="","",IF(OR(C30="Etagenwohnung",I30="N",J30="N"),0,ROUND(100*(3*IF(J30="J",1,IF(J30="N",0,0.5))+3*IF(K30="J",1,IF(K30="N",0,0.5))+2*IF(L30="J",1,IF(L30="N",0,0.5))+2*IF(M30="J",1,IF(M30="N",0,0.5))+1*IF(N30="J",1,IF(N30="N",0,0.5))+1*IF(O30="J",1,IF(O30="N",0,0.5))+1*IF(P30="J",1,IF(P30="N",0,0.5))+1*IF(Q30="J",1,IF(Q30="N",0,0.5))+2*IF(R30="J",1,IF(R30="N",0,0.5))+3*IF(S30="J",1,IF(S30="N",0,0.5))+IF(T30="",0,1*IF(T30="?",0.5,MAX(0,1-T30/3.57))))/(19+IF(T30="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G30" s="10" t="n"/>
@@ -2173,6 +2599,15 @@
         <f>IF(A30="","",IF(E30="","?",IF(AND(E30&gt;=90,E30&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T30" s="11" t="n"/>
+      <c r="U30" s="9">
+        <f>IF(OR(D30="",T30="",T30="?"),"",ROUND(D30*(Legende!$B$9+Legende!$B$10+T30/100),0))</f>
+        <v/>
+      </c>
+      <c r="V30" s="9">
+        <f>IF(U30="","",D30+U30)</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="n"/>
@@ -2181,7 +2616,7 @@
       <c r="D31" s="9" t="n"/>
       <c r="E31" s="10" t="n"/>
       <c r="F31" s="10">
-        <f>IF(A31="","",IF(OR(C31="Etagenwohnung",I31="N"),0,ROUND(100*(3*IF(J31="J",1,IF(J31="N",0,0.5))+3*IF(K31="J",1,IF(K31="N",0,0.5))+2*IF(L31="J",1,IF(L31="N",0,0.5))+2*IF(M31="J",1,IF(M31="N",0,0.5))+1*IF(N31="J",1,IF(N31="N",0,0.5))+1*IF(O31="J",1,IF(O31="N",0,0.5))+1*IF(P31="J",1,IF(P31="N",0,0.5))+1*IF(Q31="J",1,IF(Q31="N",0,0.5))+2*IF(R31="J",1,IF(R31="N",0,0.5))+3*IF(S31="J",1,IF(S31="N",0,0.5)))/19,0)))</f>
+        <f>IF(A31="","",IF(OR(C31="Etagenwohnung",I31="N",J31="N"),0,ROUND(100*(3*IF(J31="J",1,IF(J31="N",0,0.5))+3*IF(K31="J",1,IF(K31="N",0,0.5))+2*IF(L31="J",1,IF(L31="N",0,0.5))+2*IF(M31="J",1,IF(M31="N",0,0.5))+1*IF(N31="J",1,IF(N31="N",0,0.5))+1*IF(O31="J",1,IF(O31="N",0,0.5))+1*IF(P31="J",1,IF(P31="N",0,0.5))+1*IF(Q31="J",1,IF(Q31="N",0,0.5))+2*IF(R31="J",1,IF(R31="N",0,0.5))+3*IF(S31="J",1,IF(S31="N",0,0.5))+IF(T31="",0,1*IF(T31="?",0.5,MAX(0,1-T31/3.57))))/(19+IF(T31="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G31" s="10" t="n"/>
@@ -2203,6 +2638,15 @@
         <f>IF(A31="","",IF(E31="","?",IF(AND(E31&gt;=90,E31&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T31" s="11" t="n"/>
+      <c r="U31" s="9">
+        <f>IF(OR(D31="",T31="",T31="?"),"",ROUND(D31*(Legende!$B$9+Legende!$B$10+T31/100),0))</f>
+        <v/>
+      </c>
+      <c r="V31" s="9">
+        <f>IF(U31="","",D31+U31)</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="8" t="n"/>
@@ -2211,7 +2655,7 @@
       <c r="D32" s="9" t="n"/>
       <c r="E32" s="10" t="n"/>
       <c r="F32" s="10">
-        <f>IF(A32="","",IF(OR(C32="Etagenwohnung",I32="N"),0,ROUND(100*(3*IF(J32="J",1,IF(J32="N",0,0.5))+3*IF(K32="J",1,IF(K32="N",0,0.5))+2*IF(L32="J",1,IF(L32="N",0,0.5))+2*IF(M32="J",1,IF(M32="N",0,0.5))+1*IF(N32="J",1,IF(N32="N",0,0.5))+1*IF(O32="J",1,IF(O32="N",0,0.5))+1*IF(P32="J",1,IF(P32="N",0,0.5))+1*IF(Q32="J",1,IF(Q32="N",0,0.5))+2*IF(R32="J",1,IF(R32="N",0,0.5))+3*IF(S32="J",1,IF(S32="N",0,0.5)))/19,0)))</f>
+        <f>IF(A32="","",IF(OR(C32="Etagenwohnung",I32="N",J32="N"),0,ROUND(100*(3*IF(J32="J",1,IF(J32="N",0,0.5))+3*IF(K32="J",1,IF(K32="N",0,0.5))+2*IF(L32="J",1,IF(L32="N",0,0.5))+2*IF(M32="J",1,IF(M32="N",0,0.5))+1*IF(N32="J",1,IF(N32="N",0,0.5))+1*IF(O32="J",1,IF(O32="N",0,0.5))+1*IF(P32="J",1,IF(P32="N",0,0.5))+1*IF(Q32="J",1,IF(Q32="N",0,0.5))+2*IF(R32="J",1,IF(R32="N",0,0.5))+3*IF(S32="J",1,IF(S32="N",0,0.5))+IF(T32="",0,1*IF(T32="?",0.5,MAX(0,1-T32/3.57))))/(19+IF(T32="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G32" s="10" t="n"/>
@@ -2233,6 +2677,15 @@
         <f>IF(A32="","",IF(E32="","?",IF(AND(E32&gt;=90,E32&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T32" s="11" t="n"/>
+      <c r="U32" s="9">
+        <f>IF(OR(D32="",T32="",T32="?"),"",ROUND(D32*(Legende!$B$9+Legende!$B$10+T32/100),0))</f>
+        <v/>
+      </c>
+      <c r="V32" s="9">
+        <f>IF(U32="","",D32+U32)</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="n"/>
@@ -2241,7 +2694,7 @@
       <c r="D33" s="9" t="n"/>
       <c r="E33" s="10" t="n"/>
       <c r="F33" s="10">
-        <f>IF(A33="","",IF(OR(C33="Etagenwohnung",I33="N"),0,ROUND(100*(3*IF(J33="J",1,IF(J33="N",0,0.5))+3*IF(K33="J",1,IF(K33="N",0,0.5))+2*IF(L33="J",1,IF(L33="N",0,0.5))+2*IF(M33="J",1,IF(M33="N",0,0.5))+1*IF(N33="J",1,IF(N33="N",0,0.5))+1*IF(O33="J",1,IF(O33="N",0,0.5))+1*IF(P33="J",1,IF(P33="N",0,0.5))+1*IF(Q33="J",1,IF(Q33="N",0,0.5))+2*IF(R33="J",1,IF(R33="N",0,0.5))+3*IF(S33="J",1,IF(S33="N",0,0.5)))/19,0)))</f>
+        <f>IF(A33="","",IF(OR(C33="Etagenwohnung",I33="N",J33="N"),0,ROUND(100*(3*IF(J33="J",1,IF(J33="N",0,0.5))+3*IF(K33="J",1,IF(K33="N",0,0.5))+2*IF(L33="J",1,IF(L33="N",0,0.5))+2*IF(M33="J",1,IF(M33="N",0,0.5))+1*IF(N33="J",1,IF(N33="N",0,0.5))+1*IF(O33="J",1,IF(O33="N",0,0.5))+1*IF(P33="J",1,IF(P33="N",0,0.5))+1*IF(Q33="J",1,IF(Q33="N",0,0.5))+2*IF(R33="J",1,IF(R33="N",0,0.5))+3*IF(S33="J",1,IF(S33="N",0,0.5))+IF(T33="",0,1*IF(T33="?",0.5,MAX(0,1-T33/3.57))))/(19+IF(T33="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G33" s="10" t="n"/>
@@ -2263,6 +2716,15 @@
         <f>IF(A33="","",IF(E33="","?",IF(AND(E33&gt;=90,E33&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T33" s="11" t="n"/>
+      <c r="U33" s="9">
+        <f>IF(OR(D33="",T33="",T33="?"),"",ROUND(D33*(Legende!$B$9+Legende!$B$10+T33/100),0))</f>
+        <v/>
+      </c>
+      <c r="V33" s="9">
+        <f>IF(U33="","",D33+U33)</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="8" t="n"/>
@@ -2271,7 +2733,7 @@
       <c r="D34" s="9" t="n"/>
       <c r="E34" s="10" t="n"/>
       <c r="F34" s="10">
-        <f>IF(A34="","",IF(OR(C34="Etagenwohnung",I34="N"),0,ROUND(100*(3*IF(J34="J",1,IF(J34="N",0,0.5))+3*IF(K34="J",1,IF(K34="N",0,0.5))+2*IF(L34="J",1,IF(L34="N",0,0.5))+2*IF(M34="J",1,IF(M34="N",0,0.5))+1*IF(N34="J",1,IF(N34="N",0,0.5))+1*IF(O34="J",1,IF(O34="N",0,0.5))+1*IF(P34="J",1,IF(P34="N",0,0.5))+1*IF(Q34="J",1,IF(Q34="N",0,0.5))+2*IF(R34="J",1,IF(R34="N",0,0.5))+3*IF(S34="J",1,IF(S34="N",0,0.5)))/19,0)))</f>
+        <f>IF(A34="","",IF(OR(C34="Etagenwohnung",I34="N",J34="N"),0,ROUND(100*(3*IF(J34="J",1,IF(J34="N",0,0.5))+3*IF(K34="J",1,IF(K34="N",0,0.5))+2*IF(L34="J",1,IF(L34="N",0,0.5))+2*IF(M34="J",1,IF(M34="N",0,0.5))+1*IF(N34="J",1,IF(N34="N",0,0.5))+1*IF(O34="J",1,IF(O34="N",0,0.5))+1*IF(P34="J",1,IF(P34="N",0,0.5))+1*IF(Q34="J",1,IF(Q34="N",0,0.5))+2*IF(R34="J",1,IF(R34="N",0,0.5))+3*IF(S34="J",1,IF(S34="N",0,0.5))+IF(T34="",0,1*IF(T34="?",0.5,MAX(0,1-T34/3.57))))/(19+IF(T34="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G34" s="10" t="n"/>
@@ -2293,6 +2755,15 @@
         <f>IF(A34="","",IF(E34="","?",IF(AND(E34&gt;=90,E34&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T34" s="11" t="n"/>
+      <c r="U34" s="9">
+        <f>IF(OR(D34="",T34="",T34="?"),"",ROUND(D34*(Legende!$B$9+Legende!$B$10+T34/100),0))</f>
+        <v/>
+      </c>
+      <c r="V34" s="9">
+        <f>IF(U34="","",D34+U34)</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="n"/>
@@ -2301,7 +2772,7 @@
       <c r="D35" s="9" t="n"/>
       <c r="E35" s="10" t="n"/>
       <c r="F35" s="10">
-        <f>IF(A35="","",IF(OR(C35="Etagenwohnung",I35="N"),0,ROUND(100*(3*IF(J35="J",1,IF(J35="N",0,0.5))+3*IF(K35="J",1,IF(K35="N",0,0.5))+2*IF(L35="J",1,IF(L35="N",0,0.5))+2*IF(M35="J",1,IF(M35="N",0,0.5))+1*IF(N35="J",1,IF(N35="N",0,0.5))+1*IF(O35="J",1,IF(O35="N",0,0.5))+1*IF(P35="J",1,IF(P35="N",0,0.5))+1*IF(Q35="J",1,IF(Q35="N",0,0.5))+2*IF(R35="J",1,IF(R35="N",0,0.5))+3*IF(S35="J",1,IF(S35="N",0,0.5)))/19,0)))</f>
+        <f>IF(A35="","",IF(OR(C35="Etagenwohnung",I35="N",J35="N"),0,ROUND(100*(3*IF(J35="J",1,IF(J35="N",0,0.5))+3*IF(K35="J",1,IF(K35="N",0,0.5))+2*IF(L35="J",1,IF(L35="N",0,0.5))+2*IF(M35="J",1,IF(M35="N",0,0.5))+1*IF(N35="J",1,IF(N35="N",0,0.5))+1*IF(O35="J",1,IF(O35="N",0,0.5))+1*IF(P35="J",1,IF(P35="N",0,0.5))+1*IF(Q35="J",1,IF(Q35="N",0,0.5))+2*IF(R35="J",1,IF(R35="N",0,0.5))+3*IF(S35="J",1,IF(S35="N",0,0.5))+IF(T35="",0,1*IF(T35="?",0.5,MAX(0,1-T35/3.57))))/(19+IF(T35="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G35" s="10" t="n"/>
@@ -2323,6 +2794,15 @@
         <f>IF(A35="","",IF(E35="","?",IF(AND(E35&gt;=90,E35&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T35" s="11" t="n"/>
+      <c r="U35" s="9">
+        <f>IF(OR(D35="",T35="",T35="?"),"",ROUND(D35*(Legende!$B$9+Legende!$B$10+T35/100),0))</f>
+        <v/>
+      </c>
+      <c r="V35" s="9">
+        <f>IF(U35="","",D35+U35)</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="8" t="n"/>
@@ -2331,7 +2811,7 @@
       <c r="D36" s="9" t="n"/>
       <c r="E36" s="10" t="n"/>
       <c r="F36" s="10">
-        <f>IF(A36="","",IF(OR(C36="Etagenwohnung",I36="N"),0,ROUND(100*(3*IF(J36="J",1,IF(J36="N",0,0.5))+3*IF(K36="J",1,IF(K36="N",0,0.5))+2*IF(L36="J",1,IF(L36="N",0,0.5))+2*IF(M36="J",1,IF(M36="N",0,0.5))+1*IF(N36="J",1,IF(N36="N",0,0.5))+1*IF(O36="J",1,IF(O36="N",0,0.5))+1*IF(P36="J",1,IF(P36="N",0,0.5))+1*IF(Q36="J",1,IF(Q36="N",0,0.5))+2*IF(R36="J",1,IF(R36="N",0,0.5))+3*IF(S36="J",1,IF(S36="N",0,0.5)))/19,0)))</f>
+        <f>IF(A36="","",IF(OR(C36="Etagenwohnung",I36="N",J36="N"),0,ROUND(100*(3*IF(J36="J",1,IF(J36="N",0,0.5))+3*IF(K36="J",1,IF(K36="N",0,0.5))+2*IF(L36="J",1,IF(L36="N",0,0.5))+2*IF(M36="J",1,IF(M36="N",0,0.5))+1*IF(N36="J",1,IF(N36="N",0,0.5))+1*IF(O36="J",1,IF(O36="N",0,0.5))+1*IF(P36="J",1,IF(P36="N",0,0.5))+1*IF(Q36="J",1,IF(Q36="N",0,0.5))+2*IF(R36="J",1,IF(R36="N",0,0.5))+3*IF(S36="J",1,IF(S36="N",0,0.5))+IF(T36="",0,1*IF(T36="?",0.5,MAX(0,1-T36/3.57))))/(19+IF(T36="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G36" s="10" t="n"/>
@@ -2353,6 +2833,15 @@
         <f>IF(A36="","",IF(E36="","?",IF(AND(E36&gt;=90,E36&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T36" s="11" t="n"/>
+      <c r="U36" s="9">
+        <f>IF(OR(D36="",T36="",T36="?"),"",ROUND(D36*(Legende!$B$9+Legende!$B$10+T36/100),0))</f>
+        <v/>
+      </c>
+      <c r="V36" s="9">
+        <f>IF(U36="","",D36+U36)</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="n"/>
@@ -2361,7 +2850,7 @@
       <c r="D37" s="9" t="n"/>
       <c r="E37" s="10" t="n"/>
       <c r="F37" s="10">
-        <f>IF(A37="","",IF(OR(C37="Etagenwohnung",I37="N"),0,ROUND(100*(3*IF(J37="J",1,IF(J37="N",0,0.5))+3*IF(K37="J",1,IF(K37="N",0,0.5))+2*IF(L37="J",1,IF(L37="N",0,0.5))+2*IF(M37="J",1,IF(M37="N",0,0.5))+1*IF(N37="J",1,IF(N37="N",0,0.5))+1*IF(O37="J",1,IF(O37="N",0,0.5))+1*IF(P37="J",1,IF(P37="N",0,0.5))+1*IF(Q37="J",1,IF(Q37="N",0,0.5))+2*IF(R37="J",1,IF(R37="N",0,0.5))+3*IF(S37="J",1,IF(S37="N",0,0.5)))/19,0)))</f>
+        <f>IF(A37="","",IF(OR(C37="Etagenwohnung",I37="N",J37="N"),0,ROUND(100*(3*IF(J37="J",1,IF(J37="N",0,0.5))+3*IF(K37="J",1,IF(K37="N",0,0.5))+2*IF(L37="J",1,IF(L37="N",0,0.5))+2*IF(M37="J",1,IF(M37="N",0,0.5))+1*IF(N37="J",1,IF(N37="N",0,0.5))+1*IF(O37="J",1,IF(O37="N",0,0.5))+1*IF(P37="J",1,IF(P37="N",0,0.5))+1*IF(Q37="J",1,IF(Q37="N",0,0.5))+2*IF(R37="J",1,IF(R37="N",0,0.5))+3*IF(S37="J",1,IF(S37="N",0,0.5))+IF(T37="",0,1*IF(T37="?",0.5,MAX(0,1-T37/3.57))))/(19+IF(T37="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G37" s="10" t="n"/>
@@ -2383,6 +2872,15 @@
         <f>IF(A37="","",IF(E37="","?",IF(AND(E37&gt;=90,E37&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T37" s="11" t="n"/>
+      <c r="U37" s="9">
+        <f>IF(OR(D37="",T37="",T37="?"),"",ROUND(D37*(Legende!$B$9+Legende!$B$10+T37/100),0))</f>
+        <v/>
+      </c>
+      <c r="V37" s="9">
+        <f>IF(U37="","",D37+U37)</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="n"/>
@@ -2391,7 +2889,7 @@
       <c r="D38" s="9" t="n"/>
       <c r="E38" s="10" t="n"/>
       <c r="F38" s="10">
-        <f>IF(A38="","",IF(OR(C38="Etagenwohnung",I38="N"),0,ROUND(100*(3*IF(J38="J",1,IF(J38="N",0,0.5))+3*IF(K38="J",1,IF(K38="N",0,0.5))+2*IF(L38="J",1,IF(L38="N",0,0.5))+2*IF(M38="J",1,IF(M38="N",0,0.5))+1*IF(N38="J",1,IF(N38="N",0,0.5))+1*IF(O38="J",1,IF(O38="N",0,0.5))+1*IF(P38="J",1,IF(P38="N",0,0.5))+1*IF(Q38="J",1,IF(Q38="N",0,0.5))+2*IF(R38="J",1,IF(R38="N",0,0.5))+3*IF(S38="J",1,IF(S38="N",0,0.5)))/19,0)))</f>
+        <f>IF(A38="","",IF(OR(C38="Etagenwohnung",I38="N",J38="N"),0,ROUND(100*(3*IF(J38="J",1,IF(J38="N",0,0.5))+3*IF(K38="J",1,IF(K38="N",0,0.5))+2*IF(L38="J",1,IF(L38="N",0,0.5))+2*IF(M38="J",1,IF(M38="N",0,0.5))+1*IF(N38="J",1,IF(N38="N",0,0.5))+1*IF(O38="J",1,IF(O38="N",0,0.5))+1*IF(P38="J",1,IF(P38="N",0,0.5))+1*IF(Q38="J",1,IF(Q38="N",0,0.5))+2*IF(R38="J",1,IF(R38="N",0,0.5))+3*IF(S38="J",1,IF(S38="N",0,0.5))+IF(T38="",0,1*IF(T38="?",0.5,MAX(0,1-T38/3.57))))/(19+IF(T38="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G38" s="10" t="n"/>
@@ -2413,6 +2911,15 @@
         <f>IF(A38="","",IF(E38="","?",IF(AND(E38&gt;=90,E38&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T38" s="11" t="n"/>
+      <c r="U38" s="9">
+        <f>IF(OR(D38="",T38="",T38="?"),"",ROUND(D38*(Legende!$B$9+Legende!$B$10+T38/100),0))</f>
+        <v/>
+      </c>
+      <c r="V38" s="9">
+        <f>IF(U38="","",D38+U38)</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="8" t="n"/>
@@ -2421,7 +2928,7 @@
       <c r="D39" s="9" t="n"/>
       <c r="E39" s="10" t="n"/>
       <c r="F39" s="10">
-        <f>IF(A39="","",IF(OR(C39="Etagenwohnung",I39="N"),0,ROUND(100*(3*IF(J39="J",1,IF(J39="N",0,0.5))+3*IF(K39="J",1,IF(K39="N",0,0.5))+2*IF(L39="J",1,IF(L39="N",0,0.5))+2*IF(M39="J",1,IF(M39="N",0,0.5))+1*IF(N39="J",1,IF(N39="N",0,0.5))+1*IF(O39="J",1,IF(O39="N",0,0.5))+1*IF(P39="J",1,IF(P39="N",0,0.5))+1*IF(Q39="J",1,IF(Q39="N",0,0.5))+2*IF(R39="J",1,IF(R39="N",0,0.5))+3*IF(S39="J",1,IF(S39="N",0,0.5)))/19,0)))</f>
+        <f>IF(A39="","",IF(OR(C39="Etagenwohnung",I39="N",J39="N"),0,ROUND(100*(3*IF(J39="J",1,IF(J39="N",0,0.5))+3*IF(K39="J",1,IF(K39="N",0,0.5))+2*IF(L39="J",1,IF(L39="N",0,0.5))+2*IF(M39="J",1,IF(M39="N",0,0.5))+1*IF(N39="J",1,IF(N39="N",0,0.5))+1*IF(O39="J",1,IF(O39="N",0,0.5))+1*IF(P39="J",1,IF(P39="N",0,0.5))+1*IF(Q39="J",1,IF(Q39="N",0,0.5))+2*IF(R39="J",1,IF(R39="N",0,0.5))+3*IF(S39="J",1,IF(S39="N",0,0.5))+IF(T39="",0,1*IF(T39="?",0.5,MAX(0,1-T39/3.57))))/(19+IF(T39="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G39" s="10" t="n"/>
@@ -2443,6 +2950,15 @@
         <f>IF(A39="","",IF(E39="","?",IF(AND(E39&gt;=90,E39&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T39" s="11" t="n"/>
+      <c r="U39" s="9">
+        <f>IF(OR(D39="",T39="",T39="?"),"",ROUND(D39*(Legende!$B$9+Legende!$B$10+T39/100),0))</f>
+        <v/>
+      </c>
+      <c r="V39" s="9">
+        <f>IF(U39="","",D39+U39)</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="8" t="n"/>
@@ -2451,7 +2967,7 @@
       <c r="D40" s="9" t="n"/>
       <c r="E40" s="10" t="n"/>
       <c r="F40" s="10">
-        <f>IF(A40="","",IF(OR(C40="Etagenwohnung",I40="N"),0,ROUND(100*(3*IF(J40="J",1,IF(J40="N",0,0.5))+3*IF(K40="J",1,IF(K40="N",0,0.5))+2*IF(L40="J",1,IF(L40="N",0,0.5))+2*IF(M40="J",1,IF(M40="N",0,0.5))+1*IF(N40="J",1,IF(N40="N",0,0.5))+1*IF(O40="J",1,IF(O40="N",0,0.5))+1*IF(P40="J",1,IF(P40="N",0,0.5))+1*IF(Q40="J",1,IF(Q40="N",0,0.5))+2*IF(R40="J",1,IF(R40="N",0,0.5))+3*IF(S40="J",1,IF(S40="N",0,0.5)))/19,0)))</f>
+        <f>IF(A40="","",IF(OR(C40="Etagenwohnung",I40="N",J40="N"),0,ROUND(100*(3*IF(J40="J",1,IF(J40="N",0,0.5))+3*IF(K40="J",1,IF(K40="N",0,0.5))+2*IF(L40="J",1,IF(L40="N",0,0.5))+2*IF(M40="J",1,IF(M40="N",0,0.5))+1*IF(N40="J",1,IF(N40="N",0,0.5))+1*IF(O40="J",1,IF(O40="N",0,0.5))+1*IF(P40="J",1,IF(P40="N",0,0.5))+1*IF(Q40="J",1,IF(Q40="N",0,0.5))+2*IF(R40="J",1,IF(R40="N",0,0.5))+3*IF(S40="J",1,IF(S40="N",0,0.5))+IF(T40="",0,1*IF(T40="?",0.5,MAX(0,1-T40/3.57))))/(19+IF(T40="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G40" s="10" t="n"/>
@@ -2473,6 +2989,15 @@
         <f>IF(A40="","",IF(E40="","?",IF(AND(E40&gt;=90,E40&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T40" s="11" t="n"/>
+      <c r="U40" s="9">
+        <f>IF(OR(D40="",T40="",T40="?"),"",ROUND(D40*(Legende!$B$9+Legende!$B$10+T40/100),0))</f>
+        <v/>
+      </c>
+      <c r="V40" s="9">
+        <f>IF(U40="","",D40+U40)</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="n"/>
@@ -2481,7 +3006,7 @@
       <c r="D41" s="9" t="n"/>
       <c r="E41" s="10" t="n"/>
       <c r="F41" s="10">
-        <f>IF(A41="","",IF(OR(C41="Etagenwohnung",I41="N"),0,ROUND(100*(3*IF(J41="J",1,IF(J41="N",0,0.5))+3*IF(K41="J",1,IF(K41="N",0,0.5))+2*IF(L41="J",1,IF(L41="N",0,0.5))+2*IF(M41="J",1,IF(M41="N",0,0.5))+1*IF(N41="J",1,IF(N41="N",0,0.5))+1*IF(O41="J",1,IF(O41="N",0,0.5))+1*IF(P41="J",1,IF(P41="N",0,0.5))+1*IF(Q41="J",1,IF(Q41="N",0,0.5))+2*IF(R41="J",1,IF(R41="N",0,0.5))+3*IF(S41="J",1,IF(S41="N",0,0.5)))/19,0)))</f>
+        <f>IF(A41="","",IF(OR(C41="Etagenwohnung",I41="N",J41="N"),0,ROUND(100*(3*IF(J41="J",1,IF(J41="N",0,0.5))+3*IF(K41="J",1,IF(K41="N",0,0.5))+2*IF(L41="J",1,IF(L41="N",0,0.5))+2*IF(M41="J",1,IF(M41="N",0,0.5))+1*IF(N41="J",1,IF(N41="N",0,0.5))+1*IF(O41="J",1,IF(O41="N",0,0.5))+1*IF(P41="J",1,IF(P41="N",0,0.5))+1*IF(Q41="J",1,IF(Q41="N",0,0.5))+2*IF(R41="J",1,IF(R41="N",0,0.5))+3*IF(S41="J",1,IF(S41="N",0,0.5))+IF(T41="",0,1*IF(T41="?",0.5,MAX(0,1-T41/3.57))))/(19+IF(T41="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G41" s="10" t="n"/>
@@ -2503,6 +3028,15 @@
         <f>IF(A41="","",IF(E41="","?",IF(AND(E41&gt;=90,E41&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T41" s="11" t="n"/>
+      <c r="U41" s="9">
+        <f>IF(OR(D41="",T41="",T41="?"),"",ROUND(D41*(Legende!$B$9+Legende!$B$10+T41/100),0))</f>
+        <v/>
+      </c>
+      <c r="V41" s="9">
+        <f>IF(U41="","",D41+U41)</f>
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="8" t="n"/>
@@ -2511,7 +3045,7 @@
       <c r="D42" s="9" t="n"/>
       <c r="E42" s="10" t="n"/>
       <c r="F42" s="10">
-        <f>IF(A42="","",IF(OR(C42="Etagenwohnung",I42="N"),0,ROUND(100*(3*IF(J42="J",1,IF(J42="N",0,0.5))+3*IF(K42="J",1,IF(K42="N",0,0.5))+2*IF(L42="J",1,IF(L42="N",0,0.5))+2*IF(M42="J",1,IF(M42="N",0,0.5))+1*IF(N42="J",1,IF(N42="N",0,0.5))+1*IF(O42="J",1,IF(O42="N",0,0.5))+1*IF(P42="J",1,IF(P42="N",0,0.5))+1*IF(Q42="J",1,IF(Q42="N",0,0.5))+2*IF(R42="J",1,IF(R42="N",0,0.5))+3*IF(S42="J",1,IF(S42="N",0,0.5)))/19,0)))</f>
+        <f>IF(A42="","",IF(OR(C42="Etagenwohnung",I42="N",J42="N"),0,ROUND(100*(3*IF(J42="J",1,IF(J42="N",0,0.5))+3*IF(K42="J",1,IF(K42="N",0,0.5))+2*IF(L42="J",1,IF(L42="N",0,0.5))+2*IF(M42="J",1,IF(M42="N",0,0.5))+1*IF(N42="J",1,IF(N42="N",0,0.5))+1*IF(O42="J",1,IF(O42="N",0,0.5))+1*IF(P42="J",1,IF(P42="N",0,0.5))+1*IF(Q42="J",1,IF(Q42="N",0,0.5))+2*IF(R42="J",1,IF(R42="N",0,0.5))+3*IF(S42="J",1,IF(S42="N",0,0.5))+IF(T42="",0,1*IF(T42="?",0.5,MAX(0,1-T42/3.57))))/(19+IF(T42="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G42" s="10" t="n"/>
@@ -2533,6 +3067,15 @@
         <f>IF(A42="","",IF(E42="","?",IF(AND(E42&gt;=90,E42&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T42" s="11" t="n"/>
+      <c r="U42" s="9">
+        <f>IF(OR(D42="",T42="",T42="?"),"",ROUND(D42*(Legende!$B$9+Legende!$B$10+T42/100),0))</f>
+        <v/>
+      </c>
+      <c r="V42" s="9">
+        <f>IF(U42="","",D42+U42)</f>
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="n"/>
@@ -2541,7 +3084,7 @@
       <c r="D43" s="9" t="n"/>
       <c r="E43" s="10" t="n"/>
       <c r="F43" s="10">
-        <f>IF(A43="","",IF(OR(C43="Etagenwohnung",I43="N"),0,ROUND(100*(3*IF(J43="J",1,IF(J43="N",0,0.5))+3*IF(K43="J",1,IF(K43="N",0,0.5))+2*IF(L43="J",1,IF(L43="N",0,0.5))+2*IF(M43="J",1,IF(M43="N",0,0.5))+1*IF(N43="J",1,IF(N43="N",0,0.5))+1*IF(O43="J",1,IF(O43="N",0,0.5))+1*IF(P43="J",1,IF(P43="N",0,0.5))+1*IF(Q43="J",1,IF(Q43="N",0,0.5))+2*IF(R43="J",1,IF(R43="N",0,0.5))+3*IF(S43="J",1,IF(S43="N",0,0.5)))/19,0)))</f>
+        <f>IF(A43="","",IF(OR(C43="Etagenwohnung",I43="N",J43="N"),0,ROUND(100*(3*IF(J43="J",1,IF(J43="N",0,0.5))+3*IF(K43="J",1,IF(K43="N",0,0.5))+2*IF(L43="J",1,IF(L43="N",0,0.5))+2*IF(M43="J",1,IF(M43="N",0,0.5))+1*IF(N43="J",1,IF(N43="N",0,0.5))+1*IF(O43="J",1,IF(O43="N",0,0.5))+1*IF(P43="J",1,IF(P43="N",0,0.5))+1*IF(Q43="J",1,IF(Q43="N",0,0.5))+2*IF(R43="J",1,IF(R43="N",0,0.5))+3*IF(S43="J",1,IF(S43="N",0,0.5))+IF(T43="",0,1*IF(T43="?",0.5,MAX(0,1-T43/3.57))))/(19+IF(T43="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G43" s="10" t="n"/>
@@ -2563,6 +3106,15 @@
         <f>IF(A43="","",IF(E43="","?",IF(AND(E43&gt;=90,E43&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T43" s="11" t="n"/>
+      <c r="U43" s="9">
+        <f>IF(OR(D43="",T43="",T43="?"),"",ROUND(D43*(Legende!$B$9+Legende!$B$10+T43/100),0))</f>
+        <v/>
+      </c>
+      <c r="V43" s="9">
+        <f>IF(U43="","",D43+U43)</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="8" t="n"/>
@@ -2571,7 +3123,7 @@
       <c r="D44" s="9" t="n"/>
       <c r="E44" s="10" t="n"/>
       <c r="F44" s="10">
-        <f>IF(A44="","",IF(OR(C44="Etagenwohnung",I44="N"),0,ROUND(100*(3*IF(J44="J",1,IF(J44="N",0,0.5))+3*IF(K44="J",1,IF(K44="N",0,0.5))+2*IF(L44="J",1,IF(L44="N",0,0.5))+2*IF(M44="J",1,IF(M44="N",0,0.5))+1*IF(N44="J",1,IF(N44="N",0,0.5))+1*IF(O44="J",1,IF(O44="N",0,0.5))+1*IF(P44="J",1,IF(P44="N",0,0.5))+1*IF(Q44="J",1,IF(Q44="N",0,0.5))+2*IF(R44="J",1,IF(R44="N",0,0.5))+3*IF(S44="J",1,IF(S44="N",0,0.5)))/19,0)))</f>
+        <f>IF(A44="","",IF(OR(C44="Etagenwohnung",I44="N",J44="N"),0,ROUND(100*(3*IF(J44="J",1,IF(J44="N",0,0.5))+3*IF(K44="J",1,IF(K44="N",0,0.5))+2*IF(L44="J",1,IF(L44="N",0,0.5))+2*IF(M44="J",1,IF(M44="N",0,0.5))+1*IF(N44="J",1,IF(N44="N",0,0.5))+1*IF(O44="J",1,IF(O44="N",0,0.5))+1*IF(P44="J",1,IF(P44="N",0,0.5))+1*IF(Q44="J",1,IF(Q44="N",0,0.5))+2*IF(R44="J",1,IF(R44="N",0,0.5))+3*IF(S44="J",1,IF(S44="N",0,0.5))+IF(T44="",0,1*IF(T44="?",0.5,MAX(0,1-T44/3.57))))/(19+IF(T44="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G44" s="10" t="n"/>
@@ -2593,6 +3145,15 @@
         <f>IF(A44="","",IF(E44="","?",IF(AND(E44&gt;=90,E44&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T44" s="11" t="n"/>
+      <c r="U44" s="9">
+        <f>IF(OR(D44="",T44="",T44="?"),"",ROUND(D44*(Legende!$B$9+Legende!$B$10+T44/100),0))</f>
+        <v/>
+      </c>
+      <c r="V44" s="9">
+        <f>IF(U44="","",D44+U44)</f>
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="8" t="n"/>
@@ -2601,7 +3162,7 @@
       <c r="D45" s="9" t="n"/>
       <c r="E45" s="10" t="n"/>
       <c r="F45" s="10">
-        <f>IF(A45="","",IF(OR(C45="Etagenwohnung",I45="N"),0,ROUND(100*(3*IF(J45="J",1,IF(J45="N",0,0.5))+3*IF(K45="J",1,IF(K45="N",0,0.5))+2*IF(L45="J",1,IF(L45="N",0,0.5))+2*IF(M45="J",1,IF(M45="N",0,0.5))+1*IF(N45="J",1,IF(N45="N",0,0.5))+1*IF(O45="J",1,IF(O45="N",0,0.5))+1*IF(P45="J",1,IF(P45="N",0,0.5))+1*IF(Q45="J",1,IF(Q45="N",0,0.5))+2*IF(R45="J",1,IF(R45="N",0,0.5))+3*IF(S45="J",1,IF(S45="N",0,0.5)))/19,0)))</f>
+        <f>IF(A45="","",IF(OR(C45="Etagenwohnung",I45="N",J45="N"),0,ROUND(100*(3*IF(J45="J",1,IF(J45="N",0,0.5))+3*IF(K45="J",1,IF(K45="N",0,0.5))+2*IF(L45="J",1,IF(L45="N",0,0.5))+2*IF(M45="J",1,IF(M45="N",0,0.5))+1*IF(N45="J",1,IF(N45="N",0,0.5))+1*IF(O45="J",1,IF(O45="N",0,0.5))+1*IF(P45="J",1,IF(P45="N",0,0.5))+1*IF(Q45="J",1,IF(Q45="N",0,0.5))+2*IF(R45="J",1,IF(R45="N",0,0.5))+3*IF(S45="J",1,IF(S45="N",0,0.5))+IF(T45="",0,1*IF(T45="?",0.5,MAX(0,1-T45/3.57))))/(19+IF(T45="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G45" s="10" t="n"/>
@@ -2623,6 +3184,15 @@
         <f>IF(A45="","",IF(E45="","?",IF(AND(E45&gt;=90,E45&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T45" s="11" t="n"/>
+      <c r="U45" s="9">
+        <f>IF(OR(D45="",T45="",T45="?"),"",ROUND(D45*(Legende!$B$9+Legende!$B$10+T45/100),0))</f>
+        <v/>
+      </c>
+      <c r="V45" s="9">
+        <f>IF(U45="","",D45+U45)</f>
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="8" t="n"/>
@@ -2631,7 +3201,7 @@
       <c r="D46" s="9" t="n"/>
       <c r="E46" s="10" t="n"/>
       <c r="F46" s="10">
-        <f>IF(A46="","",IF(OR(C46="Etagenwohnung",I46="N"),0,ROUND(100*(3*IF(J46="J",1,IF(J46="N",0,0.5))+3*IF(K46="J",1,IF(K46="N",0,0.5))+2*IF(L46="J",1,IF(L46="N",0,0.5))+2*IF(M46="J",1,IF(M46="N",0,0.5))+1*IF(N46="J",1,IF(N46="N",0,0.5))+1*IF(O46="J",1,IF(O46="N",0,0.5))+1*IF(P46="J",1,IF(P46="N",0,0.5))+1*IF(Q46="J",1,IF(Q46="N",0,0.5))+2*IF(R46="J",1,IF(R46="N",0,0.5))+3*IF(S46="J",1,IF(S46="N",0,0.5)))/19,0)))</f>
+        <f>IF(A46="","",IF(OR(C46="Etagenwohnung",I46="N",J46="N"),0,ROUND(100*(3*IF(J46="J",1,IF(J46="N",0,0.5))+3*IF(K46="J",1,IF(K46="N",0,0.5))+2*IF(L46="J",1,IF(L46="N",0,0.5))+2*IF(M46="J",1,IF(M46="N",0,0.5))+1*IF(N46="J",1,IF(N46="N",0,0.5))+1*IF(O46="J",1,IF(O46="N",0,0.5))+1*IF(P46="J",1,IF(P46="N",0,0.5))+1*IF(Q46="J",1,IF(Q46="N",0,0.5))+2*IF(R46="J",1,IF(R46="N",0,0.5))+3*IF(S46="J",1,IF(S46="N",0,0.5))+IF(T46="",0,1*IF(T46="?",0.5,MAX(0,1-T46/3.57))))/(19+IF(T46="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G46" s="10" t="n"/>
@@ -2653,6 +3223,15 @@
         <f>IF(A46="","",IF(E46="","?",IF(AND(E46&gt;=90,E46&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T46" s="11" t="n"/>
+      <c r="U46" s="9">
+        <f>IF(OR(D46="",T46="",T46="?"),"",ROUND(D46*(Legende!$B$9+Legende!$B$10+T46/100),0))</f>
+        <v/>
+      </c>
+      <c r="V46" s="9">
+        <f>IF(U46="","",D46+U46)</f>
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="8" t="n"/>
@@ -2661,7 +3240,7 @@
       <c r="D47" s="9" t="n"/>
       <c r="E47" s="10" t="n"/>
       <c r="F47" s="10">
-        <f>IF(A47="","",IF(OR(C47="Etagenwohnung",I47="N"),0,ROUND(100*(3*IF(J47="J",1,IF(J47="N",0,0.5))+3*IF(K47="J",1,IF(K47="N",0,0.5))+2*IF(L47="J",1,IF(L47="N",0,0.5))+2*IF(M47="J",1,IF(M47="N",0,0.5))+1*IF(N47="J",1,IF(N47="N",0,0.5))+1*IF(O47="J",1,IF(O47="N",0,0.5))+1*IF(P47="J",1,IF(P47="N",0,0.5))+1*IF(Q47="J",1,IF(Q47="N",0,0.5))+2*IF(R47="J",1,IF(R47="N",0,0.5))+3*IF(S47="J",1,IF(S47="N",0,0.5)))/19,0)))</f>
+        <f>IF(A47="","",IF(OR(C47="Etagenwohnung",I47="N",J47="N"),0,ROUND(100*(3*IF(J47="J",1,IF(J47="N",0,0.5))+3*IF(K47="J",1,IF(K47="N",0,0.5))+2*IF(L47="J",1,IF(L47="N",0,0.5))+2*IF(M47="J",1,IF(M47="N",0,0.5))+1*IF(N47="J",1,IF(N47="N",0,0.5))+1*IF(O47="J",1,IF(O47="N",0,0.5))+1*IF(P47="J",1,IF(P47="N",0,0.5))+1*IF(Q47="J",1,IF(Q47="N",0,0.5))+2*IF(R47="J",1,IF(R47="N",0,0.5))+3*IF(S47="J",1,IF(S47="N",0,0.5))+IF(T47="",0,1*IF(T47="?",0.5,MAX(0,1-T47/3.57))))/(19+IF(T47="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G47" s="10" t="n"/>
@@ -2683,6 +3262,15 @@
         <f>IF(A47="","",IF(E47="","?",IF(AND(E47&gt;=90,E47&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T47" s="11" t="n"/>
+      <c r="U47" s="9">
+        <f>IF(OR(D47="",T47="",T47="?"),"",ROUND(D47*(Legende!$B$9+Legende!$B$10+T47/100),0))</f>
+        <v/>
+      </c>
+      <c r="V47" s="9">
+        <f>IF(U47="","",D47+U47)</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="8" t="n"/>
@@ -2691,7 +3279,7 @@
       <c r="D48" s="9" t="n"/>
       <c r="E48" s="10" t="n"/>
       <c r="F48" s="10">
-        <f>IF(A48="","",IF(OR(C48="Etagenwohnung",I48="N"),0,ROUND(100*(3*IF(J48="J",1,IF(J48="N",0,0.5))+3*IF(K48="J",1,IF(K48="N",0,0.5))+2*IF(L48="J",1,IF(L48="N",0,0.5))+2*IF(M48="J",1,IF(M48="N",0,0.5))+1*IF(N48="J",1,IF(N48="N",0,0.5))+1*IF(O48="J",1,IF(O48="N",0,0.5))+1*IF(P48="J",1,IF(P48="N",0,0.5))+1*IF(Q48="J",1,IF(Q48="N",0,0.5))+2*IF(R48="J",1,IF(R48="N",0,0.5))+3*IF(S48="J",1,IF(S48="N",0,0.5)))/19,0)))</f>
+        <f>IF(A48="","",IF(OR(C48="Etagenwohnung",I48="N",J48="N"),0,ROUND(100*(3*IF(J48="J",1,IF(J48="N",0,0.5))+3*IF(K48="J",1,IF(K48="N",0,0.5))+2*IF(L48="J",1,IF(L48="N",0,0.5))+2*IF(M48="J",1,IF(M48="N",0,0.5))+1*IF(N48="J",1,IF(N48="N",0,0.5))+1*IF(O48="J",1,IF(O48="N",0,0.5))+1*IF(P48="J",1,IF(P48="N",0,0.5))+1*IF(Q48="J",1,IF(Q48="N",0,0.5))+2*IF(R48="J",1,IF(R48="N",0,0.5))+3*IF(S48="J",1,IF(S48="N",0,0.5))+IF(T48="",0,1*IF(T48="?",0.5,MAX(0,1-T48/3.57))))/(19+IF(T48="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G48" s="10" t="n"/>
@@ -2713,6 +3301,15 @@
         <f>IF(A48="","",IF(E48="","?",IF(AND(E48&gt;=90,E48&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T48" s="11" t="n"/>
+      <c r="U48" s="9">
+        <f>IF(OR(D48="",T48="",T48="?"),"",ROUND(D48*(Legende!$B$9+Legende!$B$10+T48/100),0))</f>
+        <v/>
+      </c>
+      <c r="V48" s="9">
+        <f>IF(U48="","",D48+U48)</f>
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="8" t="n"/>
@@ -2721,7 +3318,7 @@
       <c r="D49" s="9" t="n"/>
       <c r="E49" s="10" t="n"/>
       <c r="F49" s="10">
-        <f>IF(A49="","",IF(OR(C49="Etagenwohnung",I49="N"),0,ROUND(100*(3*IF(J49="J",1,IF(J49="N",0,0.5))+3*IF(K49="J",1,IF(K49="N",0,0.5))+2*IF(L49="J",1,IF(L49="N",0,0.5))+2*IF(M49="J",1,IF(M49="N",0,0.5))+1*IF(N49="J",1,IF(N49="N",0,0.5))+1*IF(O49="J",1,IF(O49="N",0,0.5))+1*IF(P49="J",1,IF(P49="N",0,0.5))+1*IF(Q49="J",1,IF(Q49="N",0,0.5))+2*IF(R49="J",1,IF(R49="N",0,0.5))+3*IF(S49="J",1,IF(S49="N",0,0.5)))/19,0)))</f>
+        <f>IF(A49="","",IF(OR(C49="Etagenwohnung",I49="N",J49="N"),0,ROUND(100*(3*IF(J49="J",1,IF(J49="N",0,0.5))+3*IF(K49="J",1,IF(K49="N",0,0.5))+2*IF(L49="J",1,IF(L49="N",0,0.5))+2*IF(M49="J",1,IF(M49="N",0,0.5))+1*IF(N49="J",1,IF(N49="N",0,0.5))+1*IF(O49="J",1,IF(O49="N",0,0.5))+1*IF(P49="J",1,IF(P49="N",0,0.5))+1*IF(Q49="J",1,IF(Q49="N",0,0.5))+2*IF(R49="J",1,IF(R49="N",0,0.5))+3*IF(S49="J",1,IF(S49="N",0,0.5))+IF(T49="",0,1*IF(T49="?",0.5,MAX(0,1-T49/3.57))))/(19+IF(T49="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G49" s="10" t="n"/>
@@ -2743,6 +3340,15 @@
         <f>IF(A49="","",IF(E49="","?",IF(AND(E49&gt;=90,E49&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T49" s="11" t="n"/>
+      <c r="U49" s="9">
+        <f>IF(OR(D49="",T49="",T49="?"),"",ROUND(D49*(Legende!$B$9+Legende!$B$10+T49/100),0))</f>
+        <v/>
+      </c>
+      <c r="V49" s="9">
+        <f>IF(U49="","",D49+U49)</f>
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="8" t="n"/>
@@ -2751,7 +3357,7 @@
       <c r="D50" s="9" t="n"/>
       <c r="E50" s="10" t="n"/>
       <c r="F50" s="10">
-        <f>IF(A50="","",IF(OR(C50="Etagenwohnung",I50="N"),0,ROUND(100*(3*IF(J50="J",1,IF(J50="N",0,0.5))+3*IF(K50="J",1,IF(K50="N",0,0.5))+2*IF(L50="J",1,IF(L50="N",0,0.5))+2*IF(M50="J",1,IF(M50="N",0,0.5))+1*IF(N50="J",1,IF(N50="N",0,0.5))+1*IF(O50="J",1,IF(O50="N",0,0.5))+1*IF(P50="J",1,IF(P50="N",0,0.5))+1*IF(Q50="J",1,IF(Q50="N",0,0.5))+2*IF(R50="J",1,IF(R50="N",0,0.5))+3*IF(S50="J",1,IF(S50="N",0,0.5)))/19,0)))</f>
+        <f>IF(A50="","",IF(OR(C50="Etagenwohnung",I50="N",J50="N"),0,ROUND(100*(3*IF(J50="J",1,IF(J50="N",0,0.5))+3*IF(K50="J",1,IF(K50="N",0,0.5))+2*IF(L50="J",1,IF(L50="N",0,0.5))+2*IF(M50="J",1,IF(M50="N",0,0.5))+1*IF(N50="J",1,IF(N50="N",0,0.5))+1*IF(O50="J",1,IF(O50="N",0,0.5))+1*IF(P50="J",1,IF(P50="N",0,0.5))+1*IF(Q50="J",1,IF(Q50="N",0,0.5))+2*IF(R50="J",1,IF(R50="N",0,0.5))+3*IF(S50="J",1,IF(S50="N",0,0.5))+IF(T50="",0,1*IF(T50="?",0.5,MAX(0,1-T50/3.57))))/(19+IF(T50="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G50" s="10" t="n"/>
@@ -2773,6 +3379,15 @@
         <f>IF(A50="","",IF(E50="","?",IF(AND(E50&gt;=90,E50&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T50" s="11" t="n"/>
+      <c r="U50" s="9">
+        <f>IF(OR(D50="",T50="",T50="?"),"",ROUND(D50*(Legende!$B$9+Legende!$B$10+T50/100),0))</f>
+        <v/>
+      </c>
+      <c r="V50" s="9">
+        <f>IF(U50="","",D50+U50)</f>
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="8" t="n"/>
@@ -2781,7 +3396,7 @@
       <c r="D51" s="9" t="n"/>
       <c r="E51" s="10" t="n"/>
       <c r="F51" s="10">
-        <f>IF(A51="","",IF(OR(C51="Etagenwohnung",I51="N"),0,ROUND(100*(3*IF(J51="J",1,IF(J51="N",0,0.5))+3*IF(K51="J",1,IF(K51="N",0,0.5))+2*IF(L51="J",1,IF(L51="N",0,0.5))+2*IF(M51="J",1,IF(M51="N",0,0.5))+1*IF(N51="J",1,IF(N51="N",0,0.5))+1*IF(O51="J",1,IF(O51="N",0,0.5))+1*IF(P51="J",1,IF(P51="N",0,0.5))+1*IF(Q51="J",1,IF(Q51="N",0,0.5))+2*IF(R51="J",1,IF(R51="N",0,0.5))+3*IF(S51="J",1,IF(S51="N",0,0.5)))/19,0)))</f>
+        <f>IF(A51="","",IF(OR(C51="Etagenwohnung",I51="N",J51="N"),0,ROUND(100*(3*IF(J51="J",1,IF(J51="N",0,0.5))+3*IF(K51="J",1,IF(K51="N",0,0.5))+2*IF(L51="J",1,IF(L51="N",0,0.5))+2*IF(M51="J",1,IF(M51="N",0,0.5))+1*IF(N51="J",1,IF(N51="N",0,0.5))+1*IF(O51="J",1,IF(O51="N",0,0.5))+1*IF(P51="J",1,IF(P51="N",0,0.5))+1*IF(Q51="J",1,IF(Q51="N",0,0.5))+2*IF(R51="J",1,IF(R51="N",0,0.5))+3*IF(S51="J",1,IF(S51="N",0,0.5))+IF(T51="",0,1*IF(T51="?",0.5,MAX(0,1-T51/3.57))))/(19+IF(T51="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G51" s="10" t="n"/>
@@ -2803,6 +3418,15 @@
         <f>IF(A51="","",IF(E51="","?",IF(AND(E51&gt;=90,E51&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T51" s="11" t="n"/>
+      <c r="U51" s="9">
+        <f>IF(OR(D51="",T51="",T51="?"),"",ROUND(D51*(Legende!$B$9+Legende!$B$10+T51/100),0))</f>
+        <v/>
+      </c>
+      <c r="V51" s="9">
+        <f>IF(U51="","",D51+U51)</f>
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="8" t="n"/>
@@ -2811,7 +3435,7 @@
       <c r="D52" s="9" t="n"/>
       <c r="E52" s="10" t="n"/>
       <c r="F52" s="10">
-        <f>IF(A52="","",IF(OR(C52="Etagenwohnung",I52="N"),0,ROUND(100*(3*IF(J52="J",1,IF(J52="N",0,0.5))+3*IF(K52="J",1,IF(K52="N",0,0.5))+2*IF(L52="J",1,IF(L52="N",0,0.5))+2*IF(M52="J",1,IF(M52="N",0,0.5))+1*IF(N52="J",1,IF(N52="N",0,0.5))+1*IF(O52="J",1,IF(O52="N",0,0.5))+1*IF(P52="J",1,IF(P52="N",0,0.5))+1*IF(Q52="J",1,IF(Q52="N",0,0.5))+2*IF(R52="J",1,IF(R52="N",0,0.5))+3*IF(S52="J",1,IF(S52="N",0,0.5)))/19,0)))</f>
+        <f>IF(A52="","",IF(OR(C52="Etagenwohnung",I52="N",J52="N"),0,ROUND(100*(3*IF(J52="J",1,IF(J52="N",0,0.5))+3*IF(K52="J",1,IF(K52="N",0,0.5))+2*IF(L52="J",1,IF(L52="N",0,0.5))+2*IF(M52="J",1,IF(M52="N",0,0.5))+1*IF(N52="J",1,IF(N52="N",0,0.5))+1*IF(O52="J",1,IF(O52="N",0,0.5))+1*IF(P52="J",1,IF(P52="N",0,0.5))+1*IF(Q52="J",1,IF(Q52="N",0,0.5))+2*IF(R52="J",1,IF(R52="N",0,0.5))+3*IF(S52="J",1,IF(S52="N",0,0.5))+IF(T52="",0,1*IF(T52="?",0.5,MAX(0,1-T52/3.57))))/(19+IF(T52="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G52" s="10" t="n"/>
@@ -2833,6 +3457,15 @@
         <f>IF(A52="","",IF(E52="","?",IF(AND(E52&gt;=90,E52&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T52" s="11" t="n"/>
+      <c r="U52" s="9">
+        <f>IF(OR(D52="",T52="",T52="?"),"",ROUND(D52*(Legende!$B$9+Legende!$B$10+T52/100),0))</f>
+        <v/>
+      </c>
+      <c r="V52" s="9">
+        <f>IF(U52="","",D52+U52)</f>
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="8" t="n"/>
@@ -2841,7 +3474,7 @@
       <c r="D53" s="9" t="n"/>
       <c r="E53" s="10" t="n"/>
       <c r="F53" s="10">
-        <f>IF(A53="","",IF(OR(C53="Etagenwohnung",I53="N"),0,ROUND(100*(3*IF(J53="J",1,IF(J53="N",0,0.5))+3*IF(K53="J",1,IF(K53="N",0,0.5))+2*IF(L53="J",1,IF(L53="N",0,0.5))+2*IF(M53="J",1,IF(M53="N",0,0.5))+1*IF(N53="J",1,IF(N53="N",0,0.5))+1*IF(O53="J",1,IF(O53="N",0,0.5))+1*IF(P53="J",1,IF(P53="N",0,0.5))+1*IF(Q53="J",1,IF(Q53="N",0,0.5))+2*IF(R53="J",1,IF(R53="N",0,0.5))+3*IF(S53="J",1,IF(S53="N",0,0.5)))/19,0)))</f>
+        <f>IF(A53="","",IF(OR(C53="Etagenwohnung",I53="N",J53="N"),0,ROUND(100*(3*IF(J53="J",1,IF(J53="N",0,0.5))+3*IF(K53="J",1,IF(K53="N",0,0.5))+2*IF(L53="J",1,IF(L53="N",0,0.5))+2*IF(M53="J",1,IF(M53="N",0,0.5))+1*IF(N53="J",1,IF(N53="N",0,0.5))+1*IF(O53="J",1,IF(O53="N",0,0.5))+1*IF(P53="J",1,IF(P53="N",0,0.5))+1*IF(Q53="J",1,IF(Q53="N",0,0.5))+2*IF(R53="J",1,IF(R53="N",0,0.5))+3*IF(S53="J",1,IF(S53="N",0,0.5))+IF(T53="",0,1*IF(T53="?",0.5,MAX(0,1-T53/3.57))))/(19+IF(T53="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G53" s="10" t="n"/>
@@ -2863,6 +3496,15 @@
         <f>IF(A53="","",IF(E53="","?",IF(AND(E53&gt;=90,E53&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T53" s="11" t="n"/>
+      <c r="U53" s="9">
+        <f>IF(OR(D53="",T53="",T53="?"),"",ROUND(D53*(Legende!$B$9+Legende!$B$10+T53/100),0))</f>
+        <v/>
+      </c>
+      <c r="V53" s="9">
+        <f>IF(U53="","",D53+U53)</f>
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="8" t="n"/>
@@ -2871,7 +3513,7 @@
       <c r="D54" s="9" t="n"/>
       <c r="E54" s="10" t="n"/>
       <c r="F54" s="10">
-        <f>IF(A54="","",IF(OR(C54="Etagenwohnung",I54="N"),0,ROUND(100*(3*IF(J54="J",1,IF(J54="N",0,0.5))+3*IF(K54="J",1,IF(K54="N",0,0.5))+2*IF(L54="J",1,IF(L54="N",0,0.5))+2*IF(M54="J",1,IF(M54="N",0,0.5))+1*IF(N54="J",1,IF(N54="N",0,0.5))+1*IF(O54="J",1,IF(O54="N",0,0.5))+1*IF(P54="J",1,IF(P54="N",0,0.5))+1*IF(Q54="J",1,IF(Q54="N",0,0.5))+2*IF(R54="J",1,IF(R54="N",0,0.5))+3*IF(S54="J",1,IF(S54="N",0,0.5)))/19,0)))</f>
+        <f>IF(A54="","",IF(OR(C54="Etagenwohnung",I54="N",J54="N"),0,ROUND(100*(3*IF(J54="J",1,IF(J54="N",0,0.5))+3*IF(K54="J",1,IF(K54="N",0,0.5))+2*IF(L54="J",1,IF(L54="N",0,0.5))+2*IF(M54="J",1,IF(M54="N",0,0.5))+1*IF(N54="J",1,IF(N54="N",0,0.5))+1*IF(O54="J",1,IF(O54="N",0,0.5))+1*IF(P54="J",1,IF(P54="N",0,0.5))+1*IF(Q54="J",1,IF(Q54="N",0,0.5))+2*IF(R54="J",1,IF(R54="N",0,0.5))+3*IF(S54="J",1,IF(S54="N",0,0.5))+IF(T54="",0,1*IF(T54="?",0.5,MAX(0,1-T54/3.57))))/(19+IF(T54="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G54" s="10" t="n"/>
@@ -2893,6 +3535,15 @@
         <f>IF(A54="","",IF(E54="","?",IF(AND(E54&gt;=90,E54&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T54" s="11" t="n"/>
+      <c r="U54" s="9">
+        <f>IF(OR(D54="",T54="",T54="?"),"",ROUND(D54*(Legende!$B$9+Legende!$B$10+T54/100),0))</f>
+        <v/>
+      </c>
+      <c r="V54" s="9">
+        <f>IF(U54="","",D54+U54)</f>
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="8" t="n"/>
@@ -2901,7 +3552,7 @@
       <c r="D55" s="9" t="n"/>
       <c r="E55" s="10" t="n"/>
       <c r="F55" s="10">
-        <f>IF(A55="","",IF(OR(C55="Etagenwohnung",I55="N"),0,ROUND(100*(3*IF(J55="J",1,IF(J55="N",0,0.5))+3*IF(K55="J",1,IF(K55="N",0,0.5))+2*IF(L55="J",1,IF(L55="N",0,0.5))+2*IF(M55="J",1,IF(M55="N",0,0.5))+1*IF(N55="J",1,IF(N55="N",0,0.5))+1*IF(O55="J",1,IF(O55="N",0,0.5))+1*IF(P55="J",1,IF(P55="N",0,0.5))+1*IF(Q55="J",1,IF(Q55="N",0,0.5))+2*IF(R55="J",1,IF(R55="N",0,0.5))+3*IF(S55="J",1,IF(S55="N",0,0.5)))/19,0)))</f>
+        <f>IF(A55="","",IF(OR(C55="Etagenwohnung",I55="N",J55="N"),0,ROUND(100*(3*IF(J55="J",1,IF(J55="N",0,0.5))+3*IF(K55="J",1,IF(K55="N",0,0.5))+2*IF(L55="J",1,IF(L55="N",0,0.5))+2*IF(M55="J",1,IF(M55="N",0,0.5))+1*IF(N55="J",1,IF(N55="N",0,0.5))+1*IF(O55="J",1,IF(O55="N",0,0.5))+1*IF(P55="J",1,IF(P55="N",0,0.5))+1*IF(Q55="J",1,IF(Q55="N",0,0.5))+2*IF(R55="J",1,IF(R55="N",0,0.5))+3*IF(S55="J",1,IF(S55="N",0,0.5))+IF(T55="",0,1*IF(T55="?",0.5,MAX(0,1-T55/3.57))))/(19+IF(T55="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G55" s="10" t="n"/>
@@ -2923,6 +3574,15 @@
         <f>IF(A55="","",IF(E55="","?",IF(AND(E55&gt;=90,E55&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T55" s="11" t="n"/>
+      <c r="U55" s="9">
+        <f>IF(OR(D55="",T55="",T55="?"),"",ROUND(D55*(Legende!$B$9+Legende!$B$10+T55/100),0))</f>
+        <v/>
+      </c>
+      <c r="V55" s="9">
+        <f>IF(U55="","",D55+U55)</f>
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="8" t="n"/>
@@ -2931,7 +3591,7 @@
       <c r="D56" s="9" t="n"/>
       <c r="E56" s="10" t="n"/>
       <c r="F56" s="10">
-        <f>IF(A56="","",IF(OR(C56="Etagenwohnung",I56="N"),0,ROUND(100*(3*IF(J56="J",1,IF(J56="N",0,0.5))+3*IF(K56="J",1,IF(K56="N",0,0.5))+2*IF(L56="J",1,IF(L56="N",0,0.5))+2*IF(M56="J",1,IF(M56="N",0,0.5))+1*IF(N56="J",1,IF(N56="N",0,0.5))+1*IF(O56="J",1,IF(O56="N",0,0.5))+1*IF(P56="J",1,IF(P56="N",0,0.5))+1*IF(Q56="J",1,IF(Q56="N",0,0.5))+2*IF(R56="J",1,IF(R56="N",0,0.5))+3*IF(S56="J",1,IF(S56="N",0,0.5)))/19,0)))</f>
+        <f>IF(A56="","",IF(OR(C56="Etagenwohnung",I56="N",J56="N"),0,ROUND(100*(3*IF(J56="J",1,IF(J56="N",0,0.5))+3*IF(K56="J",1,IF(K56="N",0,0.5))+2*IF(L56="J",1,IF(L56="N",0,0.5))+2*IF(M56="J",1,IF(M56="N",0,0.5))+1*IF(N56="J",1,IF(N56="N",0,0.5))+1*IF(O56="J",1,IF(O56="N",0,0.5))+1*IF(P56="J",1,IF(P56="N",0,0.5))+1*IF(Q56="J",1,IF(Q56="N",0,0.5))+2*IF(R56="J",1,IF(R56="N",0,0.5))+3*IF(S56="J",1,IF(S56="N",0,0.5))+IF(T56="",0,1*IF(T56="?",0.5,MAX(0,1-T56/3.57))))/(19+IF(T56="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G56" s="10" t="n"/>
@@ -2953,6 +3613,15 @@
         <f>IF(A56="","",IF(E56="","?",IF(AND(E56&gt;=90,E56&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T56" s="11" t="n"/>
+      <c r="U56" s="9">
+        <f>IF(OR(D56="",T56="",T56="?"),"",ROUND(D56*(Legende!$B$9+Legende!$B$10+T56/100),0))</f>
+        <v/>
+      </c>
+      <c r="V56" s="9">
+        <f>IF(U56="","",D56+U56)</f>
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="8" t="n"/>
@@ -2961,7 +3630,7 @@
       <c r="D57" s="9" t="n"/>
       <c r="E57" s="10" t="n"/>
       <c r="F57" s="10">
-        <f>IF(A57="","",IF(OR(C57="Etagenwohnung",I57="N"),0,ROUND(100*(3*IF(J57="J",1,IF(J57="N",0,0.5))+3*IF(K57="J",1,IF(K57="N",0,0.5))+2*IF(L57="J",1,IF(L57="N",0,0.5))+2*IF(M57="J",1,IF(M57="N",0,0.5))+1*IF(N57="J",1,IF(N57="N",0,0.5))+1*IF(O57="J",1,IF(O57="N",0,0.5))+1*IF(P57="J",1,IF(P57="N",0,0.5))+1*IF(Q57="J",1,IF(Q57="N",0,0.5))+2*IF(R57="J",1,IF(R57="N",0,0.5))+3*IF(S57="J",1,IF(S57="N",0,0.5)))/19,0)))</f>
+        <f>IF(A57="","",IF(OR(C57="Etagenwohnung",I57="N",J57="N"),0,ROUND(100*(3*IF(J57="J",1,IF(J57="N",0,0.5))+3*IF(K57="J",1,IF(K57="N",0,0.5))+2*IF(L57="J",1,IF(L57="N",0,0.5))+2*IF(M57="J",1,IF(M57="N",0,0.5))+1*IF(N57="J",1,IF(N57="N",0,0.5))+1*IF(O57="J",1,IF(O57="N",0,0.5))+1*IF(P57="J",1,IF(P57="N",0,0.5))+1*IF(Q57="J",1,IF(Q57="N",0,0.5))+2*IF(R57="J",1,IF(R57="N",0,0.5))+3*IF(S57="J",1,IF(S57="N",0,0.5))+IF(T57="",0,1*IF(T57="?",0.5,MAX(0,1-T57/3.57))))/(19+IF(T57="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G57" s="10" t="n"/>
@@ -2983,6 +3652,15 @@
         <f>IF(A57="","",IF(E57="","?",IF(AND(E57&gt;=90,E57&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T57" s="11" t="n"/>
+      <c r="U57" s="9">
+        <f>IF(OR(D57="",T57="",T57="?"),"",ROUND(D57*(Legende!$B$9+Legende!$B$10+T57/100),0))</f>
+        <v/>
+      </c>
+      <c r="V57" s="9">
+        <f>IF(U57="","",D57+U57)</f>
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="8" t="n"/>
@@ -2991,7 +3669,7 @@
       <c r="D58" s="9" t="n"/>
       <c r="E58" s="10" t="n"/>
       <c r="F58" s="10">
-        <f>IF(A58="","",IF(OR(C58="Etagenwohnung",I58="N"),0,ROUND(100*(3*IF(J58="J",1,IF(J58="N",0,0.5))+3*IF(K58="J",1,IF(K58="N",0,0.5))+2*IF(L58="J",1,IF(L58="N",0,0.5))+2*IF(M58="J",1,IF(M58="N",0,0.5))+1*IF(N58="J",1,IF(N58="N",0,0.5))+1*IF(O58="J",1,IF(O58="N",0,0.5))+1*IF(P58="J",1,IF(P58="N",0,0.5))+1*IF(Q58="J",1,IF(Q58="N",0,0.5))+2*IF(R58="J",1,IF(R58="N",0,0.5))+3*IF(S58="J",1,IF(S58="N",0,0.5)))/19,0)))</f>
+        <f>IF(A58="","",IF(OR(C58="Etagenwohnung",I58="N",J58="N"),0,ROUND(100*(3*IF(J58="J",1,IF(J58="N",0,0.5))+3*IF(K58="J",1,IF(K58="N",0,0.5))+2*IF(L58="J",1,IF(L58="N",0,0.5))+2*IF(M58="J",1,IF(M58="N",0,0.5))+1*IF(N58="J",1,IF(N58="N",0,0.5))+1*IF(O58="J",1,IF(O58="N",0,0.5))+1*IF(P58="J",1,IF(P58="N",0,0.5))+1*IF(Q58="J",1,IF(Q58="N",0,0.5))+2*IF(R58="J",1,IF(R58="N",0,0.5))+3*IF(S58="J",1,IF(S58="N",0,0.5))+IF(T58="",0,1*IF(T58="?",0.5,MAX(0,1-T58/3.57))))/(19+IF(T58="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G58" s="10" t="n"/>
@@ -3013,6 +3691,15 @@
         <f>IF(A58="","",IF(E58="","?",IF(AND(E58&gt;=90,E58&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T58" s="11" t="n"/>
+      <c r="U58" s="9">
+        <f>IF(OR(D58="",T58="",T58="?"),"",ROUND(D58*(Legende!$B$9+Legende!$B$10+T58/100),0))</f>
+        <v/>
+      </c>
+      <c r="V58" s="9">
+        <f>IF(U58="","",D58+U58)</f>
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="8" t="n"/>
@@ -3021,7 +3708,7 @@
       <c r="D59" s="9" t="n"/>
       <c r="E59" s="10" t="n"/>
       <c r="F59" s="10">
-        <f>IF(A59="","",IF(OR(C59="Etagenwohnung",I59="N"),0,ROUND(100*(3*IF(J59="J",1,IF(J59="N",0,0.5))+3*IF(K59="J",1,IF(K59="N",0,0.5))+2*IF(L59="J",1,IF(L59="N",0,0.5))+2*IF(M59="J",1,IF(M59="N",0,0.5))+1*IF(N59="J",1,IF(N59="N",0,0.5))+1*IF(O59="J",1,IF(O59="N",0,0.5))+1*IF(P59="J",1,IF(P59="N",0,0.5))+1*IF(Q59="J",1,IF(Q59="N",0,0.5))+2*IF(R59="J",1,IF(R59="N",0,0.5))+3*IF(S59="J",1,IF(S59="N",0,0.5)))/19,0)))</f>
+        <f>IF(A59="","",IF(OR(C59="Etagenwohnung",I59="N",J59="N"),0,ROUND(100*(3*IF(J59="J",1,IF(J59="N",0,0.5))+3*IF(K59="J",1,IF(K59="N",0,0.5))+2*IF(L59="J",1,IF(L59="N",0,0.5))+2*IF(M59="J",1,IF(M59="N",0,0.5))+1*IF(N59="J",1,IF(N59="N",0,0.5))+1*IF(O59="J",1,IF(O59="N",0,0.5))+1*IF(P59="J",1,IF(P59="N",0,0.5))+1*IF(Q59="J",1,IF(Q59="N",0,0.5))+2*IF(R59="J",1,IF(R59="N",0,0.5))+3*IF(S59="J",1,IF(S59="N",0,0.5))+IF(T59="",0,1*IF(T59="?",0.5,MAX(0,1-T59/3.57))))/(19+IF(T59="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G59" s="10" t="n"/>
@@ -3043,6 +3730,15 @@
         <f>IF(A59="","",IF(E59="","?",IF(AND(E59&gt;=90,E59&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T59" s="11" t="n"/>
+      <c r="U59" s="9">
+        <f>IF(OR(D59="",T59="",T59="?"),"",ROUND(D59*(Legende!$B$9+Legende!$B$10+T59/100),0))</f>
+        <v/>
+      </c>
+      <c r="V59" s="9">
+        <f>IF(U59="","",D59+U59)</f>
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="8" t="n"/>
@@ -3051,7 +3747,7 @@
       <c r="D60" s="9" t="n"/>
       <c r="E60" s="10" t="n"/>
       <c r="F60" s="10">
-        <f>IF(A60="","",IF(OR(C60="Etagenwohnung",I60="N"),0,ROUND(100*(3*IF(J60="J",1,IF(J60="N",0,0.5))+3*IF(K60="J",1,IF(K60="N",0,0.5))+2*IF(L60="J",1,IF(L60="N",0,0.5))+2*IF(M60="J",1,IF(M60="N",0,0.5))+1*IF(N60="J",1,IF(N60="N",0,0.5))+1*IF(O60="J",1,IF(O60="N",0,0.5))+1*IF(P60="J",1,IF(P60="N",0,0.5))+1*IF(Q60="J",1,IF(Q60="N",0,0.5))+2*IF(R60="J",1,IF(R60="N",0,0.5))+3*IF(S60="J",1,IF(S60="N",0,0.5)))/19,0)))</f>
+        <f>IF(A60="","",IF(OR(C60="Etagenwohnung",I60="N",J60="N"),0,ROUND(100*(3*IF(J60="J",1,IF(J60="N",0,0.5))+3*IF(K60="J",1,IF(K60="N",0,0.5))+2*IF(L60="J",1,IF(L60="N",0,0.5))+2*IF(M60="J",1,IF(M60="N",0,0.5))+1*IF(N60="J",1,IF(N60="N",0,0.5))+1*IF(O60="J",1,IF(O60="N",0,0.5))+1*IF(P60="J",1,IF(P60="N",0,0.5))+1*IF(Q60="J",1,IF(Q60="N",0,0.5))+2*IF(R60="J",1,IF(R60="N",0,0.5))+3*IF(S60="J",1,IF(S60="N",0,0.5))+IF(T60="",0,1*IF(T60="?",0.5,MAX(0,1-T60/3.57))))/(19+IF(T60="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G60" s="10" t="n"/>
@@ -3073,6 +3769,15 @@
         <f>IF(A60="","",IF(E60="","?",IF(AND(E60&gt;=90,E60&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T60" s="11" t="n"/>
+      <c r="U60" s="9">
+        <f>IF(OR(D60="",T60="",T60="?"),"",ROUND(D60*(Legende!$B$9+Legende!$B$10+T60/100),0))</f>
+        <v/>
+      </c>
+      <c r="V60" s="9">
+        <f>IF(U60="","",D60+U60)</f>
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="8" t="n"/>
@@ -3081,7 +3786,7 @@
       <c r="D61" s="9" t="n"/>
       <c r="E61" s="10" t="n"/>
       <c r="F61" s="10">
-        <f>IF(A61="","",IF(OR(C61="Etagenwohnung",I61="N"),0,ROUND(100*(3*IF(J61="J",1,IF(J61="N",0,0.5))+3*IF(K61="J",1,IF(K61="N",0,0.5))+2*IF(L61="J",1,IF(L61="N",0,0.5))+2*IF(M61="J",1,IF(M61="N",0,0.5))+1*IF(N61="J",1,IF(N61="N",0,0.5))+1*IF(O61="J",1,IF(O61="N",0,0.5))+1*IF(P61="J",1,IF(P61="N",0,0.5))+1*IF(Q61="J",1,IF(Q61="N",0,0.5))+2*IF(R61="J",1,IF(R61="N",0,0.5))+3*IF(S61="J",1,IF(S61="N",0,0.5)))/19,0)))</f>
+        <f>IF(A61="","",IF(OR(C61="Etagenwohnung",I61="N",J61="N"),0,ROUND(100*(3*IF(J61="J",1,IF(J61="N",0,0.5))+3*IF(K61="J",1,IF(K61="N",0,0.5))+2*IF(L61="J",1,IF(L61="N",0,0.5))+2*IF(M61="J",1,IF(M61="N",0,0.5))+1*IF(N61="J",1,IF(N61="N",0,0.5))+1*IF(O61="J",1,IF(O61="N",0,0.5))+1*IF(P61="J",1,IF(P61="N",0,0.5))+1*IF(Q61="J",1,IF(Q61="N",0,0.5))+2*IF(R61="J",1,IF(R61="N",0,0.5))+3*IF(S61="J",1,IF(S61="N",0,0.5))+IF(T61="",0,1*IF(T61="?",0.5,MAX(0,1-T61/3.57))))/(19+IF(T61="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G61" s="10" t="n"/>
@@ -3103,6 +3808,15 @@
         <f>IF(A61="","",IF(E61="","?",IF(AND(E61&gt;=90,E61&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T61" s="11" t="n"/>
+      <c r="U61" s="9">
+        <f>IF(OR(D61="",T61="",T61="?"),"",ROUND(D61*(Legende!$B$9+Legende!$B$10+T61/100),0))</f>
+        <v/>
+      </c>
+      <c r="V61" s="9">
+        <f>IF(U61="","",D61+U61)</f>
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="8" t="n"/>
@@ -3111,7 +3825,7 @@
       <c r="D62" s="9" t="n"/>
       <c r="E62" s="10" t="n"/>
       <c r="F62" s="10">
-        <f>IF(A62="","",IF(OR(C62="Etagenwohnung",I62="N"),0,ROUND(100*(3*IF(J62="J",1,IF(J62="N",0,0.5))+3*IF(K62="J",1,IF(K62="N",0,0.5))+2*IF(L62="J",1,IF(L62="N",0,0.5))+2*IF(M62="J",1,IF(M62="N",0,0.5))+1*IF(N62="J",1,IF(N62="N",0,0.5))+1*IF(O62="J",1,IF(O62="N",0,0.5))+1*IF(P62="J",1,IF(P62="N",0,0.5))+1*IF(Q62="J",1,IF(Q62="N",0,0.5))+2*IF(R62="J",1,IF(R62="N",0,0.5))+3*IF(S62="J",1,IF(S62="N",0,0.5)))/19,0)))</f>
+        <f>IF(A62="","",IF(OR(C62="Etagenwohnung",I62="N",J62="N"),0,ROUND(100*(3*IF(J62="J",1,IF(J62="N",0,0.5))+3*IF(K62="J",1,IF(K62="N",0,0.5))+2*IF(L62="J",1,IF(L62="N",0,0.5))+2*IF(M62="J",1,IF(M62="N",0,0.5))+1*IF(N62="J",1,IF(N62="N",0,0.5))+1*IF(O62="J",1,IF(O62="N",0,0.5))+1*IF(P62="J",1,IF(P62="N",0,0.5))+1*IF(Q62="J",1,IF(Q62="N",0,0.5))+2*IF(R62="J",1,IF(R62="N",0,0.5))+3*IF(S62="J",1,IF(S62="N",0,0.5))+IF(T62="",0,1*IF(T62="?",0.5,MAX(0,1-T62/3.57))))/(19+IF(T62="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G62" s="10" t="n"/>
@@ -3133,6 +3847,15 @@
         <f>IF(A62="","",IF(E62="","?",IF(AND(E62&gt;=90,E62&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T62" s="11" t="n"/>
+      <c r="U62" s="9">
+        <f>IF(OR(D62="",T62="",T62="?"),"",ROUND(D62*(Legende!$B$9+Legende!$B$10+T62/100),0))</f>
+        <v/>
+      </c>
+      <c r="V62" s="9">
+        <f>IF(U62="","",D62+U62)</f>
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="8" t="n"/>
@@ -3141,7 +3864,7 @@
       <c r="D63" s="9" t="n"/>
       <c r="E63" s="10" t="n"/>
       <c r="F63" s="10">
-        <f>IF(A63="","",IF(OR(C63="Etagenwohnung",I63="N"),0,ROUND(100*(3*IF(J63="J",1,IF(J63="N",0,0.5))+3*IF(K63="J",1,IF(K63="N",0,0.5))+2*IF(L63="J",1,IF(L63="N",0,0.5))+2*IF(M63="J",1,IF(M63="N",0,0.5))+1*IF(N63="J",1,IF(N63="N",0,0.5))+1*IF(O63="J",1,IF(O63="N",0,0.5))+1*IF(P63="J",1,IF(P63="N",0,0.5))+1*IF(Q63="J",1,IF(Q63="N",0,0.5))+2*IF(R63="J",1,IF(R63="N",0,0.5))+3*IF(S63="J",1,IF(S63="N",0,0.5)))/19,0)))</f>
+        <f>IF(A63="","",IF(OR(C63="Etagenwohnung",I63="N",J63="N"),0,ROUND(100*(3*IF(J63="J",1,IF(J63="N",0,0.5))+3*IF(K63="J",1,IF(K63="N",0,0.5))+2*IF(L63="J",1,IF(L63="N",0,0.5))+2*IF(M63="J",1,IF(M63="N",0,0.5))+1*IF(N63="J",1,IF(N63="N",0,0.5))+1*IF(O63="J",1,IF(O63="N",0,0.5))+1*IF(P63="J",1,IF(P63="N",0,0.5))+1*IF(Q63="J",1,IF(Q63="N",0,0.5))+2*IF(R63="J",1,IF(R63="N",0,0.5))+3*IF(S63="J",1,IF(S63="N",0,0.5))+IF(T63="",0,1*IF(T63="?",0.5,MAX(0,1-T63/3.57))))/(19+IF(T63="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G63" s="10" t="n"/>
@@ -3163,6 +3886,15 @@
         <f>IF(A63="","",IF(E63="","?",IF(AND(E63&gt;=90,E63&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T63" s="11" t="n"/>
+      <c r="U63" s="9">
+        <f>IF(OR(D63="",T63="",T63="?"),"",ROUND(D63*(Legende!$B$9+Legende!$B$10+T63/100),0))</f>
+        <v/>
+      </c>
+      <c r="V63" s="9">
+        <f>IF(U63="","",D63+U63)</f>
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="8" t="n"/>
@@ -3171,7 +3903,7 @@
       <c r="D64" s="9" t="n"/>
       <c r="E64" s="10" t="n"/>
       <c r="F64" s="10">
-        <f>IF(A64="","",IF(OR(C64="Etagenwohnung",I64="N"),0,ROUND(100*(3*IF(J64="J",1,IF(J64="N",0,0.5))+3*IF(K64="J",1,IF(K64="N",0,0.5))+2*IF(L64="J",1,IF(L64="N",0,0.5))+2*IF(M64="J",1,IF(M64="N",0,0.5))+1*IF(N64="J",1,IF(N64="N",0,0.5))+1*IF(O64="J",1,IF(O64="N",0,0.5))+1*IF(P64="J",1,IF(P64="N",0,0.5))+1*IF(Q64="J",1,IF(Q64="N",0,0.5))+2*IF(R64="J",1,IF(R64="N",0,0.5))+3*IF(S64="J",1,IF(S64="N",0,0.5)))/19,0)))</f>
+        <f>IF(A64="","",IF(OR(C64="Etagenwohnung",I64="N",J64="N"),0,ROUND(100*(3*IF(J64="J",1,IF(J64="N",0,0.5))+3*IF(K64="J",1,IF(K64="N",0,0.5))+2*IF(L64="J",1,IF(L64="N",0,0.5))+2*IF(M64="J",1,IF(M64="N",0,0.5))+1*IF(N64="J",1,IF(N64="N",0,0.5))+1*IF(O64="J",1,IF(O64="N",0,0.5))+1*IF(P64="J",1,IF(P64="N",0,0.5))+1*IF(Q64="J",1,IF(Q64="N",0,0.5))+2*IF(R64="J",1,IF(R64="N",0,0.5))+3*IF(S64="J",1,IF(S64="N",0,0.5))+IF(T64="",0,1*IF(T64="?",0.5,MAX(0,1-T64/3.57))))/(19+IF(T64="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G64" s="10" t="n"/>
@@ -3193,6 +3925,15 @@
         <f>IF(A64="","",IF(E64="","?",IF(AND(E64&gt;=90,E64&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T64" s="11" t="n"/>
+      <c r="U64" s="9">
+        <f>IF(OR(D64="",T64="",T64="?"),"",ROUND(D64*(Legende!$B$9+Legende!$B$10+T64/100),0))</f>
+        <v/>
+      </c>
+      <c r="V64" s="9">
+        <f>IF(U64="","",D64+U64)</f>
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="8" t="n"/>
@@ -3201,7 +3942,7 @@
       <c r="D65" s="9" t="n"/>
       <c r="E65" s="10" t="n"/>
       <c r="F65" s="10">
-        <f>IF(A65="","",IF(OR(C65="Etagenwohnung",I65="N"),0,ROUND(100*(3*IF(J65="J",1,IF(J65="N",0,0.5))+3*IF(K65="J",1,IF(K65="N",0,0.5))+2*IF(L65="J",1,IF(L65="N",0,0.5))+2*IF(M65="J",1,IF(M65="N",0,0.5))+1*IF(N65="J",1,IF(N65="N",0,0.5))+1*IF(O65="J",1,IF(O65="N",0,0.5))+1*IF(P65="J",1,IF(P65="N",0,0.5))+1*IF(Q65="J",1,IF(Q65="N",0,0.5))+2*IF(R65="J",1,IF(R65="N",0,0.5))+3*IF(S65="J",1,IF(S65="N",0,0.5)))/19,0)))</f>
+        <f>IF(A65="","",IF(OR(C65="Etagenwohnung",I65="N",J65="N"),0,ROUND(100*(3*IF(J65="J",1,IF(J65="N",0,0.5))+3*IF(K65="J",1,IF(K65="N",0,0.5))+2*IF(L65="J",1,IF(L65="N",0,0.5))+2*IF(M65="J",1,IF(M65="N",0,0.5))+1*IF(N65="J",1,IF(N65="N",0,0.5))+1*IF(O65="J",1,IF(O65="N",0,0.5))+1*IF(P65="J",1,IF(P65="N",0,0.5))+1*IF(Q65="J",1,IF(Q65="N",0,0.5))+2*IF(R65="J",1,IF(R65="N",0,0.5))+3*IF(S65="J",1,IF(S65="N",0,0.5))+IF(T65="",0,1*IF(T65="?",0.5,MAX(0,1-T65/3.57))))/(19+IF(T65="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G65" s="10" t="n"/>
@@ -3223,6 +3964,15 @@
         <f>IF(A65="","",IF(E65="","?",IF(AND(E65&gt;=90,E65&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T65" s="11" t="n"/>
+      <c r="U65" s="9">
+        <f>IF(OR(D65="",T65="",T65="?"),"",ROUND(D65*(Legende!$B$9+Legende!$B$10+T65/100),0))</f>
+        <v/>
+      </c>
+      <c r="V65" s="9">
+        <f>IF(U65="","",D65+U65)</f>
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="8" t="n"/>
@@ -3231,7 +3981,7 @@
       <c r="D66" s="9" t="n"/>
       <c r="E66" s="10" t="n"/>
       <c r="F66" s="10">
-        <f>IF(A66="","",IF(OR(C66="Etagenwohnung",I66="N"),0,ROUND(100*(3*IF(J66="J",1,IF(J66="N",0,0.5))+3*IF(K66="J",1,IF(K66="N",0,0.5))+2*IF(L66="J",1,IF(L66="N",0,0.5))+2*IF(M66="J",1,IF(M66="N",0,0.5))+1*IF(N66="J",1,IF(N66="N",0,0.5))+1*IF(O66="J",1,IF(O66="N",0,0.5))+1*IF(P66="J",1,IF(P66="N",0,0.5))+1*IF(Q66="J",1,IF(Q66="N",0,0.5))+2*IF(R66="J",1,IF(R66="N",0,0.5))+3*IF(S66="J",1,IF(S66="N",0,0.5)))/19,0)))</f>
+        <f>IF(A66="","",IF(OR(C66="Etagenwohnung",I66="N",J66="N"),0,ROUND(100*(3*IF(J66="J",1,IF(J66="N",0,0.5))+3*IF(K66="J",1,IF(K66="N",0,0.5))+2*IF(L66="J",1,IF(L66="N",0,0.5))+2*IF(M66="J",1,IF(M66="N",0,0.5))+1*IF(N66="J",1,IF(N66="N",0,0.5))+1*IF(O66="J",1,IF(O66="N",0,0.5))+1*IF(P66="J",1,IF(P66="N",0,0.5))+1*IF(Q66="J",1,IF(Q66="N",0,0.5))+2*IF(R66="J",1,IF(R66="N",0,0.5))+3*IF(S66="J",1,IF(S66="N",0,0.5))+IF(T66="",0,1*IF(T66="?",0.5,MAX(0,1-T66/3.57))))/(19+IF(T66="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G66" s="10" t="n"/>
@@ -3253,6 +4003,15 @@
         <f>IF(A66="","",IF(E66="","?",IF(AND(E66&gt;=90,E66&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T66" s="11" t="n"/>
+      <c r="U66" s="9">
+        <f>IF(OR(D66="",T66="",T66="?"),"",ROUND(D66*(Legende!$B$9+Legende!$B$10+T66/100),0))</f>
+        <v/>
+      </c>
+      <c r="V66" s="9">
+        <f>IF(U66="","",D66+U66)</f>
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="8" t="n"/>
@@ -3261,7 +4020,7 @@
       <c r="D67" s="9" t="n"/>
       <c r="E67" s="10" t="n"/>
       <c r="F67" s="10">
-        <f>IF(A67="","",IF(OR(C67="Etagenwohnung",I67="N"),0,ROUND(100*(3*IF(J67="J",1,IF(J67="N",0,0.5))+3*IF(K67="J",1,IF(K67="N",0,0.5))+2*IF(L67="J",1,IF(L67="N",0,0.5))+2*IF(M67="J",1,IF(M67="N",0,0.5))+1*IF(N67="J",1,IF(N67="N",0,0.5))+1*IF(O67="J",1,IF(O67="N",0,0.5))+1*IF(P67="J",1,IF(P67="N",0,0.5))+1*IF(Q67="J",1,IF(Q67="N",0,0.5))+2*IF(R67="J",1,IF(R67="N",0,0.5))+3*IF(S67="J",1,IF(S67="N",0,0.5)))/19,0)))</f>
+        <f>IF(A67="","",IF(OR(C67="Etagenwohnung",I67="N",J67="N"),0,ROUND(100*(3*IF(J67="J",1,IF(J67="N",0,0.5))+3*IF(K67="J",1,IF(K67="N",0,0.5))+2*IF(L67="J",1,IF(L67="N",0,0.5))+2*IF(M67="J",1,IF(M67="N",0,0.5))+1*IF(N67="J",1,IF(N67="N",0,0.5))+1*IF(O67="J",1,IF(O67="N",0,0.5))+1*IF(P67="J",1,IF(P67="N",0,0.5))+1*IF(Q67="J",1,IF(Q67="N",0,0.5))+2*IF(R67="J",1,IF(R67="N",0,0.5))+3*IF(S67="J",1,IF(S67="N",0,0.5))+IF(T67="",0,1*IF(T67="?",0.5,MAX(0,1-T67/3.57))))/(19+IF(T67="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G67" s="10" t="n"/>
@@ -3283,6 +4042,15 @@
         <f>IF(A67="","",IF(E67="","?",IF(AND(E67&gt;=90,E67&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T67" s="11" t="n"/>
+      <c r="U67" s="9">
+        <f>IF(OR(D67="",T67="",T67="?"),"",ROUND(D67*(Legende!$B$9+Legende!$B$10+T67/100),0))</f>
+        <v/>
+      </c>
+      <c r="V67" s="9">
+        <f>IF(U67="","",D67+U67)</f>
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="8" t="n"/>
@@ -3291,7 +4059,7 @@
       <c r="D68" s="9" t="n"/>
       <c r="E68" s="10" t="n"/>
       <c r="F68" s="10">
-        <f>IF(A68="","",IF(OR(C68="Etagenwohnung",I68="N"),0,ROUND(100*(3*IF(J68="J",1,IF(J68="N",0,0.5))+3*IF(K68="J",1,IF(K68="N",0,0.5))+2*IF(L68="J",1,IF(L68="N",0,0.5))+2*IF(M68="J",1,IF(M68="N",0,0.5))+1*IF(N68="J",1,IF(N68="N",0,0.5))+1*IF(O68="J",1,IF(O68="N",0,0.5))+1*IF(P68="J",1,IF(P68="N",0,0.5))+1*IF(Q68="J",1,IF(Q68="N",0,0.5))+2*IF(R68="J",1,IF(R68="N",0,0.5))+3*IF(S68="J",1,IF(S68="N",0,0.5)))/19,0)))</f>
+        <f>IF(A68="","",IF(OR(C68="Etagenwohnung",I68="N",J68="N"),0,ROUND(100*(3*IF(J68="J",1,IF(J68="N",0,0.5))+3*IF(K68="J",1,IF(K68="N",0,0.5))+2*IF(L68="J",1,IF(L68="N",0,0.5))+2*IF(M68="J",1,IF(M68="N",0,0.5))+1*IF(N68="J",1,IF(N68="N",0,0.5))+1*IF(O68="J",1,IF(O68="N",0,0.5))+1*IF(P68="J",1,IF(P68="N",0,0.5))+1*IF(Q68="J",1,IF(Q68="N",0,0.5))+2*IF(R68="J",1,IF(R68="N",0,0.5))+3*IF(S68="J",1,IF(S68="N",0,0.5))+IF(T68="",0,1*IF(T68="?",0.5,MAX(0,1-T68/3.57))))/(19+IF(T68="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G68" s="10" t="n"/>
@@ -3313,6 +4081,15 @@
         <f>IF(A68="","",IF(E68="","?",IF(AND(E68&gt;=90,E68&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T68" s="11" t="n"/>
+      <c r="U68" s="9">
+        <f>IF(OR(D68="",T68="",T68="?"),"",ROUND(D68*(Legende!$B$9+Legende!$B$10+T68/100),0))</f>
+        <v/>
+      </c>
+      <c r="V68" s="9">
+        <f>IF(U68="","",D68+U68)</f>
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="8" t="n"/>
@@ -3321,7 +4098,7 @@
       <c r="D69" s="9" t="n"/>
       <c r="E69" s="10" t="n"/>
       <c r="F69" s="10">
-        <f>IF(A69="","",IF(OR(C69="Etagenwohnung",I69="N"),0,ROUND(100*(3*IF(J69="J",1,IF(J69="N",0,0.5))+3*IF(K69="J",1,IF(K69="N",0,0.5))+2*IF(L69="J",1,IF(L69="N",0,0.5))+2*IF(M69="J",1,IF(M69="N",0,0.5))+1*IF(N69="J",1,IF(N69="N",0,0.5))+1*IF(O69="J",1,IF(O69="N",0,0.5))+1*IF(P69="J",1,IF(P69="N",0,0.5))+1*IF(Q69="J",1,IF(Q69="N",0,0.5))+2*IF(R69="J",1,IF(R69="N",0,0.5))+3*IF(S69="J",1,IF(S69="N",0,0.5)))/19,0)))</f>
+        <f>IF(A69="","",IF(OR(C69="Etagenwohnung",I69="N",J69="N"),0,ROUND(100*(3*IF(J69="J",1,IF(J69="N",0,0.5))+3*IF(K69="J",1,IF(K69="N",0,0.5))+2*IF(L69="J",1,IF(L69="N",0,0.5))+2*IF(M69="J",1,IF(M69="N",0,0.5))+1*IF(N69="J",1,IF(N69="N",0,0.5))+1*IF(O69="J",1,IF(O69="N",0,0.5))+1*IF(P69="J",1,IF(P69="N",0,0.5))+1*IF(Q69="J",1,IF(Q69="N",0,0.5))+2*IF(R69="J",1,IF(R69="N",0,0.5))+3*IF(S69="J",1,IF(S69="N",0,0.5))+IF(T69="",0,1*IF(T69="?",0.5,MAX(0,1-T69/3.57))))/(19+IF(T69="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G69" s="10" t="n"/>
@@ -3343,6 +4120,15 @@
         <f>IF(A69="","",IF(E69="","?",IF(AND(E69&gt;=90,E69&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T69" s="11" t="n"/>
+      <c r="U69" s="9">
+        <f>IF(OR(D69="",T69="",T69="?"),"",ROUND(D69*(Legende!$B$9+Legende!$B$10+T69/100),0))</f>
+        <v/>
+      </c>
+      <c r="V69" s="9">
+        <f>IF(U69="","",D69+U69)</f>
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="8" t="n"/>
@@ -3351,7 +4137,7 @@
       <c r="D70" s="9" t="n"/>
       <c r="E70" s="10" t="n"/>
       <c r="F70" s="10">
-        <f>IF(A70="","",IF(OR(C70="Etagenwohnung",I70="N"),0,ROUND(100*(3*IF(J70="J",1,IF(J70="N",0,0.5))+3*IF(K70="J",1,IF(K70="N",0,0.5))+2*IF(L70="J",1,IF(L70="N",0,0.5))+2*IF(M70="J",1,IF(M70="N",0,0.5))+1*IF(N70="J",1,IF(N70="N",0,0.5))+1*IF(O70="J",1,IF(O70="N",0,0.5))+1*IF(P70="J",1,IF(P70="N",0,0.5))+1*IF(Q70="J",1,IF(Q70="N",0,0.5))+2*IF(R70="J",1,IF(R70="N",0,0.5))+3*IF(S70="J",1,IF(S70="N",0,0.5)))/19,0)))</f>
+        <f>IF(A70="","",IF(OR(C70="Etagenwohnung",I70="N",J70="N"),0,ROUND(100*(3*IF(J70="J",1,IF(J70="N",0,0.5))+3*IF(K70="J",1,IF(K70="N",0,0.5))+2*IF(L70="J",1,IF(L70="N",0,0.5))+2*IF(M70="J",1,IF(M70="N",0,0.5))+1*IF(N70="J",1,IF(N70="N",0,0.5))+1*IF(O70="J",1,IF(O70="N",0,0.5))+1*IF(P70="J",1,IF(P70="N",0,0.5))+1*IF(Q70="J",1,IF(Q70="N",0,0.5))+2*IF(R70="J",1,IF(R70="N",0,0.5))+3*IF(S70="J",1,IF(S70="N",0,0.5))+IF(T70="",0,1*IF(T70="?",0.5,MAX(0,1-T70/3.57))))/(19+IF(T70="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G70" s="10" t="n"/>
@@ -3373,6 +4159,15 @@
         <f>IF(A70="","",IF(E70="","?",IF(AND(E70&gt;=90,E70&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T70" s="11" t="n"/>
+      <c r="U70" s="9">
+        <f>IF(OR(D70="",T70="",T70="?"),"",ROUND(D70*(Legende!$B$9+Legende!$B$10+T70/100),0))</f>
+        <v/>
+      </c>
+      <c r="V70" s="9">
+        <f>IF(U70="","",D70+U70)</f>
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="8" t="n"/>
@@ -3381,7 +4176,7 @@
       <c r="D71" s="9" t="n"/>
       <c r="E71" s="10" t="n"/>
       <c r="F71" s="10">
-        <f>IF(A71="","",IF(OR(C71="Etagenwohnung",I71="N"),0,ROUND(100*(3*IF(J71="J",1,IF(J71="N",0,0.5))+3*IF(K71="J",1,IF(K71="N",0,0.5))+2*IF(L71="J",1,IF(L71="N",0,0.5))+2*IF(M71="J",1,IF(M71="N",0,0.5))+1*IF(N71="J",1,IF(N71="N",0,0.5))+1*IF(O71="J",1,IF(O71="N",0,0.5))+1*IF(P71="J",1,IF(P71="N",0,0.5))+1*IF(Q71="J",1,IF(Q71="N",0,0.5))+2*IF(R71="J",1,IF(R71="N",0,0.5))+3*IF(S71="J",1,IF(S71="N",0,0.5)))/19,0)))</f>
+        <f>IF(A71="","",IF(OR(C71="Etagenwohnung",I71="N",J71="N"),0,ROUND(100*(3*IF(J71="J",1,IF(J71="N",0,0.5))+3*IF(K71="J",1,IF(K71="N",0,0.5))+2*IF(L71="J",1,IF(L71="N",0,0.5))+2*IF(M71="J",1,IF(M71="N",0,0.5))+1*IF(N71="J",1,IF(N71="N",0,0.5))+1*IF(O71="J",1,IF(O71="N",0,0.5))+1*IF(P71="J",1,IF(P71="N",0,0.5))+1*IF(Q71="J",1,IF(Q71="N",0,0.5))+2*IF(R71="J",1,IF(R71="N",0,0.5))+3*IF(S71="J",1,IF(S71="N",0,0.5))+IF(T71="",0,1*IF(T71="?",0.5,MAX(0,1-T71/3.57))))/(19+IF(T71="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G71" s="10" t="n"/>
@@ -3403,6 +4198,15 @@
         <f>IF(A71="","",IF(E71="","?",IF(AND(E71&gt;=90,E71&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T71" s="11" t="n"/>
+      <c r="U71" s="9">
+        <f>IF(OR(D71="",T71="",T71="?"),"",ROUND(D71*(Legende!$B$9+Legende!$B$10+T71/100),0))</f>
+        <v/>
+      </c>
+      <c r="V71" s="9">
+        <f>IF(U71="","",D71+U71)</f>
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="8" t="n"/>
@@ -3411,7 +4215,7 @@
       <c r="D72" s="9" t="n"/>
       <c r="E72" s="10" t="n"/>
       <c r="F72" s="10">
-        <f>IF(A72="","",IF(OR(C72="Etagenwohnung",I72="N"),0,ROUND(100*(3*IF(J72="J",1,IF(J72="N",0,0.5))+3*IF(K72="J",1,IF(K72="N",0,0.5))+2*IF(L72="J",1,IF(L72="N",0,0.5))+2*IF(M72="J",1,IF(M72="N",0,0.5))+1*IF(N72="J",1,IF(N72="N",0,0.5))+1*IF(O72="J",1,IF(O72="N",0,0.5))+1*IF(P72="J",1,IF(P72="N",0,0.5))+1*IF(Q72="J",1,IF(Q72="N",0,0.5))+2*IF(R72="J",1,IF(R72="N",0,0.5))+3*IF(S72="J",1,IF(S72="N",0,0.5)))/19,0)))</f>
+        <f>IF(A72="","",IF(OR(C72="Etagenwohnung",I72="N",J72="N"),0,ROUND(100*(3*IF(J72="J",1,IF(J72="N",0,0.5))+3*IF(K72="J",1,IF(K72="N",0,0.5))+2*IF(L72="J",1,IF(L72="N",0,0.5))+2*IF(M72="J",1,IF(M72="N",0,0.5))+1*IF(N72="J",1,IF(N72="N",0,0.5))+1*IF(O72="J",1,IF(O72="N",0,0.5))+1*IF(P72="J",1,IF(P72="N",0,0.5))+1*IF(Q72="J",1,IF(Q72="N",0,0.5))+2*IF(R72="J",1,IF(R72="N",0,0.5))+3*IF(S72="J",1,IF(S72="N",0,0.5))+IF(T72="",0,1*IF(T72="?",0.5,MAX(0,1-T72/3.57))))/(19+IF(T72="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G72" s="10" t="n"/>
@@ -3433,6 +4237,15 @@
         <f>IF(A72="","",IF(E72="","?",IF(AND(E72&gt;=90,E72&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T72" s="11" t="n"/>
+      <c r="U72" s="9">
+        <f>IF(OR(D72="",T72="",T72="?"),"",ROUND(D72*(Legende!$B$9+Legende!$B$10+T72/100),0))</f>
+        <v/>
+      </c>
+      <c r="V72" s="9">
+        <f>IF(U72="","",D72+U72)</f>
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="8" t="n"/>
@@ -3441,7 +4254,7 @@
       <c r="D73" s="9" t="n"/>
       <c r="E73" s="10" t="n"/>
       <c r="F73" s="10">
-        <f>IF(A73="","",IF(OR(C73="Etagenwohnung",I73="N"),0,ROUND(100*(3*IF(J73="J",1,IF(J73="N",0,0.5))+3*IF(K73="J",1,IF(K73="N",0,0.5))+2*IF(L73="J",1,IF(L73="N",0,0.5))+2*IF(M73="J",1,IF(M73="N",0,0.5))+1*IF(N73="J",1,IF(N73="N",0,0.5))+1*IF(O73="J",1,IF(O73="N",0,0.5))+1*IF(P73="J",1,IF(P73="N",0,0.5))+1*IF(Q73="J",1,IF(Q73="N",0,0.5))+2*IF(R73="J",1,IF(R73="N",0,0.5))+3*IF(S73="J",1,IF(S73="N",0,0.5)))/19,0)))</f>
+        <f>IF(A73="","",IF(OR(C73="Etagenwohnung",I73="N",J73="N"),0,ROUND(100*(3*IF(J73="J",1,IF(J73="N",0,0.5))+3*IF(K73="J",1,IF(K73="N",0,0.5))+2*IF(L73="J",1,IF(L73="N",0,0.5))+2*IF(M73="J",1,IF(M73="N",0,0.5))+1*IF(N73="J",1,IF(N73="N",0,0.5))+1*IF(O73="J",1,IF(O73="N",0,0.5))+1*IF(P73="J",1,IF(P73="N",0,0.5))+1*IF(Q73="J",1,IF(Q73="N",0,0.5))+2*IF(R73="J",1,IF(R73="N",0,0.5))+3*IF(S73="J",1,IF(S73="N",0,0.5))+IF(T73="",0,1*IF(T73="?",0.5,MAX(0,1-T73/3.57))))/(19+IF(T73="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G73" s="10" t="n"/>
@@ -3463,6 +4276,15 @@
         <f>IF(A73="","",IF(E73="","?",IF(AND(E73&gt;=90,E73&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T73" s="11" t="n"/>
+      <c r="U73" s="9">
+        <f>IF(OR(D73="",T73="",T73="?"),"",ROUND(D73*(Legende!$B$9+Legende!$B$10+T73/100),0))</f>
+        <v/>
+      </c>
+      <c r="V73" s="9">
+        <f>IF(U73="","",D73+U73)</f>
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="8" t="n"/>
@@ -3471,7 +4293,7 @@
       <c r="D74" s="9" t="n"/>
       <c r="E74" s="10" t="n"/>
       <c r="F74" s="10">
-        <f>IF(A74="","",IF(OR(C74="Etagenwohnung",I74="N"),0,ROUND(100*(3*IF(J74="J",1,IF(J74="N",0,0.5))+3*IF(K74="J",1,IF(K74="N",0,0.5))+2*IF(L74="J",1,IF(L74="N",0,0.5))+2*IF(M74="J",1,IF(M74="N",0,0.5))+1*IF(N74="J",1,IF(N74="N",0,0.5))+1*IF(O74="J",1,IF(O74="N",0,0.5))+1*IF(P74="J",1,IF(P74="N",0,0.5))+1*IF(Q74="J",1,IF(Q74="N",0,0.5))+2*IF(R74="J",1,IF(R74="N",0,0.5))+3*IF(S74="J",1,IF(S74="N",0,0.5)))/19,0)))</f>
+        <f>IF(A74="","",IF(OR(C74="Etagenwohnung",I74="N",J74="N"),0,ROUND(100*(3*IF(J74="J",1,IF(J74="N",0,0.5))+3*IF(K74="J",1,IF(K74="N",0,0.5))+2*IF(L74="J",1,IF(L74="N",0,0.5))+2*IF(M74="J",1,IF(M74="N",0,0.5))+1*IF(N74="J",1,IF(N74="N",0,0.5))+1*IF(O74="J",1,IF(O74="N",0,0.5))+1*IF(P74="J",1,IF(P74="N",0,0.5))+1*IF(Q74="J",1,IF(Q74="N",0,0.5))+2*IF(R74="J",1,IF(R74="N",0,0.5))+3*IF(S74="J",1,IF(S74="N",0,0.5))+IF(T74="",0,1*IF(T74="?",0.5,MAX(0,1-T74/3.57))))/(19+IF(T74="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G74" s="10" t="n"/>
@@ -3493,6 +4315,15 @@
         <f>IF(A74="","",IF(E74="","?",IF(AND(E74&gt;=90,E74&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T74" s="11" t="n"/>
+      <c r="U74" s="9">
+        <f>IF(OR(D74="",T74="",T74="?"),"",ROUND(D74*(Legende!$B$9+Legende!$B$10+T74/100),0))</f>
+        <v/>
+      </c>
+      <c r="V74" s="9">
+        <f>IF(U74="","",D74+U74)</f>
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="8" t="n"/>
@@ -3501,7 +4332,7 @@
       <c r="D75" s="9" t="n"/>
       <c r="E75" s="10" t="n"/>
       <c r="F75" s="10">
-        <f>IF(A75="","",IF(OR(C75="Etagenwohnung",I75="N"),0,ROUND(100*(3*IF(J75="J",1,IF(J75="N",0,0.5))+3*IF(K75="J",1,IF(K75="N",0,0.5))+2*IF(L75="J",1,IF(L75="N",0,0.5))+2*IF(M75="J",1,IF(M75="N",0,0.5))+1*IF(N75="J",1,IF(N75="N",0,0.5))+1*IF(O75="J",1,IF(O75="N",0,0.5))+1*IF(P75="J",1,IF(P75="N",0,0.5))+1*IF(Q75="J",1,IF(Q75="N",0,0.5))+2*IF(R75="J",1,IF(R75="N",0,0.5))+3*IF(S75="J",1,IF(S75="N",0,0.5)))/19,0)))</f>
+        <f>IF(A75="","",IF(OR(C75="Etagenwohnung",I75="N",J75="N"),0,ROUND(100*(3*IF(J75="J",1,IF(J75="N",0,0.5))+3*IF(K75="J",1,IF(K75="N",0,0.5))+2*IF(L75="J",1,IF(L75="N",0,0.5))+2*IF(M75="J",1,IF(M75="N",0,0.5))+1*IF(N75="J",1,IF(N75="N",0,0.5))+1*IF(O75="J",1,IF(O75="N",0,0.5))+1*IF(P75="J",1,IF(P75="N",0,0.5))+1*IF(Q75="J",1,IF(Q75="N",0,0.5))+2*IF(R75="J",1,IF(R75="N",0,0.5))+3*IF(S75="J",1,IF(S75="N",0,0.5))+IF(T75="",0,1*IF(T75="?",0.5,MAX(0,1-T75/3.57))))/(19+IF(T75="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G75" s="10" t="n"/>
@@ -3523,6 +4354,15 @@
         <f>IF(A75="","",IF(E75="","?",IF(AND(E75&gt;=90,E75&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T75" s="11" t="n"/>
+      <c r="U75" s="9">
+        <f>IF(OR(D75="",T75="",T75="?"),"",ROUND(D75*(Legende!$B$9+Legende!$B$10+T75/100),0))</f>
+        <v/>
+      </c>
+      <c r="V75" s="9">
+        <f>IF(U75="","",D75+U75)</f>
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="8" t="n"/>
@@ -3531,7 +4371,7 @@
       <c r="D76" s="9" t="n"/>
       <c r="E76" s="10" t="n"/>
       <c r="F76" s="10">
-        <f>IF(A76="","",IF(OR(C76="Etagenwohnung",I76="N"),0,ROUND(100*(3*IF(J76="J",1,IF(J76="N",0,0.5))+3*IF(K76="J",1,IF(K76="N",0,0.5))+2*IF(L76="J",1,IF(L76="N",0,0.5))+2*IF(M76="J",1,IF(M76="N",0,0.5))+1*IF(N76="J",1,IF(N76="N",0,0.5))+1*IF(O76="J",1,IF(O76="N",0,0.5))+1*IF(P76="J",1,IF(P76="N",0,0.5))+1*IF(Q76="J",1,IF(Q76="N",0,0.5))+2*IF(R76="J",1,IF(R76="N",0,0.5))+3*IF(S76="J",1,IF(S76="N",0,0.5)))/19,0)))</f>
+        <f>IF(A76="","",IF(OR(C76="Etagenwohnung",I76="N",J76="N"),0,ROUND(100*(3*IF(J76="J",1,IF(J76="N",0,0.5))+3*IF(K76="J",1,IF(K76="N",0,0.5))+2*IF(L76="J",1,IF(L76="N",0,0.5))+2*IF(M76="J",1,IF(M76="N",0,0.5))+1*IF(N76="J",1,IF(N76="N",0,0.5))+1*IF(O76="J",1,IF(O76="N",0,0.5))+1*IF(P76="J",1,IF(P76="N",0,0.5))+1*IF(Q76="J",1,IF(Q76="N",0,0.5))+2*IF(R76="J",1,IF(R76="N",0,0.5))+3*IF(S76="J",1,IF(S76="N",0,0.5))+IF(T76="",0,1*IF(T76="?",0.5,MAX(0,1-T76/3.57))))/(19+IF(T76="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G76" s="10" t="n"/>
@@ -3553,6 +4393,15 @@
         <f>IF(A76="","",IF(E76="","?",IF(AND(E76&gt;=90,E76&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T76" s="11" t="n"/>
+      <c r="U76" s="9">
+        <f>IF(OR(D76="",T76="",T76="?"),"",ROUND(D76*(Legende!$B$9+Legende!$B$10+T76/100),0))</f>
+        <v/>
+      </c>
+      <c r="V76" s="9">
+        <f>IF(U76="","",D76+U76)</f>
+        <v/>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="8" t="n"/>
@@ -3561,7 +4410,7 @@
       <c r="D77" s="9" t="n"/>
       <c r="E77" s="10" t="n"/>
       <c r="F77" s="10">
-        <f>IF(A77="","",IF(OR(C77="Etagenwohnung",I77="N"),0,ROUND(100*(3*IF(J77="J",1,IF(J77="N",0,0.5))+3*IF(K77="J",1,IF(K77="N",0,0.5))+2*IF(L77="J",1,IF(L77="N",0,0.5))+2*IF(M77="J",1,IF(M77="N",0,0.5))+1*IF(N77="J",1,IF(N77="N",0,0.5))+1*IF(O77="J",1,IF(O77="N",0,0.5))+1*IF(P77="J",1,IF(P77="N",0,0.5))+1*IF(Q77="J",1,IF(Q77="N",0,0.5))+2*IF(R77="J",1,IF(R77="N",0,0.5))+3*IF(S77="J",1,IF(S77="N",0,0.5)))/19,0)))</f>
+        <f>IF(A77="","",IF(OR(C77="Etagenwohnung",I77="N",J77="N"),0,ROUND(100*(3*IF(J77="J",1,IF(J77="N",0,0.5))+3*IF(K77="J",1,IF(K77="N",0,0.5))+2*IF(L77="J",1,IF(L77="N",0,0.5))+2*IF(M77="J",1,IF(M77="N",0,0.5))+1*IF(N77="J",1,IF(N77="N",0,0.5))+1*IF(O77="J",1,IF(O77="N",0,0.5))+1*IF(P77="J",1,IF(P77="N",0,0.5))+1*IF(Q77="J",1,IF(Q77="N",0,0.5))+2*IF(R77="J",1,IF(R77="N",0,0.5))+3*IF(S77="J",1,IF(S77="N",0,0.5))+IF(T77="",0,1*IF(T77="?",0.5,MAX(0,1-T77/3.57))))/(19+IF(T77="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G77" s="10" t="n"/>
@@ -3583,6 +4432,15 @@
         <f>IF(A77="","",IF(E77="","?",IF(AND(E77&gt;=90,E77&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T77" s="11" t="n"/>
+      <c r="U77" s="9">
+        <f>IF(OR(D77="",T77="",T77="?"),"",ROUND(D77*(Legende!$B$9+Legende!$B$10+T77/100),0))</f>
+        <v/>
+      </c>
+      <c r="V77" s="9">
+        <f>IF(U77="","",D77+U77)</f>
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="8" t="n"/>
@@ -3591,7 +4449,7 @@
       <c r="D78" s="9" t="n"/>
       <c r="E78" s="10" t="n"/>
       <c r="F78" s="10">
-        <f>IF(A78="","",IF(OR(C78="Etagenwohnung",I78="N"),0,ROUND(100*(3*IF(J78="J",1,IF(J78="N",0,0.5))+3*IF(K78="J",1,IF(K78="N",0,0.5))+2*IF(L78="J",1,IF(L78="N",0,0.5))+2*IF(M78="J",1,IF(M78="N",0,0.5))+1*IF(N78="J",1,IF(N78="N",0,0.5))+1*IF(O78="J",1,IF(O78="N",0,0.5))+1*IF(P78="J",1,IF(P78="N",0,0.5))+1*IF(Q78="J",1,IF(Q78="N",0,0.5))+2*IF(R78="J",1,IF(R78="N",0,0.5))+3*IF(S78="J",1,IF(S78="N",0,0.5)))/19,0)))</f>
+        <f>IF(A78="","",IF(OR(C78="Etagenwohnung",I78="N",J78="N"),0,ROUND(100*(3*IF(J78="J",1,IF(J78="N",0,0.5))+3*IF(K78="J",1,IF(K78="N",0,0.5))+2*IF(L78="J",1,IF(L78="N",0,0.5))+2*IF(M78="J",1,IF(M78="N",0,0.5))+1*IF(N78="J",1,IF(N78="N",0,0.5))+1*IF(O78="J",1,IF(O78="N",0,0.5))+1*IF(P78="J",1,IF(P78="N",0,0.5))+1*IF(Q78="J",1,IF(Q78="N",0,0.5))+2*IF(R78="J",1,IF(R78="N",0,0.5))+3*IF(S78="J",1,IF(S78="N",0,0.5))+IF(T78="",0,1*IF(T78="?",0.5,MAX(0,1-T78/3.57))))/(19+IF(T78="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G78" s="10" t="n"/>
@@ -3613,6 +4471,15 @@
         <f>IF(A78="","",IF(E78="","?",IF(AND(E78&gt;=90,E78&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T78" s="11" t="n"/>
+      <c r="U78" s="9">
+        <f>IF(OR(D78="",T78="",T78="?"),"",ROUND(D78*(Legende!$B$9+Legende!$B$10+T78/100),0))</f>
+        <v/>
+      </c>
+      <c r="V78" s="9">
+        <f>IF(U78="","",D78+U78)</f>
+        <v/>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="8" t="n"/>
@@ -3621,7 +4488,7 @@
       <c r="D79" s="9" t="n"/>
       <c r="E79" s="10" t="n"/>
       <c r="F79" s="10">
-        <f>IF(A79="","",IF(OR(C79="Etagenwohnung",I79="N"),0,ROUND(100*(3*IF(J79="J",1,IF(J79="N",0,0.5))+3*IF(K79="J",1,IF(K79="N",0,0.5))+2*IF(L79="J",1,IF(L79="N",0,0.5))+2*IF(M79="J",1,IF(M79="N",0,0.5))+1*IF(N79="J",1,IF(N79="N",0,0.5))+1*IF(O79="J",1,IF(O79="N",0,0.5))+1*IF(P79="J",1,IF(P79="N",0,0.5))+1*IF(Q79="J",1,IF(Q79="N",0,0.5))+2*IF(R79="J",1,IF(R79="N",0,0.5))+3*IF(S79="J",1,IF(S79="N",0,0.5)))/19,0)))</f>
+        <f>IF(A79="","",IF(OR(C79="Etagenwohnung",I79="N",J79="N"),0,ROUND(100*(3*IF(J79="J",1,IF(J79="N",0,0.5))+3*IF(K79="J",1,IF(K79="N",0,0.5))+2*IF(L79="J",1,IF(L79="N",0,0.5))+2*IF(M79="J",1,IF(M79="N",0,0.5))+1*IF(N79="J",1,IF(N79="N",0,0.5))+1*IF(O79="J",1,IF(O79="N",0,0.5))+1*IF(P79="J",1,IF(P79="N",0,0.5))+1*IF(Q79="J",1,IF(Q79="N",0,0.5))+2*IF(R79="J",1,IF(R79="N",0,0.5))+3*IF(S79="J",1,IF(S79="N",0,0.5))+IF(T79="",0,1*IF(T79="?",0.5,MAX(0,1-T79/3.57))))/(19+IF(T79="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G79" s="10" t="n"/>
@@ -3643,6 +4510,15 @@
         <f>IF(A79="","",IF(E79="","?",IF(AND(E79&gt;=90,E79&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T79" s="11" t="n"/>
+      <c r="U79" s="9">
+        <f>IF(OR(D79="",T79="",T79="?"),"",ROUND(D79*(Legende!$B$9+Legende!$B$10+T79/100),0))</f>
+        <v/>
+      </c>
+      <c r="V79" s="9">
+        <f>IF(U79="","",D79+U79)</f>
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="8" t="n"/>
@@ -3651,7 +4527,7 @@
       <c r="D80" s="9" t="n"/>
       <c r="E80" s="10" t="n"/>
       <c r="F80" s="10">
-        <f>IF(A80="","",IF(OR(C80="Etagenwohnung",I80="N"),0,ROUND(100*(3*IF(J80="J",1,IF(J80="N",0,0.5))+3*IF(K80="J",1,IF(K80="N",0,0.5))+2*IF(L80="J",1,IF(L80="N",0,0.5))+2*IF(M80="J",1,IF(M80="N",0,0.5))+1*IF(N80="J",1,IF(N80="N",0,0.5))+1*IF(O80="J",1,IF(O80="N",0,0.5))+1*IF(P80="J",1,IF(P80="N",0,0.5))+1*IF(Q80="J",1,IF(Q80="N",0,0.5))+2*IF(R80="J",1,IF(R80="N",0,0.5))+3*IF(S80="J",1,IF(S80="N",0,0.5)))/19,0)))</f>
+        <f>IF(A80="","",IF(OR(C80="Etagenwohnung",I80="N",J80="N"),0,ROUND(100*(3*IF(J80="J",1,IF(J80="N",0,0.5))+3*IF(K80="J",1,IF(K80="N",0,0.5))+2*IF(L80="J",1,IF(L80="N",0,0.5))+2*IF(M80="J",1,IF(M80="N",0,0.5))+1*IF(N80="J",1,IF(N80="N",0,0.5))+1*IF(O80="J",1,IF(O80="N",0,0.5))+1*IF(P80="J",1,IF(P80="N",0,0.5))+1*IF(Q80="J",1,IF(Q80="N",0,0.5))+2*IF(R80="J",1,IF(R80="N",0,0.5))+3*IF(S80="J",1,IF(S80="N",0,0.5))+IF(T80="",0,1*IF(T80="?",0.5,MAX(0,1-T80/3.57))))/(19+IF(T80="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G80" s="10" t="n"/>
@@ -3673,6 +4549,15 @@
         <f>IF(A80="","",IF(E80="","?",IF(AND(E80&gt;=90,E80&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T80" s="11" t="n"/>
+      <c r="U80" s="9">
+        <f>IF(OR(D80="",T80="",T80="?"),"",ROUND(D80*(Legende!$B$9+Legende!$B$10+T80/100),0))</f>
+        <v/>
+      </c>
+      <c r="V80" s="9">
+        <f>IF(U80="","",D80+U80)</f>
+        <v/>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="8" t="n"/>
@@ -3681,7 +4566,7 @@
       <c r="D81" s="9" t="n"/>
       <c r="E81" s="10" t="n"/>
       <c r="F81" s="10">
-        <f>IF(A81="","",IF(OR(C81="Etagenwohnung",I81="N"),0,ROUND(100*(3*IF(J81="J",1,IF(J81="N",0,0.5))+3*IF(K81="J",1,IF(K81="N",0,0.5))+2*IF(L81="J",1,IF(L81="N",0,0.5))+2*IF(M81="J",1,IF(M81="N",0,0.5))+1*IF(N81="J",1,IF(N81="N",0,0.5))+1*IF(O81="J",1,IF(O81="N",0,0.5))+1*IF(P81="J",1,IF(P81="N",0,0.5))+1*IF(Q81="J",1,IF(Q81="N",0,0.5))+2*IF(R81="J",1,IF(R81="N",0,0.5))+3*IF(S81="J",1,IF(S81="N",0,0.5)))/19,0)))</f>
+        <f>IF(A81="","",IF(OR(C81="Etagenwohnung",I81="N",J81="N"),0,ROUND(100*(3*IF(J81="J",1,IF(J81="N",0,0.5))+3*IF(K81="J",1,IF(K81="N",0,0.5))+2*IF(L81="J",1,IF(L81="N",0,0.5))+2*IF(M81="J",1,IF(M81="N",0,0.5))+1*IF(N81="J",1,IF(N81="N",0,0.5))+1*IF(O81="J",1,IF(O81="N",0,0.5))+1*IF(P81="J",1,IF(P81="N",0,0.5))+1*IF(Q81="J",1,IF(Q81="N",0,0.5))+2*IF(R81="J",1,IF(R81="N",0,0.5))+3*IF(S81="J",1,IF(S81="N",0,0.5))+IF(T81="",0,1*IF(T81="?",0.5,MAX(0,1-T81/3.57))))/(19+IF(T81="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G81" s="10" t="n"/>
@@ -3703,6 +4588,15 @@
         <f>IF(A81="","",IF(E81="","?",IF(AND(E81&gt;=90,E81&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T81" s="11" t="n"/>
+      <c r="U81" s="9">
+        <f>IF(OR(D81="",T81="",T81="?"),"",ROUND(D81*(Legende!$B$9+Legende!$B$10+T81/100),0))</f>
+        <v/>
+      </c>
+      <c r="V81" s="9">
+        <f>IF(U81="","",D81+U81)</f>
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="8" t="n"/>
@@ -3711,7 +4605,7 @@
       <c r="D82" s="9" t="n"/>
       <c r="E82" s="10" t="n"/>
       <c r="F82" s="10">
-        <f>IF(A82="","",IF(OR(C82="Etagenwohnung",I82="N"),0,ROUND(100*(3*IF(J82="J",1,IF(J82="N",0,0.5))+3*IF(K82="J",1,IF(K82="N",0,0.5))+2*IF(L82="J",1,IF(L82="N",0,0.5))+2*IF(M82="J",1,IF(M82="N",0,0.5))+1*IF(N82="J",1,IF(N82="N",0,0.5))+1*IF(O82="J",1,IF(O82="N",0,0.5))+1*IF(P82="J",1,IF(P82="N",0,0.5))+1*IF(Q82="J",1,IF(Q82="N",0,0.5))+2*IF(R82="J",1,IF(R82="N",0,0.5))+3*IF(S82="J",1,IF(S82="N",0,0.5)))/19,0)))</f>
+        <f>IF(A82="","",IF(OR(C82="Etagenwohnung",I82="N",J82="N"),0,ROUND(100*(3*IF(J82="J",1,IF(J82="N",0,0.5))+3*IF(K82="J",1,IF(K82="N",0,0.5))+2*IF(L82="J",1,IF(L82="N",0,0.5))+2*IF(M82="J",1,IF(M82="N",0,0.5))+1*IF(N82="J",1,IF(N82="N",0,0.5))+1*IF(O82="J",1,IF(O82="N",0,0.5))+1*IF(P82="J",1,IF(P82="N",0,0.5))+1*IF(Q82="J",1,IF(Q82="N",0,0.5))+2*IF(R82="J",1,IF(R82="N",0,0.5))+3*IF(S82="J",1,IF(S82="N",0,0.5))+IF(T82="",0,1*IF(T82="?",0.5,MAX(0,1-T82/3.57))))/(19+IF(T82="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G82" s="10" t="n"/>
@@ -3733,6 +4627,15 @@
         <f>IF(A82="","",IF(E82="","?",IF(AND(E82&gt;=90,E82&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T82" s="11" t="n"/>
+      <c r="U82" s="9">
+        <f>IF(OR(D82="",T82="",T82="?"),"",ROUND(D82*(Legende!$B$9+Legende!$B$10+T82/100),0))</f>
+        <v/>
+      </c>
+      <c r="V82" s="9">
+        <f>IF(U82="","",D82+U82)</f>
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="8" t="n"/>
@@ -3741,7 +4644,7 @@
       <c r="D83" s="9" t="n"/>
       <c r="E83" s="10" t="n"/>
       <c r="F83" s="10">
-        <f>IF(A83="","",IF(OR(C83="Etagenwohnung",I83="N"),0,ROUND(100*(3*IF(J83="J",1,IF(J83="N",0,0.5))+3*IF(K83="J",1,IF(K83="N",0,0.5))+2*IF(L83="J",1,IF(L83="N",0,0.5))+2*IF(M83="J",1,IF(M83="N",0,0.5))+1*IF(N83="J",1,IF(N83="N",0,0.5))+1*IF(O83="J",1,IF(O83="N",0,0.5))+1*IF(P83="J",1,IF(P83="N",0,0.5))+1*IF(Q83="J",1,IF(Q83="N",0,0.5))+2*IF(R83="J",1,IF(R83="N",0,0.5))+3*IF(S83="J",1,IF(S83="N",0,0.5)))/19,0)))</f>
+        <f>IF(A83="","",IF(OR(C83="Etagenwohnung",I83="N",J83="N"),0,ROUND(100*(3*IF(J83="J",1,IF(J83="N",0,0.5))+3*IF(K83="J",1,IF(K83="N",0,0.5))+2*IF(L83="J",1,IF(L83="N",0,0.5))+2*IF(M83="J",1,IF(M83="N",0,0.5))+1*IF(N83="J",1,IF(N83="N",0,0.5))+1*IF(O83="J",1,IF(O83="N",0,0.5))+1*IF(P83="J",1,IF(P83="N",0,0.5))+1*IF(Q83="J",1,IF(Q83="N",0,0.5))+2*IF(R83="J",1,IF(R83="N",0,0.5))+3*IF(S83="J",1,IF(S83="N",0,0.5))+IF(T83="",0,1*IF(T83="?",0.5,MAX(0,1-T83/3.57))))/(19+IF(T83="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G83" s="10" t="n"/>
@@ -3763,6 +4666,15 @@
         <f>IF(A83="","",IF(E83="","?",IF(AND(E83&gt;=90,E83&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T83" s="11" t="n"/>
+      <c r="U83" s="9">
+        <f>IF(OR(D83="",T83="",T83="?"),"",ROUND(D83*(Legende!$B$9+Legende!$B$10+T83/100),0))</f>
+        <v/>
+      </c>
+      <c r="V83" s="9">
+        <f>IF(U83="","",D83+U83)</f>
+        <v/>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="8" t="n"/>
@@ -3771,7 +4683,7 @@
       <c r="D84" s="9" t="n"/>
       <c r="E84" s="10" t="n"/>
       <c r="F84" s="10">
-        <f>IF(A84="","",IF(OR(C84="Etagenwohnung",I84="N"),0,ROUND(100*(3*IF(J84="J",1,IF(J84="N",0,0.5))+3*IF(K84="J",1,IF(K84="N",0,0.5))+2*IF(L84="J",1,IF(L84="N",0,0.5))+2*IF(M84="J",1,IF(M84="N",0,0.5))+1*IF(N84="J",1,IF(N84="N",0,0.5))+1*IF(O84="J",1,IF(O84="N",0,0.5))+1*IF(P84="J",1,IF(P84="N",0,0.5))+1*IF(Q84="J",1,IF(Q84="N",0,0.5))+2*IF(R84="J",1,IF(R84="N",0,0.5))+3*IF(S84="J",1,IF(S84="N",0,0.5)))/19,0)))</f>
+        <f>IF(A84="","",IF(OR(C84="Etagenwohnung",I84="N",J84="N"),0,ROUND(100*(3*IF(J84="J",1,IF(J84="N",0,0.5))+3*IF(K84="J",1,IF(K84="N",0,0.5))+2*IF(L84="J",1,IF(L84="N",0,0.5))+2*IF(M84="J",1,IF(M84="N",0,0.5))+1*IF(N84="J",1,IF(N84="N",0,0.5))+1*IF(O84="J",1,IF(O84="N",0,0.5))+1*IF(P84="J",1,IF(P84="N",0,0.5))+1*IF(Q84="J",1,IF(Q84="N",0,0.5))+2*IF(R84="J",1,IF(R84="N",0,0.5))+3*IF(S84="J",1,IF(S84="N",0,0.5))+IF(T84="",0,1*IF(T84="?",0.5,MAX(0,1-T84/3.57))))/(19+IF(T84="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G84" s="10" t="n"/>
@@ -3793,6 +4705,15 @@
         <f>IF(A84="","",IF(E84="","?",IF(AND(E84&gt;=90,E84&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T84" s="11" t="n"/>
+      <c r="U84" s="9">
+        <f>IF(OR(D84="",T84="",T84="?"),"",ROUND(D84*(Legende!$B$9+Legende!$B$10+T84/100),0))</f>
+        <v/>
+      </c>
+      <c r="V84" s="9">
+        <f>IF(U84="","",D84+U84)</f>
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="8" t="n"/>
@@ -3801,7 +4722,7 @@
       <c r="D85" s="9" t="n"/>
       <c r="E85" s="10" t="n"/>
       <c r="F85" s="10">
-        <f>IF(A85="","",IF(OR(C85="Etagenwohnung",I85="N"),0,ROUND(100*(3*IF(J85="J",1,IF(J85="N",0,0.5))+3*IF(K85="J",1,IF(K85="N",0,0.5))+2*IF(L85="J",1,IF(L85="N",0,0.5))+2*IF(M85="J",1,IF(M85="N",0,0.5))+1*IF(N85="J",1,IF(N85="N",0,0.5))+1*IF(O85="J",1,IF(O85="N",0,0.5))+1*IF(P85="J",1,IF(P85="N",0,0.5))+1*IF(Q85="J",1,IF(Q85="N",0,0.5))+2*IF(R85="J",1,IF(R85="N",0,0.5))+3*IF(S85="J",1,IF(S85="N",0,0.5)))/19,0)))</f>
+        <f>IF(A85="","",IF(OR(C85="Etagenwohnung",I85="N",J85="N"),0,ROUND(100*(3*IF(J85="J",1,IF(J85="N",0,0.5))+3*IF(K85="J",1,IF(K85="N",0,0.5))+2*IF(L85="J",1,IF(L85="N",0,0.5))+2*IF(M85="J",1,IF(M85="N",0,0.5))+1*IF(N85="J",1,IF(N85="N",0,0.5))+1*IF(O85="J",1,IF(O85="N",0,0.5))+1*IF(P85="J",1,IF(P85="N",0,0.5))+1*IF(Q85="J",1,IF(Q85="N",0,0.5))+2*IF(R85="J",1,IF(R85="N",0,0.5))+3*IF(S85="J",1,IF(S85="N",0,0.5))+IF(T85="",0,1*IF(T85="?",0.5,MAX(0,1-T85/3.57))))/(19+IF(T85="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G85" s="10" t="n"/>
@@ -3823,6 +4744,15 @@
         <f>IF(A85="","",IF(E85="","?",IF(AND(E85&gt;=90,E85&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T85" s="11" t="n"/>
+      <c r="U85" s="9">
+        <f>IF(OR(D85="",T85="",T85="?"),"",ROUND(D85*(Legende!$B$9+Legende!$B$10+T85/100),0))</f>
+        <v/>
+      </c>
+      <c r="V85" s="9">
+        <f>IF(U85="","",D85+U85)</f>
+        <v/>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="8" t="n"/>
@@ -3831,7 +4761,7 @@
       <c r="D86" s="9" t="n"/>
       <c r="E86" s="10" t="n"/>
       <c r="F86" s="10">
-        <f>IF(A86="","",IF(OR(C86="Etagenwohnung",I86="N"),0,ROUND(100*(3*IF(J86="J",1,IF(J86="N",0,0.5))+3*IF(K86="J",1,IF(K86="N",0,0.5))+2*IF(L86="J",1,IF(L86="N",0,0.5))+2*IF(M86="J",1,IF(M86="N",0,0.5))+1*IF(N86="J",1,IF(N86="N",0,0.5))+1*IF(O86="J",1,IF(O86="N",0,0.5))+1*IF(P86="J",1,IF(P86="N",0,0.5))+1*IF(Q86="J",1,IF(Q86="N",0,0.5))+2*IF(R86="J",1,IF(R86="N",0,0.5))+3*IF(S86="J",1,IF(S86="N",0,0.5)))/19,0)))</f>
+        <f>IF(A86="","",IF(OR(C86="Etagenwohnung",I86="N",J86="N"),0,ROUND(100*(3*IF(J86="J",1,IF(J86="N",0,0.5))+3*IF(K86="J",1,IF(K86="N",0,0.5))+2*IF(L86="J",1,IF(L86="N",0,0.5))+2*IF(M86="J",1,IF(M86="N",0,0.5))+1*IF(N86="J",1,IF(N86="N",0,0.5))+1*IF(O86="J",1,IF(O86="N",0,0.5))+1*IF(P86="J",1,IF(P86="N",0,0.5))+1*IF(Q86="J",1,IF(Q86="N",0,0.5))+2*IF(R86="J",1,IF(R86="N",0,0.5))+3*IF(S86="J",1,IF(S86="N",0,0.5))+IF(T86="",0,1*IF(T86="?",0.5,MAX(0,1-T86/3.57))))/(19+IF(T86="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G86" s="10" t="n"/>
@@ -3853,6 +4783,15 @@
         <f>IF(A86="","",IF(E86="","?",IF(AND(E86&gt;=90,E86&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T86" s="11" t="n"/>
+      <c r="U86" s="9">
+        <f>IF(OR(D86="",T86="",T86="?"),"",ROUND(D86*(Legende!$B$9+Legende!$B$10+T86/100),0))</f>
+        <v/>
+      </c>
+      <c r="V86" s="9">
+        <f>IF(U86="","",D86+U86)</f>
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="8" t="n"/>
@@ -3861,7 +4800,7 @@
       <c r="D87" s="9" t="n"/>
       <c r="E87" s="10" t="n"/>
       <c r="F87" s="10">
-        <f>IF(A87="","",IF(OR(C87="Etagenwohnung",I87="N"),0,ROUND(100*(3*IF(J87="J",1,IF(J87="N",0,0.5))+3*IF(K87="J",1,IF(K87="N",0,0.5))+2*IF(L87="J",1,IF(L87="N",0,0.5))+2*IF(M87="J",1,IF(M87="N",0,0.5))+1*IF(N87="J",1,IF(N87="N",0,0.5))+1*IF(O87="J",1,IF(O87="N",0,0.5))+1*IF(P87="J",1,IF(P87="N",0,0.5))+1*IF(Q87="J",1,IF(Q87="N",0,0.5))+2*IF(R87="J",1,IF(R87="N",0,0.5))+3*IF(S87="J",1,IF(S87="N",0,0.5)))/19,0)))</f>
+        <f>IF(A87="","",IF(OR(C87="Etagenwohnung",I87="N",J87="N"),0,ROUND(100*(3*IF(J87="J",1,IF(J87="N",0,0.5))+3*IF(K87="J",1,IF(K87="N",0,0.5))+2*IF(L87="J",1,IF(L87="N",0,0.5))+2*IF(M87="J",1,IF(M87="N",0,0.5))+1*IF(N87="J",1,IF(N87="N",0,0.5))+1*IF(O87="J",1,IF(O87="N",0,0.5))+1*IF(P87="J",1,IF(P87="N",0,0.5))+1*IF(Q87="J",1,IF(Q87="N",0,0.5))+2*IF(R87="J",1,IF(R87="N",0,0.5))+3*IF(S87="J",1,IF(S87="N",0,0.5))+IF(T87="",0,1*IF(T87="?",0.5,MAX(0,1-T87/3.57))))/(19+IF(T87="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G87" s="10" t="n"/>
@@ -3883,6 +4822,15 @@
         <f>IF(A87="","",IF(E87="","?",IF(AND(E87&gt;=90,E87&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T87" s="11" t="n"/>
+      <c r="U87" s="9">
+        <f>IF(OR(D87="",T87="",T87="?"),"",ROUND(D87*(Legende!$B$9+Legende!$B$10+T87/100),0))</f>
+        <v/>
+      </c>
+      <c r="V87" s="9">
+        <f>IF(U87="","",D87+U87)</f>
+        <v/>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="8" t="n"/>
@@ -3891,7 +4839,7 @@
       <c r="D88" s="9" t="n"/>
       <c r="E88" s="10" t="n"/>
       <c r="F88" s="10">
-        <f>IF(A88="","",IF(OR(C88="Etagenwohnung",I88="N"),0,ROUND(100*(3*IF(J88="J",1,IF(J88="N",0,0.5))+3*IF(K88="J",1,IF(K88="N",0,0.5))+2*IF(L88="J",1,IF(L88="N",0,0.5))+2*IF(M88="J",1,IF(M88="N",0,0.5))+1*IF(N88="J",1,IF(N88="N",0,0.5))+1*IF(O88="J",1,IF(O88="N",0,0.5))+1*IF(P88="J",1,IF(P88="N",0,0.5))+1*IF(Q88="J",1,IF(Q88="N",0,0.5))+2*IF(R88="J",1,IF(R88="N",0,0.5))+3*IF(S88="J",1,IF(S88="N",0,0.5)))/19,0)))</f>
+        <f>IF(A88="","",IF(OR(C88="Etagenwohnung",I88="N",J88="N"),0,ROUND(100*(3*IF(J88="J",1,IF(J88="N",0,0.5))+3*IF(K88="J",1,IF(K88="N",0,0.5))+2*IF(L88="J",1,IF(L88="N",0,0.5))+2*IF(M88="J",1,IF(M88="N",0,0.5))+1*IF(N88="J",1,IF(N88="N",0,0.5))+1*IF(O88="J",1,IF(O88="N",0,0.5))+1*IF(P88="J",1,IF(P88="N",0,0.5))+1*IF(Q88="J",1,IF(Q88="N",0,0.5))+2*IF(R88="J",1,IF(R88="N",0,0.5))+3*IF(S88="J",1,IF(S88="N",0,0.5))+IF(T88="",0,1*IF(T88="?",0.5,MAX(0,1-T88/3.57))))/(19+IF(T88="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G88" s="10" t="n"/>
@@ -3913,6 +4861,15 @@
         <f>IF(A88="","",IF(E88="","?",IF(AND(E88&gt;=90,E88&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T88" s="11" t="n"/>
+      <c r="U88" s="9">
+        <f>IF(OR(D88="",T88="",T88="?"),"",ROUND(D88*(Legende!$B$9+Legende!$B$10+T88/100),0))</f>
+        <v/>
+      </c>
+      <c r="V88" s="9">
+        <f>IF(U88="","",D88+U88)</f>
+        <v/>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="8" t="n"/>
@@ -3921,7 +4878,7 @@
       <c r="D89" s="9" t="n"/>
       <c r="E89" s="10" t="n"/>
       <c r="F89" s="10">
-        <f>IF(A89="","",IF(OR(C89="Etagenwohnung",I89="N"),0,ROUND(100*(3*IF(J89="J",1,IF(J89="N",0,0.5))+3*IF(K89="J",1,IF(K89="N",0,0.5))+2*IF(L89="J",1,IF(L89="N",0,0.5))+2*IF(M89="J",1,IF(M89="N",0,0.5))+1*IF(N89="J",1,IF(N89="N",0,0.5))+1*IF(O89="J",1,IF(O89="N",0,0.5))+1*IF(P89="J",1,IF(P89="N",0,0.5))+1*IF(Q89="J",1,IF(Q89="N",0,0.5))+2*IF(R89="J",1,IF(R89="N",0,0.5))+3*IF(S89="J",1,IF(S89="N",0,0.5)))/19,0)))</f>
+        <f>IF(A89="","",IF(OR(C89="Etagenwohnung",I89="N",J89="N"),0,ROUND(100*(3*IF(J89="J",1,IF(J89="N",0,0.5))+3*IF(K89="J",1,IF(K89="N",0,0.5))+2*IF(L89="J",1,IF(L89="N",0,0.5))+2*IF(M89="J",1,IF(M89="N",0,0.5))+1*IF(N89="J",1,IF(N89="N",0,0.5))+1*IF(O89="J",1,IF(O89="N",0,0.5))+1*IF(P89="J",1,IF(P89="N",0,0.5))+1*IF(Q89="J",1,IF(Q89="N",0,0.5))+2*IF(R89="J",1,IF(R89="N",0,0.5))+3*IF(S89="J",1,IF(S89="N",0,0.5))+IF(T89="",0,1*IF(T89="?",0.5,MAX(0,1-T89/3.57))))/(19+IF(T89="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G89" s="10" t="n"/>
@@ -3943,6 +4900,15 @@
         <f>IF(A89="","",IF(E89="","?",IF(AND(E89&gt;=90,E89&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T89" s="11" t="n"/>
+      <c r="U89" s="9">
+        <f>IF(OR(D89="",T89="",T89="?"),"",ROUND(D89*(Legende!$B$9+Legende!$B$10+T89/100),0))</f>
+        <v/>
+      </c>
+      <c r="V89" s="9">
+        <f>IF(U89="","",D89+U89)</f>
+        <v/>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="8" t="n"/>
@@ -3951,7 +4917,7 @@
       <c r="D90" s="9" t="n"/>
       <c r="E90" s="10" t="n"/>
       <c r="F90" s="10">
-        <f>IF(A90="","",IF(OR(C90="Etagenwohnung",I90="N"),0,ROUND(100*(3*IF(J90="J",1,IF(J90="N",0,0.5))+3*IF(K90="J",1,IF(K90="N",0,0.5))+2*IF(L90="J",1,IF(L90="N",0,0.5))+2*IF(M90="J",1,IF(M90="N",0,0.5))+1*IF(N90="J",1,IF(N90="N",0,0.5))+1*IF(O90="J",1,IF(O90="N",0,0.5))+1*IF(P90="J",1,IF(P90="N",0,0.5))+1*IF(Q90="J",1,IF(Q90="N",0,0.5))+2*IF(R90="J",1,IF(R90="N",0,0.5))+3*IF(S90="J",1,IF(S90="N",0,0.5)))/19,0)))</f>
+        <f>IF(A90="","",IF(OR(C90="Etagenwohnung",I90="N",J90="N"),0,ROUND(100*(3*IF(J90="J",1,IF(J90="N",0,0.5))+3*IF(K90="J",1,IF(K90="N",0,0.5))+2*IF(L90="J",1,IF(L90="N",0,0.5))+2*IF(M90="J",1,IF(M90="N",0,0.5))+1*IF(N90="J",1,IF(N90="N",0,0.5))+1*IF(O90="J",1,IF(O90="N",0,0.5))+1*IF(P90="J",1,IF(P90="N",0,0.5))+1*IF(Q90="J",1,IF(Q90="N",0,0.5))+2*IF(R90="J",1,IF(R90="N",0,0.5))+3*IF(S90="J",1,IF(S90="N",0,0.5))+IF(T90="",0,1*IF(T90="?",0.5,MAX(0,1-T90/3.57))))/(19+IF(T90="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G90" s="10" t="n"/>
@@ -3973,6 +4939,15 @@
         <f>IF(A90="","",IF(E90="","?",IF(AND(E90&gt;=90,E90&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T90" s="11" t="n"/>
+      <c r="U90" s="9">
+        <f>IF(OR(D90="",T90="",T90="?"),"",ROUND(D90*(Legende!$B$9+Legende!$B$10+T90/100),0))</f>
+        <v/>
+      </c>
+      <c r="V90" s="9">
+        <f>IF(U90="","",D90+U90)</f>
+        <v/>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="8" t="n"/>
@@ -3981,7 +4956,7 @@
       <c r="D91" s="9" t="n"/>
       <c r="E91" s="10" t="n"/>
       <c r="F91" s="10">
-        <f>IF(A91="","",IF(OR(C91="Etagenwohnung",I91="N"),0,ROUND(100*(3*IF(J91="J",1,IF(J91="N",0,0.5))+3*IF(K91="J",1,IF(K91="N",0,0.5))+2*IF(L91="J",1,IF(L91="N",0,0.5))+2*IF(M91="J",1,IF(M91="N",0,0.5))+1*IF(N91="J",1,IF(N91="N",0,0.5))+1*IF(O91="J",1,IF(O91="N",0,0.5))+1*IF(P91="J",1,IF(P91="N",0,0.5))+1*IF(Q91="J",1,IF(Q91="N",0,0.5))+2*IF(R91="J",1,IF(R91="N",0,0.5))+3*IF(S91="J",1,IF(S91="N",0,0.5)))/19,0)))</f>
+        <f>IF(A91="","",IF(OR(C91="Etagenwohnung",I91="N",J91="N"),0,ROUND(100*(3*IF(J91="J",1,IF(J91="N",0,0.5))+3*IF(K91="J",1,IF(K91="N",0,0.5))+2*IF(L91="J",1,IF(L91="N",0,0.5))+2*IF(M91="J",1,IF(M91="N",0,0.5))+1*IF(N91="J",1,IF(N91="N",0,0.5))+1*IF(O91="J",1,IF(O91="N",0,0.5))+1*IF(P91="J",1,IF(P91="N",0,0.5))+1*IF(Q91="J",1,IF(Q91="N",0,0.5))+2*IF(R91="J",1,IF(R91="N",0,0.5))+3*IF(S91="J",1,IF(S91="N",0,0.5))+IF(T91="",0,1*IF(T91="?",0.5,MAX(0,1-T91/3.57))))/(19+IF(T91="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G91" s="10" t="n"/>
@@ -4003,6 +4978,15 @@
         <f>IF(A91="","",IF(E91="","?",IF(AND(E91&gt;=90,E91&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T91" s="11" t="n"/>
+      <c r="U91" s="9">
+        <f>IF(OR(D91="",T91="",T91="?"),"",ROUND(D91*(Legende!$B$9+Legende!$B$10+T91/100),0))</f>
+        <v/>
+      </c>
+      <c r="V91" s="9">
+        <f>IF(U91="","",D91+U91)</f>
+        <v/>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="8" t="n"/>
@@ -4011,7 +4995,7 @@
       <c r="D92" s="9" t="n"/>
       <c r="E92" s="10" t="n"/>
       <c r="F92" s="10">
-        <f>IF(A92="","",IF(OR(C92="Etagenwohnung",I92="N"),0,ROUND(100*(3*IF(J92="J",1,IF(J92="N",0,0.5))+3*IF(K92="J",1,IF(K92="N",0,0.5))+2*IF(L92="J",1,IF(L92="N",0,0.5))+2*IF(M92="J",1,IF(M92="N",0,0.5))+1*IF(N92="J",1,IF(N92="N",0,0.5))+1*IF(O92="J",1,IF(O92="N",0,0.5))+1*IF(P92="J",1,IF(P92="N",0,0.5))+1*IF(Q92="J",1,IF(Q92="N",0,0.5))+2*IF(R92="J",1,IF(R92="N",0,0.5))+3*IF(S92="J",1,IF(S92="N",0,0.5)))/19,0)))</f>
+        <f>IF(A92="","",IF(OR(C92="Etagenwohnung",I92="N",J92="N"),0,ROUND(100*(3*IF(J92="J",1,IF(J92="N",0,0.5))+3*IF(K92="J",1,IF(K92="N",0,0.5))+2*IF(L92="J",1,IF(L92="N",0,0.5))+2*IF(M92="J",1,IF(M92="N",0,0.5))+1*IF(N92="J",1,IF(N92="N",0,0.5))+1*IF(O92="J",1,IF(O92="N",0,0.5))+1*IF(P92="J",1,IF(P92="N",0,0.5))+1*IF(Q92="J",1,IF(Q92="N",0,0.5))+2*IF(R92="J",1,IF(R92="N",0,0.5))+3*IF(S92="J",1,IF(S92="N",0,0.5))+IF(T92="",0,1*IF(T92="?",0.5,MAX(0,1-T92/3.57))))/(19+IF(T92="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G92" s="10" t="n"/>
@@ -4033,6 +5017,15 @@
         <f>IF(A92="","",IF(E92="","?",IF(AND(E92&gt;=90,E92&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T92" s="11" t="n"/>
+      <c r="U92" s="9">
+        <f>IF(OR(D92="",T92="",T92="?"),"",ROUND(D92*(Legende!$B$9+Legende!$B$10+T92/100),0))</f>
+        <v/>
+      </c>
+      <c r="V92" s="9">
+        <f>IF(U92="","",D92+U92)</f>
+        <v/>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="8" t="n"/>
@@ -4041,7 +5034,7 @@
       <c r="D93" s="9" t="n"/>
       <c r="E93" s="10" t="n"/>
       <c r="F93" s="10">
-        <f>IF(A93="","",IF(OR(C93="Etagenwohnung",I93="N"),0,ROUND(100*(3*IF(J93="J",1,IF(J93="N",0,0.5))+3*IF(K93="J",1,IF(K93="N",0,0.5))+2*IF(L93="J",1,IF(L93="N",0,0.5))+2*IF(M93="J",1,IF(M93="N",0,0.5))+1*IF(N93="J",1,IF(N93="N",0,0.5))+1*IF(O93="J",1,IF(O93="N",0,0.5))+1*IF(P93="J",1,IF(P93="N",0,0.5))+1*IF(Q93="J",1,IF(Q93="N",0,0.5))+2*IF(R93="J",1,IF(R93="N",0,0.5))+3*IF(S93="J",1,IF(S93="N",0,0.5)))/19,0)))</f>
+        <f>IF(A93="","",IF(OR(C93="Etagenwohnung",I93="N",J93="N"),0,ROUND(100*(3*IF(J93="J",1,IF(J93="N",0,0.5))+3*IF(K93="J",1,IF(K93="N",0,0.5))+2*IF(L93="J",1,IF(L93="N",0,0.5))+2*IF(M93="J",1,IF(M93="N",0,0.5))+1*IF(N93="J",1,IF(N93="N",0,0.5))+1*IF(O93="J",1,IF(O93="N",0,0.5))+1*IF(P93="J",1,IF(P93="N",0,0.5))+1*IF(Q93="J",1,IF(Q93="N",0,0.5))+2*IF(R93="J",1,IF(R93="N",0,0.5))+3*IF(S93="J",1,IF(S93="N",0,0.5))+IF(T93="",0,1*IF(T93="?",0.5,MAX(0,1-T93/3.57))))/(19+IF(T93="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G93" s="10" t="n"/>
@@ -4063,6 +5056,15 @@
         <f>IF(A93="","",IF(E93="","?",IF(AND(E93&gt;=90,E93&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T93" s="11" t="n"/>
+      <c r="U93" s="9">
+        <f>IF(OR(D93="",T93="",T93="?"),"",ROUND(D93*(Legende!$B$9+Legende!$B$10+T93/100),0))</f>
+        <v/>
+      </c>
+      <c r="V93" s="9">
+        <f>IF(U93="","",D93+U93)</f>
+        <v/>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="8" t="n"/>
@@ -4071,7 +5073,7 @@
       <c r="D94" s="9" t="n"/>
       <c r="E94" s="10" t="n"/>
       <c r="F94" s="10">
-        <f>IF(A94="","",IF(OR(C94="Etagenwohnung",I94="N"),0,ROUND(100*(3*IF(J94="J",1,IF(J94="N",0,0.5))+3*IF(K94="J",1,IF(K94="N",0,0.5))+2*IF(L94="J",1,IF(L94="N",0,0.5))+2*IF(M94="J",1,IF(M94="N",0,0.5))+1*IF(N94="J",1,IF(N94="N",0,0.5))+1*IF(O94="J",1,IF(O94="N",0,0.5))+1*IF(P94="J",1,IF(P94="N",0,0.5))+1*IF(Q94="J",1,IF(Q94="N",0,0.5))+2*IF(R94="J",1,IF(R94="N",0,0.5))+3*IF(S94="J",1,IF(S94="N",0,0.5)))/19,0)))</f>
+        <f>IF(A94="","",IF(OR(C94="Etagenwohnung",I94="N",J94="N"),0,ROUND(100*(3*IF(J94="J",1,IF(J94="N",0,0.5))+3*IF(K94="J",1,IF(K94="N",0,0.5))+2*IF(L94="J",1,IF(L94="N",0,0.5))+2*IF(M94="J",1,IF(M94="N",0,0.5))+1*IF(N94="J",1,IF(N94="N",0,0.5))+1*IF(O94="J",1,IF(O94="N",0,0.5))+1*IF(P94="J",1,IF(P94="N",0,0.5))+1*IF(Q94="J",1,IF(Q94="N",0,0.5))+2*IF(R94="J",1,IF(R94="N",0,0.5))+3*IF(S94="J",1,IF(S94="N",0,0.5))+IF(T94="",0,1*IF(T94="?",0.5,MAX(0,1-T94/3.57))))/(19+IF(T94="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G94" s="10" t="n"/>
@@ -4093,6 +5095,15 @@
         <f>IF(A94="","",IF(E94="","?",IF(AND(E94&gt;=90,E94&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T94" s="11" t="n"/>
+      <c r="U94" s="9">
+        <f>IF(OR(D94="",T94="",T94="?"),"",ROUND(D94*(Legende!$B$9+Legende!$B$10+T94/100),0))</f>
+        <v/>
+      </c>
+      <c r="V94" s="9">
+        <f>IF(U94="","",D94+U94)</f>
+        <v/>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="8" t="n"/>
@@ -4101,7 +5112,7 @@
       <c r="D95" s="9" t="n"/>
       <c r="E95" s="10" t="n"/>
       <c r="F95" s="10">
-        <f>IF(A95="","",IF(OR(C95="Etagenwohnung",I95="N"),0,ROUND(100*(3*IF(J95="J",1,IF(J95="N",0,0.5))+3*IF(K95="J",1,IF(K95="N",0,0.5))+2*IF(L95="J",1,IF(L95="N",0,0.5))+2*IF(M95="J",1,IF(M95="N",0,0.5))+1*IF(N95="J",1,IF(N95="N",0,0.5))+1*IF(O95="J",1,IF(O95="N",0,0.5))+1*IF(P95="J",1,IF(P95="N",0,0.5))+1*IF(Q95="J",1,IF(Q95="N",0,0.5))+2*IF(R95="J",1,IF(R95="N",0,0.5))+3*IF(S95="J",1,IF(S95="N",0,0.5)))/19,0)))</f>
+        <f>IF(A95="","",IF(OR(C95="Etagenwohnung",I95="N",J95="N"),0,ROUND(100*(3*IF(J95="J",1,IF(J95="N",0,0.5))+3*IF(K95="J",1,IF(K95="N",0,0.5))+2*IF(L95="J",1,IF(L95="N",0,0.5))+2*IF(M95="J",1,IF(M95="N",0,0.5))+1*IF(N95="J",1,IF(N95="N",0,0.5))+1*IF(O95="J",1,IF(O95="N",0,0.5))+1*IF(P95="J",1,IF(P95="N",0,0.5))+1*IF(Q95="J",1,IF(Q95="N",0,0.5))+2*IF(R95="J",1,IF(R95="N",0,0.5))+3*IF(S95="J",1,IF(S95="N",0,0.5))+IF(T95="",0,1*IF(T95="?",0.5,MAX(0,1-T95/3.57))))/(19+IF(T95="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G95" s="10" t="n"/>
@@ -4123,6 +5134,15 @@
         <f>IF(A95="","",IF(E95="","?",IF(AND(E95&gt;=90,E95&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T95" s="11" t="n"/>
+      <c r="U95" s="9">
+        <f>IF(OR(D95="",T95="",T95="?"),"",ROUND(D95*(Legende!$B$9+Legende!$B$10+T95/100),0))</f>
+        <v/>
+      </c>
+      <c r="V95" s="9">
+        <f>IF(U95="","",D95+U95)</f>
+        <v/>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="8" t="n"/>
@@ -4131,7 +5151,7 @@
       <c r="D96" s="9" t="n"/>
       <c r="E96" s="10" t="n"/>
       <c r="F96" s="10">
-        <f>IF(A96="","",IF(OR(C96="Etagenwohnung",I96="N"),0,ROUND(100*(3*IF(J96="J",1,IF(J96="N",0,0.5))+3*IF(K96="J",1,IF(K96="N",0,0.5))+2*IF(L96="J",1,IF(L96="N",0,0.5))+2*IF(M96="J",1,IF(M96="N",0,0.5))+1*IF(N96="J",1,IF(N96="N",0,0.5))+1*IF(O96="J",1,IF(O96="N",0,0.5))+1*IF(P96="J",1,IF(P96="N",0,0.5))+1*IF(Q96="J",1,IF(Q96="N",0,0.5))+2*IF(R96="J",1,IF(R96="N",0,0.5))+3*IF(S96="J",1,IF(S96="N",0,0.5)))/19,0)))</f>
+        <f>IF(A96="","",IF(OR(C96="Etagenwohnung",I96="N",J96="N"),0,ROUND(100*(3*IF(J96="J",1,IF(J96="N",0,0.5))+3*IF(K96="J",1,IF(K96="N",0,0.5))+2*IF(L96="J",1,IF(L96="N",0,0.5))+2*IF(M96="J",1,IF(M96="N",0,0.5))+1*IF(N96="J",1,IF(N96="N",0,0.5))+1*IF(O96="J",1,IF(O96="N",0,0.5))+1*IF(P96="J",1,IF(P96="N",0,0.5))+1*IF(Q96="J",1,IF(Q96="N",0,0.5))+2*IF(R96="J",1,IF(R96="N",0,0.5))+3*IF(S96="J",1,IF(S96="N",0,0.5))+IF(T96="",0,1*IF(T96="?",0.5,MAX(0,1-T96/3.57))))/(19+IF(T96="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G96" s="10" t="n"/>
@@ -4153,6 +5173,15 @@
         <f>IF(A96="","",IF(E96="","?",IF(AND(E96&gt;=90,E96&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T96" s="11" t="n"/>
+      <c r="U96" s="9">
+        <f>IF(OR(D96="",T96="",T96="?"),"",ROUND(D96*(Legende!$B$9+Legende!$B$10+T96/100),0))</f>
+        <v/>
+      </c>
+      <c r="V96" s="9">
+        <f>IF(U96="","",D96+U96)</f>
+        <v/>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="8" t="n"/>
@@ -4161,7 +5190,7 @@
       <c r="D97" s="9" t="n"/>
       <c r="E97" s="10" t="n"/>
       <c r="F97" s="10">
-        <f>IF(A97="","",IF(OR(C97="Etagenwohnung",I97="N"),0,ROUND(100*(3*IF(J97="J",1,IF(J97="N",0,0.5))+3*IF(K97="J",1,IF(K97="N",0,0.5))+2*IF(L97="J",1,IF(L97="N",0,0.5))+2*IF(M97="J",1,IF(M97="N",0,0.5))+1*IF(N97="J",1,IF(N97="N",0,0.5))+1*IF(O97="J",1,IF(O97="N",0,0.5))+1*IF(P97="J",1,IF(P97="N",0,0.5))+1*IF(Q97="J",1,IF(Q97="N",0,0.5))+2*IF(R97="J",1,IF(R97="N",0,0.5))+3*IF(S97="J",1,IF(S97="N",0,0.5)))/19,0)))</f>
+        <f>IF(A97="","",IF(OR(C97="Etagenwohnung",I97="N",J97="N"),0,ROUND(100*(3*IF(J97="J",1,IF(J97="N",0,0.5))+3*IF(K97="J",1,IF(K97="N",0,0.5))+2*IF(L97="J",1,IF(L97="N",0,0.5))+2*IF(M97="J",1,IF(M97="N",0,0.5))+1*IF(N97="J",1,IF(N97="N",0,0.5))+1*IF(O97="J",1,IF(O97="N",0,0.5))+1*IF(P97="J",1,IF(P97="N",0,0.5))+1*IF(Q97="J",1,IF(Q97="N",0,0.5))+2*IF(R97="J",1,IF(R97="N",0,0.5))+3*IF(S97="J",1,IF(S97="N",0,0.5))+IF(T97="",0,1*IF(T97="?",0.5,MAX(0,1-T97/3.57))))/(19+IF(T97="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G97" s="10" t="n"/>
@@ -4183,6 +5212,15 @@
         <f>IF(A97="","",IF(E97="","?",IF(AND(E97&gt;=90,E97&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T97" s="11" t="n"/>
+      <c r="U97" s="9">
+        <f>IF(OR(D97="",T97="",T97="?"),"",ROUND(D97*(Legende!$B$9+Legende!$B$10+T97/100),0))</f>
+        <v/>
+      </c>
+      <c r="V97" s="9">
+        <f>IF(U97="","",D97+U97)</f>
+        <v/>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="8" t="n"/>
@@ -4191,7 +5229,7 @@
       <c r="D98" s="9" t="n"/>
       <c r="E98" s="10" t="n"/>
       <c r="F98" s="10">
-        <f>IF(A98="","",IF(OR(C98="Etagenwohnung",I98="N"),0,ROUND(100*(3*IF(J98="J",1,IF(J98="N",0,0.5))+3*IF(K98="J",1,IF(K98="N",0,0.5))+2*IF(L98="J",1,IF(L98="N",0,0.5))+2*IF(M98="J",1,IF(M98="N",0,0.5))+1*IF(N98="J",1,IF(N98="N",0,0.5))+1*IF(O98="J",1,IF(O98="N",0,0.5))+1*IF(P98="J",1,IF(P98="N",0,0.5))+1*IF(Q98="J",1,IF(Q98="N",0,0.5))+2*IF(R98="J",1,IF(R98="N",0,0.5))+3*IF(S98="J",1,IF(S98="N",0,0.5)))/19,0)))</f>
+        <f>IF(A98="","",IF(OR(C98="Etagenwohnung",I98="N",J98="N"),0,ROUND(100*(3*IF(J98="J",1,IF(J98="N",0,0.5))+3*IF(K98="J",1,IF(K98="N",0,0.5))+2*IF(L98="J",1,IF(L98="N",0,0.5))+2*IF(M98="J",1,IF(M98="N",0,0.5))+1*IF(N98="J",1,IF(N98="N",0,0.5))+1*IF(O98="J",1,IF(O98="N",0,0.5))+1*IF(P98="J",1,IF(P98="N",0,0.5))+1*IF(Q98="J",1,IF(Q98="N",0,0.5))+2*IF(R98="J",1,IF(R98="N",0,0.5))+3*IF(S98="J",1,IF(S98="N",0,0.5))+IF(T98="",0,1*IF(T98="?",0.5,MAX(0,1-T98/3.57))))/(19+IF(T98="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G98" s="10" t="n"/>
@@ -4213,6 +5251,15 @@
         <f>IF(A98="","",IF(E98="","?",IF(AND(E98&gt;=90,E98&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T98" s="11" t="n"/>
+      <c r="U98" s="9">
+        <f>IF(OR(D98="",T98="",T98="?"),"",ROUND(D98*(Legende!$B$9+Legende!$B$10+T98/100),0))</f>
+        <v/>
+      </c>
+      <c r="V98" s="9">
+        <f>IF(U98="","",D98+U98)</f>
+        <v/>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="8" t="n"/>
@@ -4221,7 +5268,7 @@
       <c r="D99" s="9" t="n"/>
       <c r="E99" s="10" t="n"/>
       <c r="F99" s="10">
-        <f>IF(A99="","",IF(OR(C99="Etagenwohnung",I99="N"),0,ROUND(100*(3*IF(J99="J",1,IF(J99="N",0,0.5))+3*IF(K99="J",1,IF(K99="N",0,0.5))+2*IF(L99="J",1,IF(L99="N",0,0.5))+2*IF(M99="J",1,IF(M99="N",0,0.5))+1*IF(N99="J",1,IF(N99="N",0,0.5))+1*IF(O99="J",1,IF(O99="N",0,0.5))+1*IF(P99="J",1,IF(P99="N",0,0.5))+1*IF(Q99="J",1,IF(Q99="N",0,0.5))+2*IF(R99="J",1,IF(R99="N",0,0.5))+3*IF(S99="J",1,IF(S99="N",0,0.5)))/19,0)))</f>
+        <f>IF(A99="","",IF(OR(C99="Etagenwohnung",I99="N",J99="N"),0,ROUND(100*(3*IF(J99="J",1,IF(J99="N",0,0.5))+3*IF(K99="J",1,IF(K99="N",0,0.5))+2*IF(L99="J",1,IF(L99="N",0,0.5))+2*IF(M99="J",1,IF(M99="N",0,0.5))+1*IF(N99="J",1,IF(N99="N",0,0.5))+1*IF(O99="J",1,IF(O99="N",0,0.5))+1*IF(P99="J",1,IF(P99="N",0,0.5))+1*IF(Q99="J",1,IF(Q99="N",0,0.5))+2*IF(R99="J",1,IF(R99="N",0,0.5))+3*IF(S99="J",1,IF(S99="N",0,0.5))+IF(T99="",0,1*IF(T99="?",0.5,MAX(0,1-T99/3.57))))/(19+IF(T99="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G99" s="10" t="n"/>
@@ -4243,6 +5290,15 @@
         <f>IF(A99="","",IF(E99="","?",IF(AND(E99&gt;=90,E99&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T99" s="11" t="n"/>
+      <c r="U99" s="9">
+        <f>IF(OR(D99="",T99="",T99="?"),"",ROUND(D99*(Legende!$B$9+Legende!$B$10+T99/100),0))</f>
+        <v/>
+      </c>
+      <c r="V99" s="9">
+        <f>IF(U99="","",D99+U99)</f>
+        <v/>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="8" t="n"/>
@@ -4251,7 +5307,7 @@
       <c r="D100" s="9" t="n"/>
       <c r="E100" s="10" t="n"/>
       <c r="F100" s="10">
-        <f>IF(A100="","",IF(OR(C100="Etagenwohnung",I100="N"),0,ROUND(100*(3*IF(J100="J",1,IF(J100="N",0,0.5))+3*IF(K100="J",1,IF(K100="N",0,0.5))+2*IF(L100="J",1,IF(L100="N",0,0.5))+2*IF(M100="J",1,IF(M100="N",0,0.5))+1*IF(N100="J",1,IF(N100="N",0,0.5))+1*IF(O100="J",1,IF(O100="N",0,0.5))+1*IF(P100="J",1,IF(P100="N",0,0.5))+1*IF(Q100="J",1,IF(Q100="N",0,0.5))+2*IF(R100="J",1,IF(R100="N",0,0.5))+3*IF(S100="J",1,IF(S100="N",0,0.5)))/19,0)))</f>
+        <f>IF(A100="","",IF(OR(C100="Etagenwohnung",I100="N",J100="N"),0,ROUND(100*(3*IF(J100="J",1,IF(J100="N",0,0.5))+3*IF(K100="J",1,IF(K100="N",0,0.5))+2*IF(L100="J",1,IF(L100="N",0,0.5))+2*IF(M100="J",1,IF(M100="N",0,0.5))+1*IF(N100="J",1,IF(N100="N",0,0.5))+1*IF(O100="J",1,IF(O100="N",0,0.5))+1*IF(P100="J",1,IF(P100="N",0,0.5))+1*IF(Q100="J",1,IF(Q100="N",0,0.5))+2*IF(R100="J",1,IF(R100="N",0,0.5))+3*IF(S100="J",1,IF(S100="N",0,0.5))+IF(T100="",0,1*IF(T100="?",0.5,MAX(0,1-T100/3.57))))/(19+IF(T100="",0,1)),0)))</f>
         <v/>
       </c>
       <c r="G100" s="10" t="n"/>
@@ -4273,9 +5329,18 @@
         <f>IF(A100="","",IF(E100="","?",IF(AND(E100&gt;=90,E100&lt;=115),"J","N")))</f>
         <v/>
       </c>
+      <c r="T100" s="11" t="n"/>
+      <c r="U100" s="9">
+        <f>IF(OR(D100="",T100="",T100="?"),"",ROUND(D100*(Legende!$B$9+Legende!$B$10+T100/100),0))</f>
+        <v/>
+      </c>
+      <c r="V100" s="9">
+        <f>IF(U100="","",D100+U100)</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S100"/>
+  <autoFilter ref="A1:V100"/>
   <conditionalFormatting sqref="F2:F100">
     <cfRule type="colorScale" priority="1">
       <colorScale>
@@ -4288,7 +5353,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:S100">
+  <conditionalFormatting sqref="I2:V100">
     <cfRule type="cellIs" priority="2" operator="equal" dxfId="0">
       <formula>"J"</formula>
     </cfRule>
@@ -4328,7 +5393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -4351,7 +5416,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>K.O. (Score 0): Typ = Etagenwohnung oder Aufzug = N.</t>
+          <t>K.O. (Score 0): Typ = Etagenwohnung, Aufzug = N oder keine große Terrasse (Südterrasse = N; Balkon/überdachter Balkon zählt nicht).</t>
         </is>
       </c>
     </row>
@@ -4374,6 +5439,40 @@
         <is>
           <t>Kriterien-Spalten (I–S) lassen sich über das [–] oben einklappen.</t>
         </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Kosten (ab 21.10.2026, nur NEUE Objekte): Spalte „Provision %“ eintragen (0 = provisionsfrei, ? = unbekannt) → Nebenkosten und Gesamtkosten rechnen sich selbst.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Provision im Score: Gewicht ×1 (klein). Provisionsfrei = volle Punkte, 3,57 % = 0 Punkte. Leer = zählt nicht (alte Objekte bleiben unverändert).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Annahme Grunderwerbsteuer Bayern</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="n">
+        <v>0.035</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Annahme Notar + Grundbuch (ca.)</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="n">
+        <v>0.02</v>
       </c>
     </row>
   </sheetData>

</xml_diff>